<commit_message>
publica cambios de rutas y mejora refresh
</commit_message>
<xml_diff>
--- a/Template_Calendario_CCS_GPX.xlsx
+++ b/Template_Calendario_CCS_GPX.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cesarmora/Library/Mobile Documents/com~apple~CloudDocs/Personal/Ciclismo/Calendario/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB659B93-38D4-9C4F-967C-A03A61F13431}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C8DA118-5956-0D44-BE5E-E774E6EBC98B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="720" yWindow="780" windowWidth="34340" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="720" yWindow="780" windowWidth="34340" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template_Calendario_CCS" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="344">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="346">
   <si>
     <t>Fecha</t>
   </si>
@@ -71,18 +71,12 @@
     <t>Coda - Colliguay</t>
   </si>
   <si>
-    <t>Farellones Full Moon + tres Valles</t>
-  </si>
-  <si>
     <t>Kross - Pangue - Ibacache (GFC)</t>
   </si>
   <si>
     <t>Mc Chamisero - Til Til - Cumbre La Dormida (Bis)</t>
   </si>
   <si>
-    <t xml:space="preserve">Portillo </t>
-  </si>
-  <si>
     <t>Vizcachas - Embalse el Yeso (Bis)</t>
   </si>
   <si>
@@ -1053,6 +1047,18 @@
   </si>
   <si>
     <t>Montero</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Farellones Full Moon </t>
+  </si>
+  <si>
+    <t>Portillo  IDA</t>
+  </si>
+  <si>
+    <t>Quilapilun - La Dormida</t>
+  </si>
+  <si>
+    <t>Quilapilun - La Dormida.gpx</t>
   </si>
 </sst>
 </file>
@@ -1523,7 +1529,7 @@
     <col min="2" max="2" width="18" customWidth="1"/>
     <col min="3" max="3" width="51.1640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="24" customWidth="1"/>
-    <col min="5" max="5" width="42" customWidth="1"/>
+    <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="49.5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="7.83203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10.83203125" bestFit="1" customWidth="1"/>
@@ -1552,19 +1558,19 @@
         <v>5</v>
       </c>
       <c r="G1" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="H1" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="I1" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="J1" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="K1" s="12" t="s">
         <v>47</v>
-      </c>
-      <c r="J1" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="K1" s="12" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:11">
@@ -1578,13 +1584,13 @@
         <v>8</v>
       </c>
       <c r="D2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -1598,13 +1604,13 @@
         <v>9</v>
       </c>
       <c r="D3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -1618,13 +1624,13 @@
         <v>10</v>
       </c>
       <c r="D4" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -1638,13 +1644,13 @@
         <v>11</v>
       </c>
       <c r="D5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -1658,13 +1664,13 @@
         <v>12</v>
       </c>
       <c r="D6" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -1678,13 +1684,13 @@
         <v>13</v>
       </c>
       <c r="D7" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -1698,13 +1704,13 @@
         <v>14</v>
       </c>
       <c r="D8" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -1718,13 +1724,13 @@
         <v>15</v>
       </c>
       <c r="D9" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -1735,16 +1741,16 @@
         <v>7</v>
       </c>
       <c r="C10" t="s">
-        <v>16</v>
+        <v>342</v>
       </c>
       <c r="D10" t="s">
-        <v>16</v>
+        <v>342</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -1755,16 +1761,16 @@
         <v>7</v>
       </c>
       <c r="C11" t="s">
-        <v>16</v>
+        <v>342</v>
       </c>
       <c r="D11" t="s">
-        <v>16</v>
+        <v>342</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -1775,16 +1781,16 @@
         <v>6</v>
       </c>
       <c r="C12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D12" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -1795,16 +1801,16 @@
         <v>6</v>
       </c>
       <c r="C13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D13" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -1815,16 +1821,16 @@
         <v>6</v>
       </c>
       <c r="C14" t="s">
-        <v>19</v>
+        <v>343</v>
       </c>
       <c r="D14" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -1835,16 +1841,16 @@
         <v>6</v>
       </c>
       <c r="C15" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D15" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -1855,16 +1861,16 @@
         <v>6</v>
       </c>
       <c r="C16" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D16" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -1875,16 +1881,16 @@
         <v>6</v>
       </c>
       <c r="C17" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D17" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -1895,16 +1901,16 @@
         <v>6</v>
       </c>
       <c r="C18" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D18" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -1918,13 +1924,13 @@
         <v>11</v>
       </c>
       <c r="D19" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -1935,16 +1941,16 @@
         <v>6</v>
       </c>
       <c r="C20" t="s">
-        <v>18</v>
+        <v>344</v>
       </c>
       <c r="D20" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>50</v>
+        <v>345</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -1955,16 +1961,16 @@
         <v>7</v>
       </c>
       <c r="C21" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D21" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E21" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -1975,16 +1981,16 @@
         <v>7</v>
       </c>
       <c r="C22" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D22" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E22" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -1995,16 +2001,16 @@
         <v>7</v>
       </c>
       <c r="C23" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D23" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E23" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -2015,16 +2021,16 @@
         <v>6</v>
       </c>
       <c r="C24" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="D24" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -2035,16 +2041,16 @@
         <v>6</v>
       </c>
       <c r="C25" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D25" t="s">
+        <v>39</v>
+      </c>
+      <c r="E25" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="E25" s="10" t="s">
-        <v>43</v>
-      </c>
       <c r="F25" s="5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -2055,16 +2061,16 @@
         <v>6</v>
       </c>
       <c r="C26" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D26" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -2075,16 +2081,16 @@
         <v>6</v>
       </c>
       <c r="C27" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D27" t="s">
+        <v>39</v>
+      </c>
+      <c r="E27" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="E27" s="10" t="s">
-        <v>43</v>
-      </c>
       <c r="F27" s="5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -2095,16 +2101,16 @@
         <v>6</v>
       </c>
       <c r="C28" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D28" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -2115,16 +2121,16 @@
         <v>6</v>
       </c>
       <c r="C29" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D29" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="30" spans="1:6">
@@ -2135,16 +2141,16 @@
         <v>6</v>
       </c>
       <c r="C30" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D30" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="31" spans="1:6">
@@ -2155,16 +2161,16 @@
         <v>7</v>
       </c>
       <c r="C31" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D31" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E31" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -2175,16 +2181,16 @@
         <v>7</v>
       </c>
       <c r="C32" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D32" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E32" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="33" spans="1:6">
@@ -2195,16 +2201,16 @@
         <v>7</v>
       </c>
       <c r="C33" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D33" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E33" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="34" spans="1:6">
@@ -2215,25 +2221,37 @@
         <v>6</v>
       </c>
       <c r="C34" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D34" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="35" spans="1:6">
-      <c r="A35" s="3"/>
-      <c r="B35" s="4"/>
-      <c r="C35" s="4"/>
-      <c r="D35" s="4"/>
-      <c r="E35" s="4"/>
-      <c r="F35" s="5"/>
+      <c r="A35" s="13">
+        <v>46214</v>
+      </c>
+      <c r="B35" t="s">
+        <v>6</v>
+      </c>
+      <c r="C35" t="s">
+        <v>9</v>
+      </c>
+      <c r="D35" t="s">
+        <v>30</v>
+      </c>
+      <c r="E35" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="F35" s="5" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="36" spans="1:6">
       <c r="A36" s="3"/>
@@ -2346,12 +2364,13 @@
     <hyperlink ref="E28" r:id="rId19" xr:uid="{7CC30E5B-2CD8-AB40-B4D7-C3C7DE75034F}"/>
     <hyperlink ref="E29" r:id="rId20" xr:uid="{30CE1ED5-38D9-794D-99A0-4169C9F63FB9}"/>
     <hyperlink ref="E30" r:id="rId21" xr:uid="{3C231A25-5D10-9E42-9424-03B487C9F031}"/>
-    <hyperlink ref="E20" r:id="rId22" xr:uid="{5E464D1D-F337-434D-AA1D-A89B7D6249F7}"/>
-    <hyperlink ref="E24" r:id="rId23" xr:uid="{26A0E119-9616-884A-AE84-9036AE3323B7}"/>
-    <hyperlink ref="E34" r:id="rId24" xr:uid="{7CBDAD5C-DF2C-FC4B-BA08-275AF964144A}"/>
-    <hyperlink ref="E25" r:id="rId25" xr:uid="{E2A3AE02-8FC9-1C4A-BE4A-AFA67B68D56F}"/>
-    <hyperlink ref="E16" r:id="rId26" xr:uid="{35C172B7-7936-AF4E-B1C2-147C8E7867CA}"/>
-    <hyperlink ref="E19" r:id="rId27" xr:uid="{08AE7119-345F-9D47-997F-67E247E970E5}"/>
+    <hyperlink ref="E34" r:id="rId22" xr:uid="{7CBDAD5C-DF2C-FC4B-BA08-275AF964144A}"/>
+    <hyperlink ref="E25" r:id="rId23" xr:uid="{E2A3AE02-8FC9-1C4A-BE4A-AFA67B68D56F}"/>
+    <hyperlink ref="E16" r:id="rId24" xr:uid="{35C172B7-7936-AF4E-B1C2-147C8E7867CA}"/>
+    <hyperlink ref="E19" r:id="rId25" xr:uid="{08AE7119-345F-9D47-997F-67E247E970E5}"/>
+    <hyperlink ref="E35" r:id="rId26" xr:uid="{13AFCAE5-A888-BD46-A83F-C77F11E366D7}"/>
+    <hyperlink ref="E24" r:id="rId27" xr:uid="{CF7403E1-E9E7-EC40-BE26-3A6B792A99C1}"/>
+    <hyperlink ref="E20" r:id="rId28" xr:uid="{8866888E-71DF-3944-9620-4E948829D43F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2371,19 +2390,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="B1" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="C1" s="16" t="s">
         <v>78</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="D1" s="16" t="s">
         <v>79</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="E1" s="17" t="s">
         <v>80</v>
-      </c>
-      <c r="D1" s="16" t="s">
-        <v>81</v>
-      </c>
-      <c r="E1" s="17" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -2391,16 +2410,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="C2" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="D2" s="20" t="s">
         <v>83</v>
       </c>
-      <c r="C2" s="20" t="s">
+      <c r="E2" s="21" t="s">
         <v>84</v>
-      </c>
-      <c r="D2" s="20" t="s">
-        <v>85</v>
-      </c>
-      <c r="E2" s="21" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -2408,16 +2427,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C3" s="20" t="s">
+        <v>85</v>
+      </c>
+      <c r="D3" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="E3" s="21" t="s">
         <v>87</v>
-      </c>
-      <c r="D3" s="20" t="s">
-        <v>88</v>
-      </c>
-      <c r="E3" s="21" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -2425,16 +2444,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C4" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="D4" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="E4" s="22" t="s">
         <v>90</v>
-      </c>
-      <c r="D4" s="22" t="s">
-        <v>91</v>
-      </c>
-      <c r="E4" s="22" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -2442,16 +2461,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C5" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="D5" s="22" t="s">
+        <v>92</v>
+      </c>
+      <c r="E5" s="22" t="s">
         <v>93</v>
-      </c>
-      <c r="D5" s="22" t="s">
-        <v>94</v>
-      </c>
-      <c r="E5" s="22" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -2459,16 +2478,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C6" s="20" t="s">
+        <v>94</v>
+      </c>
+      <c r="D6" s="22" t="s">
+        <v>95</v>
+      </c>
+      <c r="E6" s="22" t="s">
         <v>96</v>
-      </c>
-      <c r="D6" s="22" t="s">
-        <v>97</v>
-      </c>
-      <c r="E6" s="22" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -2476,16 +2495,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C7" s="20" t="s">
+        <v>97</v>
+      </c>
+      <c r="D7" s="20" t="s">
+        <v>98</v>
+      </c>
+      <c r="E7" s="20" t="s">
         <v>99</v>
-      </c>
-      <c r="D7" s="20" t="s">
-        <v>100</v>
-      </c>
-      <c r="E7" s="20" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -2493,16 +2512,16 @@
         <v>7</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C8" s="20" t="s">
+        <v>100</v>
+      </c>
+      <c r="D8" s="20" t="s">
+        <v>101</v>
+      </c>
+      <c r="E8" s="21" t="s">
         <v>102</v>
-      </c>
-      <c r="D8" s="20" t="s">
-        <v>103</v>
-      </c>
-      <c r="E8" s="21" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -2510,16 +2529,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C9" s="20" t="s">
+        <v>103</v>
+      </c>
+      <c r="D9" s="20" t="s">
+        <v>104</v>
+      </c>
+      <c r="E9" s="21" t="s">
         <v>105</v>
-      </c>
-      <c r="D9" s="20" t="s">
-        <v>106</v>
-      </c>
-      <c r="E9" s="21" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -2527,16 +2546,16 @@
         <v>9</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C10" s="20" t="s">
+        <v>106</v>
+      </c>
+      <c r="D10" s="22" t="s">
+        <v>107</v>
+      </c>
+      <c r="E10" s="22" t="s">
         <v>108</v>
-      </c>
-      <c r="D10" s="22" t="s">
-        <v>109</v>
-      </c>
-      <c r="E10" s="22" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -2544,16 +2563,16 @@
         <v>10</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C11" s="20" t="s">
+        <v>109</v>
+      </c>
+      <c r="D11" s="22" t="s">
+        <v>110</v>
+      </c>
+      <c r="E11" s="22" t="s">
         <v>111</v>
-      </c>
-      <c r="D11" s="22" t="s">
-        <v>112</v>
-      </c>
-      <c r="E11" s="22" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -2561,16 +2580,16 @@
         <v>11</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C12" s="20" t="s">
+        <v>112</v>
+      </c>
+      <c r="D12" s="20" t="s">
+        <v>113</v>
+      </c>
+      <c r="E12" s="21" t="s">
         <v>114</v>
-      </c>
-      <c r="D12" s="20" t="s">
-        <v>115</v>
-      </c>
-      <c r="E12" s="21" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -2578,16 +2597,16 @@
         <v>12</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C13" s="20" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D13" s="20" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -2595,16 +2614,16 @@
         <v>13</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C14" s="20" t="s">
+        <v>117</v>
+      </c>
+      <c r="D14" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="E14" s="21" t="s">
         <v>119</v>
-      </c>
-      <c r="D14" s="20" t="s">
-        <v>120</v>
-      </c>
-      <c r="E14" s="21" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -2612,16 +2631,16 @@
         <v>14</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C15" s="20" t="s">
+        <v>120</v>
+      </c>
+      <c r="D15" s="20" t="s">
+        <v>121</v>
+      </c>
+      <c r="E15" s="21" t="s">
         <v>122</v>
-      </c>
-      <c r="D15" s="20" t="s">
-        <v>123</v>
-      </c>
-      <c r="E15" s="21" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -2629,16 +2648,16 @@
         <v>15</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C16" s="20" t="s">
+        <v>123</v>
+      </c>
+      <c r="D16" s="20" t="s">
+        <v>124</v>
+      </c>
+      <c r="E16" s="21" t="s">
         <v>125</v>
-      </c>
-      <c r="D16" s="20" t="s">
-        <v>126</v>
-      </c>
-      <c r="E16" s="21" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -2646,16 +2665,16 @@
         <v>16</v>
       </c>
       <c r="B17" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C17" s="20" t="s">
+        <v>126</v>
+      </c>
+      <c r="D17" s="20" t="s">
+        <v>127</v>
+      </c>
+      <c r="E17" s="21" t="s">
         <v>128</v>
-      </c>
-      <c r="D17" s="20" t="s">
-        <v>129</v>
-      </c>
-      <c r="E17" s="21" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -2663,16 +2682,16 @@
         <v>17</v>
       </c>
       <c r="B18" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C18" s="20" t="s">
+        <v>129</v>
+      </c>
+      <c r="D18" s="20" t="s">
+        <v>130</v>
+      </c>
+      <c r="E18" s="21" t="s">
         <v>131</v>
-      </c>
-      <c r="D18" s="20" t="s">
-        <v>132</v>
-      </c>
-      <c r="E18" s="21" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -2680,16 +2699,16 @@
         <v>18</v>
       </c>
       <c r="B19" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C19" s="20" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="D19" s="20" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E19" s="21" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -2697,16 +2716,16 @@
         <v>19</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C20" s="20" t="s">
+        <v>134</v>
+      </c>
+      <c r="D20" s="20" t="s">
+        <v>135</v>
+      </c>
+      <c r="E20" s="21" t="s">
         <v>136</v>
-      </c>
-      <c r="D20" s="20" t="s">
-        <v>137</v>
-      </c>
-      <c r="E20" s="21" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -2714,16 +2733,16 @@
         <v>20</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C21" s="20" t="s">
+        <v>137</v>
+      </c>
+      <c r="D21" s="22" t="s">
+        <v>138</v>
+      </c>
+      <c r="E21" s="22" t="s">
         <v>139</v>
-      </c>
-      <c r="D21" s="22" t="s">
-        <v>140</v>
-      </c>
-      <c r="E21" s="22" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -2731,16 +2750,16 @@
         <v>21</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C22" s="20" t="s">
+        <v>140</v>
+      </c>
+      <c r="D22" s="22" t="s">
+        <v>141</v>
+      </c>
+      <c r="E22" s="22" t="s">
         <v>142</v>
-      </c>
-      <c r="D22" s="22" t="s">
-        <v>143</v>
-      </c>
-      <c r="E22" s="22" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -2748,16 +2767,16 @@
         <v>22</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C23" s="20" t="s">
+        <v>143</v>
+      </c>
+      <c r="D23" s="20" t="s">
+        <v>144</v>
+      </c>
+      <c r="E23" s="21" t="s">
         <v>145</v>
-      </c>
-      <c r="D23" s="20" t="s">
-        <v>146</v>
-      </c>
-      <c r="E23" s="21" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -2765,16 +2784,16 @@
         <v>23</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C24" s="20" t="s">
+        <v>146</v>
+      </c>
+      <c r="D24" s="20" t="s">
+        <v>147</v>
+      </c>
+      <c r="E24" s="21" t="s">
         <v>148</v>
-      </c>
-      <c r="D24" s="20" t="s">
-        <v>149</v>
-      </c>
-      <c r="E24" s="21" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -2782,16 +2801,16 @@
         <v>24</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C25" s="20" t="s">
+        <v>149</v>
+      </c>
+      <c r="D25" s="20" t="s">
+        <v>150</v>
+      </c>
+      <c r="E25" s="21" t="s">
         <v>151</v>
-      </c>
-      <c r="D25" s="20" t="s">
-        <v>152</v>
-      </c>
-      <c r="E25" s="21" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -2799,16 +2818,16 @@
         <v>25</v>
       </c>
       <c r="B26" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C26" s="20" t="s">
+        <v>152</v>
+      </c>
+      <c r="D26" s="22" t="s">
+        <v>153</v>
+      </c>
+      <c r="E26" s="22" t="s">
         <v>154</v>
-      </c>
-      <c r="D26" s="22" t="s">
-        <v>155</v>
-      </c>
-      <c r="E26" s="22" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -2816,16 +2835,16 @@
         <v>26</v>
       </c>
       <c r="B27" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C27" s="20" t="s">
+        <v>155</v>
+      </c>
+      <c r="D27" s="20" t="s">
+        <v>156</v>
+      </c>
+      <c r="E27" s="21" t="s">
         <v>157</v>
-      </c>
-      <c r="D27" s="20" t="s">
-        <v>158</v>
-      </c>
-      <c r="E27" s="21" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -2833,16 +2852,16 @@
         <v>27</v>
       </c>
       <c r="B28" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C28" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="D28" s="20" t="s">
+        <v>159</v>
+      </c>
+      <c r="E28" s="21" t="s">
         <v>160</v>
-      </c>
-      <c r="D28" s="20" t="s">
-        <v>161</v>
-      </c>
-      <c r="E28" s="21" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -2850,16 +2869,16 @@
         <v>28</v>
       </c>
       <c r="B29" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C29" s="20" t="s">
+        <v>161</v>
+      </c>
+      <c r="D29" s="20" t="s">
+        <v>162</v>
+      </c>
+      <c r="E29" s="21" t="s">
         <v>163</v>
-      </c>
-      <c r="D29" s="20" t="s">
-        <v>164</v>
-      </c>
-      <c r="E29" s="21" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="30" spans="1:5">
@@ -2867,16 +2886,16 @@
         <v>29</v>
       </c>
       <c r="B30" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C30" s="20" t="s">
+        <v>164</v>
+      </c>
+      <c r="D30" s="22" t="s">
+        <v>165</v>
+      </c>
+      <c r="E30" s="22" t="s">
         <v>166</v>
-      </c>
-      <c r="D30" s="22" t="s">
-        <v>167</v>
-      </c>
-      <c r="E30" s="22" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="31" spans="1:5">
@@ -2884,16 +2903,16 @@
         <v>30</v>
       </c>
       <c r="B31" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C31" s="20" t="s">
+        <v>167</v>
+      </c>
+      <c r="D31" s="20" t="s">
+        <v>168</v>
+      </c>
+      <c r="E31" s="21" t="s">
         <v>169</v>
-      </c>
-      <c r="D31" s="20" t="s">
-        <v>170</v>
-      </c>
-      <c r="E31" s="21" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="32" spans="1:5">
@@ -2901,16 +2920,16 @@
         <v>31</v>
       </c>
       <c r="B32" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C32" s="20" t="s">
+        <v>170</v>
+      </c>
+      <c r="D32" s="20" t="s">
+        <v>171</v>
+      </c>
+      <c r="E32" s="21" t="s">
         <v>172</v>
-      </c>
-      <c r="D32" s="20" t="s">
-        <v>173</v>
-      </c>
-      <c r="E32" s="21" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="33" spans="1:5">
@@ -2918,16 +2937,16 @@
         <v>32</v>
       </c>
       <c r="B33" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C33" s="20" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="D33" s="20" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="E33" s="21" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="34" spans="1:5">
@@ -2935,16 +2954,16 @@
         <v>33</v>
       </c>
       <c r="B34" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C34" s="20" t="s">
+        <v>174</v>
+      </c>
+      <c r="D34" s="20" t="s">
+        <v>175</v>
+      </c>
+      <c r="E34" s="21" t="s">
         <v>176</v>
-      </c>
-      <c r="D34" s="20" t="s">
-        <v>177</v>
-      </c>
-      <c r="E34" s="21" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="35" spans="1:5">
@@ -2952,16 +2971,16 @@
         <v>34</v>
       </c>
       <c r="B35" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C35" s="20" t="s">
+        <v>177</v>
+      </c>
+      <c r="D35" s="20" t="s">
+        <v>178</v>
+      </c>
+      <c r="E35" s="21" t="s">
         <v>179</v>
-      </c>
-      <c r="D35" s="20" t="s">
-        <v>180</v>
-      </c>
-      <c r="E35" s="21" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="36" spans="1:5">
@@ -2969,16 +2988,16 @@
         <v>35</v>
       </c>
       <c r="B36" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C36" s="20" t="s">
+        <v>180</v>
+      </c>
+      <c r="D36" s="20" t="s">
+        <v>181</v>
+      </c>
+      <c r="E36" s="21" t="s">
         <v>182</v>
-      </c>
-      <c r="D36" s="20" t="s">
-        <v>183</v>
-      </c>
-      <c r="E36" s="21" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="37" spans="1:5">
@@ -2986,16 +3005,16 @@
         <v>36</v>
       </c>
       <c r="B37" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C37" s="20" t="s">
+        <v>183</v>
+      </c>
+      <c r="D37" s="20" t="s">
+        <v>184</v>
+      </c>
+      <c r="E37" s="21" t="s">
         <v>185</v>
-      </c>
-      <c r="D37" s="20" t="s">
-        <v>186</v>
-      </c>
-      <c r="E37" s="21" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="38" spans="1:5">
@@ -3003,16 +3022,16 @@
         <v>37</v>
       </c>
       <c r="B38" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C38" s="20" t="s">
+        <v>186</v>
+      </c>
+      <c r="D38" s="20" t="s">
+        <v>187</v>
+      </c>
+      <c r="E38" s="21" t="s">
         <v>188</v>
-      </c>
-      <c r="D38" s="20" t="s">
-        <v>189</v>
-      </c>
-      <c r="E38" s="21" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="39" spans="1:5">
@@ -3020,16 +3039,16 @@
         <v>38</v>
       </c>
       <c r="B39" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C39" s="20" t="s">
+        <v>189</v>
+      </c>
+      <c r="D39" s="20" t="s">
+        <v>190</v>
+      </c>
+      <c r="E39" s="21" t="s">
         <v>191</v>
-      </c>
-      <c r="D39" s="20" t="s">
-        <v>192</v>
-      </c>
-      <c r="E39" s="21" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="40" spans="1:5">
@@ -3037,16 +3056,16 @@
         <v>39</v>
       </c>
       <c r="B40" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C40" s="20" t="s">
+        <v>192</v>
+      </c>
+      <c r="D40" s="20" t="s">
+        <v>193</v>
+      </c>
+      <c r="E40" s="21" t="s">
         <v>194</v>
-      </c>
-      <c r="D40" s="20" t="s">
-        <v>195</v>
-      </c>
-      <c r="E40" s="21" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="41" spans="1:5">
@@ -3054,16 +3073,16 @@
         <v>40</v>
       </c>
       <c r="B41" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C41" s="24" t="s">
+        <v>195</v>
+      </c>
+      <c r="D41" s="20" t="s">
+        <v>196</v>
+      </c>
+      <c r="E41" s="21" t="s">
         <v>197</v>
-      </c>
-      <c r="D41" s="20" t="s">
-        <v>198</v>
-      </c>
-      <c r="E41" s="21" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="42" spans="1:5">
@@ -3071,16 +3090,16 @@
         <v>41</v>
       </c>
       <c r="B42" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C42" s="20" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="D42" s="22" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="E42" s="22" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
     </row>
     <row r="43" spans="1:5">
@@ -3088,16 +3107,16 @@
         <v>42</v>
       </c>
       <c r="B43" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C43" s="20" t="s">
+        <v>200</v>
+      </c>
+      <c r="D43" s="22" t="s">
+        <v>201</v>
+      </c>
+      <c r="E43" s="22" t="s">
         <v>202</v>
-      </c>
-      <c r="D43" s="22" t="s">
-        <v>203</v>
-      </c>
-      <c r="E43" s="22" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="44" spans="1:5">
@@ -3105,16 +3124,16 @@
         <v>43</v>
       </c>
       <c r="B44" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C44" s="20" t="s">
+        <v>203</v>
+      </c>
+      <c r="D44" s="20" t="s">
+        <v>204</v>
+      </c>
+      <c r="E44" s="21" t="s">
         <v>205</v>
-      </c>
-      <c r="D44" s="20" t="s">
-        <v>206</v>
-      </c>
-      <c r="E44" s="21" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="45" spans="1:5">
@@ -3122,16 +3141,16 @@
         <v>44</v>
       </c>
       <c r="B45" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C45" s="20" t="s">
+        <v>206</v>
+      </c>
+      <c r="D45" s="22" t="s">
+        <v>207</v>
+      </c>
+      <c r="E45" s="22" t="s">
         <v>208</v>
-      </c>
-      <c r="D45" s="22" t="s">
-        <v>209</v>
-      </c>
-      <c r="E45" s="22" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="46" spans="1:5">
@@ -3139,16 +3158,16 @@
         <v>45</v>
       </c>
       <c r="B46" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C46" s="23" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="D46" s="20" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="E46" s="21" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="47" spans="1:5">
@@ -3156,16 +3175,16 @@
         <v>46</v>
       </c>
       <c r="B47" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C47" s="20" t="s">
+        <v>211</v>
+      </c>
+      <c r="D47" s="20" t="s">
+        <v>212</v>
+      </c>
+      <c r="E47" s="21" t="s">
         <v>213</v>
-      </c>
-      <c r="D47" s="20" t="s">
-        <v>214</v>
-      </c>
-      <c r="E47" s="21" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="48" spans="1:5">
@@ -3173,16 +3192,16 @@
         <v>47</v>
       </c>
       <c r="B48" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C48" s="20" t="s">
+        <v>214</v>
+      </c>
+      <c r="D48" s="20" t="s">
+        <v>215</v>
+      </c>
+      <c r="E48" s="21" t="s">
         <v>216</v>
-      </c>
-      <c r="D48" s="20" t="s">
-        <v>217</v>
-      </c>
-      <c r="E48" s="21" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="49" spans="1:5">
@@ -3190,16 +3209,16 @@
         <v>48</v>
       </c>
       <c r="B49" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C49" s="20" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="D49" s="20" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="E49" s="21" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="50" spans="1:5">
@@ -3207,16 +3226,16 @@
         <v>49</v>
       </c>
       <c r="B50" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C50" s="20" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="D50" s="22" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="E50" s="22" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
     </row>
     <row r="51" spans="1:5">
@@ -3224,16 +3243,16 @@
         <v>50</v>
       </c>
       <c r="B51" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C51" s="20" t="s">
+        <v>221</v>
+      </c>
+      <c r="D51" s="20" t="s">
+        <v>222</v>
+      </c>
+      <c r="E51" s="21" t="s">
         <v>223</v>
-      </c>
-      <c r="D51" s="20" t="s">
-        <v>224</v>
-      </c>
-      <c r="E51" s="21" t="s">
-        <v>225</v>
       </c>
     </row>
     <row r="52" spans="1:5">
@@ -3241,16 +3260,16 @@
         <v>51</v>
       </c>
       <c r="B52" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C52" s="20" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="D52" s="20" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="E52" s="21" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
     </row>
     <row r="53" spans="1:5">
@@ -3258,16 +3277,16 @@
         <v>52</v>
       </c>
       <c r="B53" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C53" s="20" t="s">
+        <v>226</v>
+      </c>
+      <c r="D53" s="20" t="s">
+        <v>227</v>
+      </c>
+      <c r="E53" s="21" t="s">
         <v>228</v>
-      </c>
-      <c r="D53" s="20" t="s">
-        <v>229</v>
-      </c>
-      <c r="E53" s="21" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="54" spans="1:5">
@@ -3275,16 +3294,16 @@
         <v>53</v>
       </c>
       <c r="B54" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C54" s="20" t="s">
+        <v>229</v>
+      </c>
+      <c r="D54" s="20" t="s">
+        <v>230</v>
+      </c>
+      <c r="E54" s="21" t="s">
         <v>231</v>
-      </c>
-      <c r="D54" s="20" t="s">
-        <v>232</v>
-      </c>
-      <c r="E54" s="21" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="55" spans="1:5">
@@ -3292,16 +3311,16 @@
         <v>54</v>
       </c>
       <c r="B55" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C55" s="20" t="s">
+        <v>232</v>
+      </c>
+      <c r="D55" s="20" t="s">
+        <v>233</v>
+      </c>
+      <c r="E55" s="21" t="s">
         <v>234</v>
-      </c>
-      <c r="D55" s="20" t="s">
-        <v>235</v>
-      </c>
-      <c r="E55" s="21" t="s">
-        <v>236</v>
       </c>
     </row>
     <row r="56" spans="1:5">
@@ -3309,16 +3328,16 @@
         <v>55</v>
       </c>
       <c r="B56" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C56" s="20" t="s">
+        <v>235</v>
+      </c>
+      <c r="D56" s="22" t="s">
+        <v>236</v>
+      </c>
+      <c r="E56" s="22" t="s">
         <v>237</v>
-      </c>
-      <c r="D56" s="22" t="s">
-        <v>238</v>
-      </c>
-      <c r="E56" s="22" t="s">
-        <v>239</v>
       </c>
     </row>
     <row r="57" spans="1:5">
@@ -3326,16 +3345,16 @@
         <v>56</v>
       </c>
       <c r="B57" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C57" s="20" t="s">
+        <v>238</v>
+      </c>
+      <c r="D57" s="22" t="s">
+        <v>239</v>
+      </c>
+      <c r="E57" s="22" t="s">
         <v>240</v>
-      </c>
-      <c r="D57" s="22" t="s">
-        <v>241</v>
-      </c>
-      <c r="E57" s="22" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="58" spans="1:5">
@@ -3343,16 +3362,16 @@
         <v>57</v>
       </c>
       <c r="B58" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C58" s="20" t="s">
+        <v>241</v>
+      </c>
+      <c r="D58" s="20" t="s">
+        <v>242</v>
+      </c>
+      <c r="E58" s="21" t="s">
         <v>243</v>
-      </c>
-      <c r="D58" s="20" t="s">
-        <v>244</v>
-      </c>
-      <c r="E58" s="21" t="s">
-        <v>245</v>
       </c>
     </row>
     <row r="59" spans="1:5">
@@ -3360,16 +3379,16 @@
         <v>58</v>
       </c>
       <c r="B59" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C59" s="20" t="s">
+        <v>244</v>
+      </c>
+      <c r="D59" s="22" t="s">
+        <v>245</v>
+      </c>
+      <c r="E59" s="22" t="s">
         <v>246</v>
-      </c>
-      <c r="D59" s="22" t="s">
-        <v>247</v>
-      </c>
-      <c r="E59" s="22" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="60" spans="1:5">
@@ -3377,16 +3396,16 @@
         <v>59</v>
       </c>
       <c r="B60" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C60" s="20" t="s">
+        <v>247</v>
+      </c>
+      <c r="D60" s="20" t="s">
+        <v>248</v>
+      </c>
+      <c r="E60" s="21" t="s">
         <v>249</v>
-      </c>
-      <c r="D60" s="20" t="s">
-        <v>250</v>
-      </c>
-      <c r="E60" s="21" t="s">
-        <v>251</v>
       </c>
     </row>
     <row r="61" spans="1:5">
@@ -3394,16 +3413,16 @@
         <v>60</v>
       </c>
       <c r="B61" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C61" s="20" t="s">
+        <v>250</v>
+      </c>
+      <c r="D61" s="20" t="s">
+        <v>251</v>
+      </c>
+      <c r="E61" s="21" t="s">
         <v>252</v>
-      </c>
-      <c r="D61" s="20" t="s">
-        <v>253</v>
-      </c>
-      <c r="E61" s="21" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="62" spans="1:5">
@@ -3411,16 +3430,16 @@
         <v>61</v>
       </c>
       <c r="B62" s="22" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C62" s="20" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="D62" s="20" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="E62" s="21" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
     </row>
     <row r="63" spans="1:5">
@@ -3428,16 +3447,16 @@
         <v>62</v>
       </c>
       <c r="B63" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C63" s="20" t="s">
+        <v>255</v>
+      </c>
+      <c r="D63" s="20" t="s">
+        <v>256</v>
+      </c>
+      <c r="E63" s="21" t="s">
         <v>257</v>
-      </c>
-      <c r="D63" s="20" t="s">
-        <v>258</v>
-      </c>
-      <c r="E63" s="21" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="64" spans="1:5">
@@ -3445,16 +3464,16 @@
         <v>63</v>
       </c>
       <c r="B64" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C64" s="20" t="s">
+        <v>258</v>
+      </c>
+      <c r="D64" s="20" t="s">
+        <v>259</v>
+      </c>
+      <c r="E64" s="21" t="s">
         <v>260</v>
-      </c>
-      <c r="D64" s="20" t="s">
-        <v>261</v>
-      </c>
-      <c r="E64" s="21" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="65" spans="1:5">
@@ -3462,16 +3481,16 @@
         <v>64</v>
       </c>
       <c r="B65" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C65" s="20" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="D65" s="20" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E65" s="21" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
     </row>
     <row r="66" spans="1:5">
@@ -3479,16 +3498,16 @@
         <v>65</v>
       </c>
       <c r="B66" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C66" s="20">
         <v>132403031</v>
       </c>
       <c r="D66" s="20" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="E66" s="21" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
     </row>
     <row r="67" spans="1:5">
@@ -3496,16 +3515,16 @@
         <v>66</v>
       </c>
       <c r="B67" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C67" s="20" t="s">
+        <v>265</v>
+      </c>
+      <c r="D67" s="20" t="s">
+        <v>266</v>
+      </c>
+      <c r="E67" s="21" t="s">
         <v>267</v>
-      </c>
-      <c r="D67" s="20" t="s">
-        <v>268</v>
-      </c>
-      <c r="E67" s="21" t="s">
-        <v>269</v>
       </c>
     </row>
     <row r="68" spans="1:5">
@@ -3513,16 +3532,16 @@
         <v>67</v>
       </c>
       <c r="B68" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C68" s="20" t="s">
+        <v>268</v>
+      </c>
+      <c r="D68" s="20" t="s">
+        <v>269</v>
+      </c>
+      <c r="E68" s="21" t="s">
         <v>270</v>
-      </c>
-      <c r="D68" s="20" t="s">
-        <v>271</v>
-      </c>
-      <c r="E68" s="21" t="s">
-        <v>272</v>
       </c>
     </row>
     <row r="69" spans="1:5">
@@ -3530,16 +3549,16 @@
         <v>68</v>
       </c>
       <c r="B69" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C69" s="20" t="s">
+        <v>271</v>
+      </c>
+      <c r="D69" s="20" t="s">
+        <v>272</v>
+      </c>
+      <c r="E69" s="21" t="s">
         <v>273</v>
-      </c>
-      <c r="D69" s="20" t="s">
-        <v>274</v>
-      </c>
-      <c r="E69" s="21" t="s">
-        <v>275</v>
       </c>
     </row>
     <row r="70" spans="1:5">
@@ -3547,16 +3566,16 @@
         <v>69</v>
       </c>
       <c r="B70" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C70" s="20" t="s">
+        <v>274</v>
+      </c>
+      <c r="D70" s="22" t="s">
+        <v>275</v>
+      </c>
+      <c r="E70" s="22" t="s">
         <v>276</v>
-      </c>
-      <c r="D70" s="22" t="s">
-        <v>277</v>
-      </c>
-      <c r="E70" s="22" t="s">
-        <v>278</v>
       </c>
     </row>
     <row r="71" spans="1:5">
@@ -3564,16 +3583,16 @@
         <v>70</v>
       </c>
       <c r="B71" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C71" s="20" t="s">
+        <v>277</v>
+      </c>
+      <c r="D71" s="20" t="s">
+        <v>278</v>
+      </c>
+      <c r="E71" s="21" t="s">
         <v>279</v>
-      </c>
-      <c r="D71" s="20" t="s">
-        <v>280</v>
-      </c>
-      <c r="E71" s="21" t="s">
-        <v>281</v>
       </c>
     </row>
     <row r="72" spans="1:5">
@@ -3581,16 +3600,16 @@
         <v>71</v>
       </c>
       <c r="B72" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C72" s="20" t="s">
+        <v>280</v>
+      </c>
+      <c r="D72" s="22" t="s">
+        <v>281</v>
+      </c>
+      <c r="E72" s="22" t="s">
         <v>282</v>
-      </c>
-      <c r="D72" s="22" t="s">
-        <v>283</v>
-      </c>
-      <c r="E72" s="22" t="s">
-        <v>284</v>
       </c>
     </row>
     <row r="73" spans="1:5">
@@ -3598,16 +3617,16 @@
         <v>72</v>
       </c>
       <c r="B73" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C73" s="20" t="s">
+        <v>283</v>
+      </c>
+      <c r="D73" s="20" t="s">
+        <v>284</v>
+      </c>
+      <c r="E73" s="21" t="s">
         <v>285</v>
-      </c>
-      <c r="D73" s="20" t="s">
-        <v>286</v>
-      </c>
-      <c r="E73" s="21" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="74" spans="1:5">
@@ -3615,16 +3634,16 @@
         <v>73</v>
       </c>
       <c r="B74" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C74" s="20" t="s">
+        <v>286</v>
+      </c>
+      <c r="D74" s="20" t="s">
+        <v>287</v>
+      </c>
+      <c r="E74" s="21" t="s">
         <v>288</v>
-      </c>
-      <c r="D74" s="20" t="s">
-        <v>289</v>
-      </c>
-      <c r="E74" s="21" t="s">
-        <v>290</v>
       </c>
     </row>
     <row r="75" spans="1:5">
@@ -3632,16 +3651,16 @@
         <v>74</v>
       </c>
       <c r="B75" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C75" s="20" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="D75" s="22" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="E75" s="22" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
     </row>
     <row r="76" spans="1:5">
@@ -3649,16 +3668,16 @@
         <v>75</v>
       </c>
       <c r="B76" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C76" s="20" t="s">
+        <v>291</v>
+      </c>
+      <c r="D76" s="22" t="s">
+        <v>292</v>
+      </c>
+      <c r="E76" s="22" t="s">
         <v>293</v>
-      </c>
-      <c r="D76" s="22" t="s">
-        <v>294</v>
-      </c>
-      <c r="E76" s="22" t="s">
-        <v>295</v>
       </c>
     </row>
     <row r="77" spans="1:5">
@@ -3666,16 +3685,16 @@
         <v>76</v>
       </c>
       <c r="B77" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C77" s="20" t="s">
+        <v>294</v>
+      </c>
+      <c r="D77" s="22" t="s">
+        <v>295</v>
+      </c>
+      <c r="E77" s="22" t="s">
         <v>296</v>
-      </c>
-      <c r="D77" s="22" t="s">
-        <v>297</v>
-      </c>
-      <c r="E77" s="22" t="s">
-        <v>298</v>
       </c>
     </row>
     <row r="78" spans="1:5">
@@ -3683,16 +3702,16 @@
         <v>77</v>
       </c>
       <c r="B78" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C78" s="20" t="s">
+        <v>297</v>
+      </c>
+      <c r="D78" s="22" t="s">
+        <v>298</v>
+      </c>
+      <c r="E78" s="22" t="s">
         <v>299</v>
-      </c>
-      <c r="D78" s="22" t="s">
-        <v>300</v>
-      </c>
-      <c r="E78" s="22" t="s">
-        <v>301</v>
       </c>
     </row>
     <row r="79" spans="1:5">
@@ -3700,16 +3719,16 @@
         <v>78</v>
       </c>
       <c r="B79" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C79" s="20" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="D79" s="20" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="E79" s="21" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="80" spans="1:5">
@@ -3717,16 +3736,16 @@
         <v>79</v>
       </c>
       <c r="B80" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C80" s="20" t="s">
+        <v>302</v>
+      </c>
+      <c r="D80" s="22" t="s">
+        <v>303</v>
+      </c>
+      <c r="E80" s="22" t="s">
         <v>304</v>
-      </c>
-      <c r="D80" s="22" t="s">
-        <v>305</v>
-      </c>
-      <c r="E80" s="22" t="s">
-        <v>306</v>
       </c>
     </row>
     <row r="81" spans="1:5">
@@ -3734,16 +3753,16 @@
         <v>80</v>
       </c>
       <c r="B81" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C81" s="20" t="s">
+        <v>305</v>
+      </c>
+      <c r="D81" s="20" t="s">
+        <v>306</v>
+      </c>
+      <c r="E81" s="21" t="s">
         <v>307</v>
-      </c>
-      <c r="D81" s="20" t="s">
-        <v>308</v>
-      </c>
-      <c r="E81" s="21" t="s">
-        <v>309</v>
       </c>
     </row>
     <row r="82" spans="1:5">
@@ -3751,16 +3770,16 @@
         <v>81</v>
       </c>
       <c r="B82" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C82" s="20" t="s">
+        <v>308</v>
+      </c>
+      <c r="D82" s="20" t="s">
+        <v>309</v>
+      </c>
+      <c r="E82" s="21" t="s">
         <v>310</v>
-      </c>
-      <c r="D82" s="20" t="s">
-        <v>311</v>
-      </c>
-      <c r="E82" s="21" t="s">
-        <v>312</v>
       </c>
     </row>
     <row r="83" spans="1:5">
@@ -3768,16 +3787,16 @@
         <v>82</v>
       </c>
       <c r="B83" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C83" s="20" t="s">
+        <v>311</v>
+      </c>
+      <c r="D83" s="20" t="s">
+        <v>312</v>
+      </c>
+      <c r="E83" s="21" t="s">
         <v>313</v>
-      </c>
-      <c r="D83" s="20" t="s">
-        <v>314</v>
-      </c>
-      <c r="E83" s="21" t="s">
-        <v>315</v>
       </c>
     </row>
     <row r="84" spans="1:5">
@@ -3785,16 +3804,16 @@
         <v>83</v>
       </c>
       <c r="B84" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C84" s="20" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="D84" s="20" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="E84" s="21" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
     </row>
     <row r="85" spans="1:5">
@@ -3802,16 +3821,16 @@
         <v>84</v>
       </c>
       <c r="B85" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C85" s="20" t="s">
+        <v>316</v>
+      </c>
+      <c r="D85" s="20" t="s">
+        <v>317</v>
+      </c>
+      <c r="E85" s="21" t="s">
         <v>318</v>
-      </c>
-      <c r="D85" s="20" t="s">
-        <v>319</v>
-      </c>
-      <c r="E85" s="21" t="s">
-        <v>320</v>
       </c>
     </row>
     <row r="86" spans="1:5">
@@ -3819,16 +3838,16 @@
         <v>85</v>
       </c>
       <c r="B86" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C86" s="20" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="D86" s="20" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="E86" s="21" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
     </row>
     <row r="87" spans="1:5">
@@ -3836,16 +3855,16 @@
         <v>86</v>
       </c>
       <c r="B87" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C87" s="20" t="s">
+        <v>321</v>
+      </c>
+      <c r="D87" s="20" t="s">
+        <v>322</v>
+      </c>
+      <c r="E87" s="21" t="s">
         <v>323</v>
-      </c>
-      <c r="D87" s="20" t="s">
-        <v>324</v>
-      </c>
-      <c r="E87" s="21" t="s">
-        <v>325</v>
       </c>
     </row>
     <row r="88" spans="1:5">
@@ -3853,16 +3872,16 @@
         <v>87</v>
       </c>
       <c r="B88" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C88" s="20" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="D88" s="20" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="E88" s="21" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
     </row>
     <row r="89" spans="1:5">
@@ -3870,16 +3889,16 @@
         <v>88</v>
       </c>
       <c r="B89" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C89" s="20" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="D89" s="20" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="E89" s="21" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="90" spans="1:5">
@@ -3887,16 +3906,16 @@
         <v>89</v>
       </c>
       <c r="B90" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C90" s="20" t="s">
+        <v>328</v>
+      </c>
+      <c r="D90" s="20" t="s">
+        <v>329</v>
+      </c>
+      <c r="E90" s="21" t="s">
         <v>330</v>
-      </c>
-      <c r="D90" s="20" t="s">
-        <v>331</v>
-      </c>
-      <c r="E90" s="21" t="s">
-        <v>332</v>
       </c>
     </row>
     <row r="91" spans="1:5">
@@ -3904,16 +3923,16 @@
         <v>90</v>
       </c>
       <c r="B91" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C91" s="20" t="s">
+        <v>331</v>
+      </c>
+      <c r="D91" s="20" t="s">
+        <v>332</v>
+      </c>
+      <c r="E91" s="21" t="s">
         <v>333</v>
-      </c>
-      <c r="D91" s="20" t="s">
-        <v>334</v>
-      </c>
-      <c r="E91" s="21" t="s">
-        <v>335</v>
       </c>
     </row>
     <row r="92" spans="1:5">
@@ -3921,16 +3940,16 @@
         <v>91</v>
       </c>
       <c r="B92" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C92" s="20" t="s">
+        <v>334</v>
+      </c>
+      <c r="D92" s="20" t="s">
+        <v>335</v>
+      </c>
+      <c r="E92" s="21" t="s">
         <v>336</v>
-      </c>
-      <c r="D92" s="20" t="s">
-        <v>337</v>
-      </c>
-      <c r="E92" s="21" t="s">
-        <v>338</v>
       </c>
     </row>
     <row r="93" spans="1:5">
@@ -3938,16 +3957,16 @@
         <v>92</v>
       </c>
       <c r="B93" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C93" s="20" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="D93" s="20" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E93" s="21" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="94" spans="1:5">
@@ -3955,16 +3974,16 @@
         <v>93</v>
       </c>
       <c r="B94" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C94" s="20" t="s">
+        <v>339</v>
+      </c>
+      <c r="D94" s="22" t="s">
+        <v>340</v>
+      </c>
+      <c r="E94" s="22" t="s">
         <v>341</v>
-      </c>
-      <c r="D94" s="22" t="s">
-        <v>342</v>
-      </c>
-      <c r="E94" s="22" t="s">
-        <v>343</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
actualiza excel con usuarios corregidos
</commit_message>
<xml_diff>
--- a/Template_Calendario_CCS_GPX.xlsx
+++ b/Template_Calendario_CCS_GPX.xlsx
@@ -8,20 +8,33 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cesarmora/Library/Mobile Documents/com~apple~CloudDocs/Personal/Ciclismo/Calendario/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C8DA118-5956-0D44-BE5E-E774E6EBC98B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0865E891-110F-BD41-8940-B74838D0B8F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="720" yWindow="780" windowWidth="34340" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12200" yWindow="1420" windowWidth="20720" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template_Calendario_CCS" sheetId="1" r:id="rId1"/>
     <sheet name="Usuarios" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="346">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="359">
   <si>
     <t>Fecha</t>
   </si>
@@ -755,9 +768,6 @@
     <t>Maturana</t>
   </si>
   <si>
-    <t>18.220.962-k</t>
-  </si>
-  <si>
     <t xml:space="preserve">Fabian </t>
   </si>
   <si>
@@ -1059,6 +1069,48 @@
   </si>
   <si>
     <t>Quilapilun - La Dormida.gpx</t>
+  </si>
+  <si>
+    <t>Tiltil - Caleu - Quebrada Alvarado - Niño Dios (Bis)</t>
+  </si>
+  <si>
+    <t>Manuel Rodriguez Til Til - El Oregano - Niño Dios.gpx</t>
+  </si>
+  <si>
+    <t>Manuel Rodriguez - Til Til</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leonardo </t>
+  </si>
+  <si>
+    <t>Lobato</t>
+  </si>
+  <si>
+    <t>18.220.062-k</t>
+  </si>
+  <si>
+    <t>10.160.334-2</t>
+  </si>
+  <si>
+    <t>8327118-3</t>
+  </si>
+  <si>
+    <t>12239638-K</t>
+  </si>
+  <si>
+    <t>27150755-0</t>
+  </si>
+  <si>
+    <t>Álvaro</t>
+  </si>
+  <si>
+    <t>Larco</t>
+  </si>
+  <si>
+    <t>Simonetti</t>
+  </si>
+  <si>
+    <t>Guajardo</t>
   </si>
 </sst>
 </file>
@@ -1068,7 +1120,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0_ ;\-#,##0\ "/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -1123,8 +1175,15 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1136,8 +1195,14 @@
         <fgColor rgb="FFFFF200"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="13">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -1299,12 +1364,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1355,10 +1432,21 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="2" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 3 2" xfId="2" xr:uid="{3B3660B6-36B2-6C4C-8FC4-3C8693358251}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1741,10 +1829,10 @@
         <v>7</v>
       </c>
       <c r="C10" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D10" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>41</v>
@@ -1761,10 +1849,10 @@
         <v>7</v>
       </c>
       <c r="C11" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D11" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>41</v>
@@ -1821,7 +1909,7 @@
         <v>6</v>
       </c>
       <c r="C14" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="D14" t="s">
         <v>35</v>
@@ -1941,7 +2029,7 @@
         <v>6</v>
       </c>
       <c r="C20" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="D20" t="s">
         <v>30</v>
@@ -1950,7 +2038,7 @@
         <v>41</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -2021,16 +2109,16 @@
         <v>6</v>
       </c>
       <c r="C24" t="s">
-        <v>17</v>
+        <v>345</v>
       </c>
       <c r="D24" t="s">
-        <v>34</v>
+        <v>347</v>
       </c>
       <c r="E24" s="10" t="s">
         <v>41</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>48</v>
+        <v>346</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -2041,16 +2129,16 @@
         <v>6</v>
       </c>
       <c r="C25" t="s">
-        <v>24</v>
+        <v>345</v>
       </c>
       <c r="D25" t="s">
-        <v>39</v>
+        <v>347</v>
       </c>
       <c r="E25" s="10" t="s">
         <v>41</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>69</v>
+        <v>346</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -2365,12 +2453,12 @@
     <hyperlink ref="E29" r:id="rId20" xr:uid="{30CE1ED5-38D9-794D-99A0-4169C9F63FB9}"/>
     <hyperlink ref="E30" r:id="rId21" xr:uid="{3C231A25-5D10-9E42-9424-03B487C9F031}"/>
     <hyperlink ref="E34" r:id="rId22" xr:uid="{7CBDAD5C-DF2C-FC4B-BA08-275AF964144A}"/>
-    <hyperlink ref="E25" r:id="rId23" xr:uid="{E2A3AE02-8FC9-1C4A-BE4A-AFA67B68D56F}"/>
-    <hyperlink ref="E16" r:id="rId24" xr:uid="{35C172B7-7936-AF4E-B1C2-147C8E7867CA}"/>
-    <hyperlink ref="E19" r:id="rId25" xr:uid="{08AE7119-345F-9D47-997F-67E247E970E5}"/>
-    <hyperlink ref="E35" r:id="rId26" xr:uid="{13AFCAE5-A888-BD46-A83F-C77F11E366D7}"/>
-    <hyperlink ref="E24" r:id="rId27" xr:uid="{CF7403E1-E9E7-EC40-BE26-3A6B792A99C1}"/>
-    <hyperlink ref="E20" r:id="rId28" xr:uid="{8866888E-71DF-3944-9620-4E948829D43F}"/>
+    <hyperlink ref="E16" r:id="rId23" xr:uid="{35C172B7-7936-AF4E-B1C2-147C8E7867CA}"/>
+    <hyperlink ref="E19" r:id="rId24" xr:uid="{08AE7119-345F-9D47-997F-67E247E970E5}"/>
+    <hyperlink ref="E35" r:id="rId25" xr:uid="{13AFCAE5-A888-BD46-A83F-C77F11E366D7}"/>
+    <hyperlink ref="E24" r:id="rId26" xr:uid="{CF7403E1-E9E7-EC40-BE26-3A6B792A99C1}"/>
+    <hyperlink ref="E20" r:id="rId27" xr:uid="{8866888E-71DF-3944-9620-4E948829D43F}"/>
+    <hyperlink ref="E25" r:id="rId28" xr:uid="{F67F5632-1B2B-C049-8C5C-D8F9CF9A87E3}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2378,7 +2466,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B1CA8C7-05A5-DA44-B969-9E41B832BB96}">
-  <dimension ref="A1:E94"/>
+  <dimension ref="A1:E98"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.1640625" bestFit="1" customWidth="1"/>
@@ -3382,13 +3470,13 @@
         <v>81</v>
       </c>
       <c r="C59" s="20" t="s">
+        <v>350</v>
+      </c>
+      <c r="D59" s="22" t="s">
         <v>244</v>
       </c>
-      <c r="D59" s="22" t="s">
+      <c r="E59" s="22" t="s">
         <v>245</v>
-      </c>
-      <c r="E59" s="22" t="s">
-        <v>246</v>
       </c>
     </row>
     <row r="60" spans="1:5">
@@ -3399,13 +3487,13 @@
         <v>81</v>
       </c>
       <c r="C60" s="20" t="s">
+        <v>246</v>
+      </c>
+      <c r="D60" s="20" t="s">
         <v>247</v>
       </c>
-      <c r="D60" s="20" t="s">
+      <c r="E60" s="21" t="s">
         <v>248</v>
-      </c>
-      <c r="E60" s="21" t="s">
-        <v>249</v>
       </c>
     </row>
     <row r="61" spans="1:5">
@@ -3416,13 +3504,13 @@
         <v>81</v>
       </c>
       <c r="C61" s="20" t="s">
+        <v>249</v>
+      </c>
+      <c r="D61" s="20" t="s">
         <v>250</v>
       </c>
-      <c r="D61" s="20" t="s">
+      <c r="E61" s="21" t="s">
         <v>251</v>
-      </c>
-      <c r="E61" s="21" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="62" spans="1:5">
@@ -3433,13 +3521,13 @@
         <v>81</v>
       </c>
       <c r="C62" s="20" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D62" s="20" t="s">
         <v>181</v>
       </c>
       <c r="E62" s="21" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="63" spans="1:5">
@@ -3450,13 +3538,13 @@
         <v>81</v>
       </c>
       <c r="C63" s="20" t="s">
+        <v>254</v>
+      </c>
+      <c r="D63" s="20" t="s">
         <v>255</v>
       </c>
-      <c r="D63" s="20" t="s">
+      <c r="E63" s="21" t="s">
         <v>256</v>
-      </c>
-      <c r="E63" s="21" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="64" spans="1:5">
@@ -3467,13 +3555,13 @@
         <v>81</v>
       </c>
       <c r="C64" s="20" t="s">
+        <v>257</v>
+      </c>
+      <c r="D64" s="20" t="s">
         <v>258</v>
       </c>
-      <c r="D64" s="20" t="s">
+      <c r="E64" s="21" t="s">
         <v>259</v>
-      </c>
-      <c r="E64" s="21" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="65" spans="1:5">
@@ -3484,13 +3572,13 @@
         <v>81</v>
       </c>
       <c r="C65" s="20" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D65" s="20" t="s">
         <v>86</v>
       </c>
       <c r="E65" s="21" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="66" spans="1:5">
@@ -3504,10 +3592,10 @@
         <v>132403031</v>
       </c>
       <c r="D66" s="20" t="s">
+        <v>262</v>
+      </c>
+      <c r="E66" s="21" t="s">
         <v>263</v>
-      </c>
-      <c r="E66" s="21" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="67" spans="1:5">
@@ -3518,13 +3606,13 @@
         <v>81</v>
       </c>
       <c r="C67" s="20" t="s">
+        <v>264</v>
+      </c>
+      <c r="D67" s="20" t="s">
         <v>265</v>
       </c>
-      <c r="D67" s="20" t="s">
+      <c r="E67" s="21" t="s">
         <v>266</v>
-      </c>
-      <c r="E67" s="21" t="s">
-        <v>267</v>
       </c>
     </row>
     <row r="68" spans="1:5">
@@ -3535,13 +3623,13 @@
         <v>81</v>
       </c>
       <c r="C68" s="20" t="s">
+        <v>267</v>
+      </c>
+      <c r="D68" s="20" t="s">
         <v>268</v>
       </c>
-      <c r="D68" s="20" t="s">
+      <c r="E68" s="21" t="s">
         <v>269</v>
-      </c>
-      <c r="E68" s="21" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="69" spans="1:5">
@@ -3552,13 +3640,13 @@
         <v>81</v>
       </c>
       <c r="C69" s="20" t="s">
+        <v>270</v>
+      </c>
+      <c r="D69" s="20" t="s">
         <v>271</v>
       </c>
-      <c r="D69" s="20" t="s">
+      <c r="E69" s="21" t="s">
         <v>272</v>
-      </c>
-      <c r="E69" s="21" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="70" spans="1:5">
@@ -3569,13 +3657,13 @@
         <v>81</v>
       </c>
       <c r="C70" s="20" t="s">
+        <v>273</v>
+      </c>
+      <c r="D70" s="22" t="s">
         <v>274</v>
       </c>
-      <c r="D70" s="22" t="s">
+      <c r="E70" s="22" t="s">
         <v>275</v>
-      </c>
-      <c r="E70" s="22" t="s">
-        <v>276</v>
       </c>
     </row>
     <row r="71" spans="1:5">
@@ -3586,13 +3674,13 @@
         <v>81</v>
       </c>
       <c r="C71" s="20" t="s">
+        <v>276</v>
+      </c>
+      <c r="D71" s="20" t="s">
         <v>277</v>
       </c>
-      <c r="D71" s="20" t="s">
+      <c r="E71" s="21" t="s">
         <v>278</v>
-      </c>
-      <c r="E71" s="21" t="s">
-        <v>279</v>
       </c>
     </row>
     <row r="72" spans="1:5">
@@ -3603,13 +3691,13 @@
         <v>81</v>
       </c>
       <c r="C72" s="20" t="s">
+        <v>279</v>
+      </c>
+      <c r="D72" s="22" t="s">
         <v>280</v>
       </c>
-      <c r="D72" s="22" t="s">
+      <c r="E72" s="22" t="s">
         <v>281</v>
-      </c>
-      <c r="E72" s="22" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="73" spans="1:5">
@@ -3620,13 +3708,13 @@
         <v>81</v>
       </c>
       <c r="C73" s="20" t="s">
+        <v>282</v>
+      </c>
+      <c r="D73" s="20" t="s">
         <v>283</v>
       </c>
-      <c r="D73" s="20" t="s">
+      <c r="E73" s="21" t="s">
         <v>284</v>
-      </c>
-      <c r="E73" s="21" t="s">
-        <v>285</v>
       </c>
     </row>
     <row r="74" spans="1:5">
@@ -3637,13 +3725,13 @@
         <v>81</v>
       </c>
       <c r="C74" s="20" t="s">
+        <v>285</v>
+      </c>
+      <c r="D74" s="20" t="s">
         <v>286</v>
       </c>
-      <c r="D74" s="20" t="s">
+      <c r="E74" s="21" t="s">
         <v>287</v>
-      </c>
-      <c r="E74" s="21" t="s">
-        <v>288</v>
       </c>
     </row>
     <row r="75" spans="1:5">
@@ -3654,13 +3742,13 @@
         <v>81</v>
       </c>
       <c r="C75" s="20" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D75" s="22" t="s">
         <v>116</v>
       </c>
       <c r="E75" s="22" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="76" spans="1:5">
@@ -3671,13 +3759,13 @@
         <v>81</v>
       </c>
       <c r="C76" s="20" t="s">
+        <v>290</v>
+      </c>
+      <c r="D76" s="22" t="s">
         <v>291</v>
       </c>
-      <c r="D76" s="22" t="s">
+      <c r="E76" s="22" t="s">
         <v>292</v>
-      </c>
-      <c r="E76" s="22" t="s">
-        <v>293</v>
       </c>
     </row>
     <row r="77" spans="1:5">
@@ -3688,13 +3776,13 @@
         <v>81</v>
       </c>
       <c r="C77" s="20" t="s">
+        <v>293</v>
+      </c>
+      <c r="D77" s="22" t="s">
         <v>294</v>
       </c>
-      <c r="D77" s="22" t="s">
+      <c r="E77" s="22" t="s">
         <v>295</v>
-      </c>
-      <c r="E77" s="22" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="78" spans="1:5">
@@ -3705,13 +3793,13 @@
         <v>81</v>
       </c>
       <c r="C78" s="20" t="s">
+        <v>296</v>
+      </c>
+      <c r="D78" s="22" t="s">
         <v>297</v>
       </c>
-      <c r="D78" s="22" t="s">
+      <c r="E78" s="22" t="s">
         <v>298</v>
-      </c>
-      <c r="E78" s="22" t="s">
-        <v>299</v>
       </c>
     </row>
     <row r="79" spans="1:5">
@@ -3722,13 +3810,13 @@
         <v>81</v>
       </c>
       <c r="C79" s="20" t="s">
+        <v>299</v>
+      </c>
+      <c r="D79" s="20" t="s">
+        <v>277</v>
+      </c>
+      <c r="E79" s="21" t="s">
         <v>300</v>
-      </c>
-      <c r="D79" s="20" t="s">
-        <v>278</v>
-      </c>
-      <c r="E79" s="21" t="s">
-        <v>301</v>
       </c>
     </row>
     <row r="80" spans="1:5">
@@ -3739,13 +3827,13 @@
         <v>81</v>
       </c>
       <c r="C80" s="20" t="s">
+        <v>301</v>
+      </c>
+      <c r="D80" s="22" t="s">
         <v>302</v>
       </c>
-      <c r="D80" s="22" t="s">
+      <c r="E80" s="22" t="s">
         <v>303</v>
-      </c>
-      <c r="E80" s="22" t="s">
-        <v>304</v>
       </c>
     </row>
     <row r="81" spans="1:5">
@@ -3756,13 +3844,13 @@
         <v>81</v>
       </c>
       <c r="C81" s="20" t="s">
+        <v>304</v>
+      </c>
+      <c r="D81" s="20" t="s">
         <v>305</v>
       </c>
-      <c r="D81" s="20" t="s">
+      <c r="E81" s="21" t="s">
         <v>306</v>
-      </c>
-      <c r="E81" s="21" t="s">
-        <v>307</v>
       </c>
     </row>
     <row r="82" spans="1:5">
@@ -3773,13 +3861,13 @@
         <v>81</v>
       </c>
       <c r="C82" s="20" t="s">
+        <v>307</v>
+      </c>
+      <c r="D82" s="20" t="s">
         <v>308</v>
       </c>
-      <c r="D82" s="20" t="s">
+      <c r="E82" s="21" t="s">
         <v>309</v>
-      </c>
-      <c r="E82" s="21" t="s">
-        <v>310</v>
       </c>
     </row>
     <row r="83" spans="1:5">
@@ -3790,13 +3878,13 @@
         <v>81</v>
       </c>
       <c r="C83" s="20" t="s">
+        <v>310</v>
+      </c>
+      <c r="D83" s="20" t="s">
         <v>311</v>
       </c>
-      <c r="D83" s="20" t="s">
+      <c r="E83" s="21" t="s">
         <v>312</v>
-      </c>
-      <c r="E83" s="21" t="s">
-        <v>313</v>
       </c>
     </row>
     <row r="84" spans="1:5">
@@ -3807,13 +3895,13 @@
         <v>81</v>
       </c>
       <c r="C84" s="20" t="s">
+        <v>313</v>
+      </c>
+      <c r="D84" s="20" t="s">
         <v>314</v>
       </c>
-      <c r="D84" s="20" t="s">
-        <v>315</v>
-      </c>
       <c r="E84" s="21" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="85" spans="1:5">
@@ -3824,13 +3912,13 @@
         <v>81</v>
       </c>
       <c r="C85" s="20" t="s">
+        <v>315</v>
+      </c>
+      <c r="D85" s="20" t="s">
         <v>316</v>
       </c>
-      <c r="D85" s="20" t="s">
+      <c r="E85" s="21" t="s">
         <v>317</v>
-      </c>
-      <c r="E85" s="21" t="s">
-        <v>318</v>
       </c>
     </row>
     <row r="86" spans="1:5">
@@ -3841,13 +3929,13 @@
         <v>81</v>
       </c>
       <c r="C86" s="20" t="s">
+        <v>318</v>
+      </c>
+      <c r="D86" s="20" t="s">
+        <v>305</v>
+      </c>
+      <c r="E86" s="21" t="s">
         <v>319</v>
-      </c>
-      <c r="D86" s="20" t="s">
-        <v>306</v>
-      </c>
-      <c r="E86" s="21" t="s">
-        <v>320</v>
       </c>
     </row>
     <row r="87" spans="1:5">
@@ -3858,13 +3946,13 @@
         <v>81</v>
       </c>
       <c r="C87" s="20" t="s">
+        <v>320</v>
+      </c>
+      <c r="D87" s="20" t="s">
         <v>321</v>
       </c>
-      <c r="D87" s="20" t="s">
+      <c r="E87" s="21" t="s">
         <v>322</v>
-      </c>
-      <c r="E87" s="21" t="s">
-        <v>323</v>
       </c>
     </row>
     <row r="88" spans="1:5">
@@ -3875,13 +3963,13 @@
         <v>81</v>
       </c>
       <c r="C88" s="20" t="s">
+        <v>323</v>
+      </c>
+      <c r="D88" s="20" t="s">
+        <v>308</v>
+      </c>
+      <c r="E88" s="21" t="s">
         <v>324</v>
-      </c>
-      <c r="D88" s="20" t="s">
-        <v>309</v>
-      </c>
-      <c r="E88" s="21" t="s">
-        <v>325</v>
       </c>
     </row>
     <row r="89" spans="1:5">
@@ -3892,13 +3980,13 @@
         <v>81</v>
       </c>
       <c r="C89" s="20" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="D89" s="20" t="s">
         <v>101</v>
       </c>
       <c r="E89" s="21" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="90" spans="1:5">
@@ -3909,13 +3997,13 @@
         <v>81</v>
       </c>
       <c r="C90" s="20" t="s">
+        <v>327</v>
+      </c>
+      <c r="D90" s="20" t="s">
         <v>328</v>
       </c>
-      <c r="D90" s="20" t="s">
+      <c r="E90" s="21" t="s">
         <v>329</v>
-      </c>
-      <c r="E90" s="21" t="s">
-        <v>330</v>
       </c>
     </row>
     <row r="91" spans="1:5">
@@ -3926,13 +4014,13 @@
         <v>81</v>
       </c>
       <c r="C91" s="20" t="s">
+        <v>330</v>
+      </c>
+      <c r="D91" s="20" t="s">
         <v>331</v>
       </c>
-      <c r="D91" s="20" t="s">
+      <c r="E91" s="21" t="s">
         <v>332</v>
-      </c>
-      <c r="E91" s="21" t="s">
-        <v>333</v>
       </c>
     </row>
     <row r="92" spans="1:5">
@@ -3943,13 +4031,13 @@
         <v>81</v>
       </c>
       <c r="C92" s="20" t="s">
+        <v>333</v>
+      </c>
+      <c r="D92" s="20" t="s">
         <v>334</v>
       </c>
-      <c r="D92" s="20" t="s">
+      <c r="E92" s="21" t="s">
         <v>335</v>
-      </c>
-      <c r="E92" s="21" t="s">
-        <v>336</v>
       </c>
     </row>
     <row r="93" spans="1:5">
@@ -3960,13 +4048,13 @@
         <v>81</v>
       </c>
       <c r="C93" s="20" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D93" s="20" t="s">
         <v>193</v>
       </c>
       <c r="E93" s="21" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="94" spans="1:5">
@@ -3977,13 +4065,84 @@
         <v>81</v>
       </c>
       <c r="C94" s="20" t="s">
+        <v>338</v>
+      </c>
+      <c r="D94" s="22" t="s">
         <v>339</v>
       </c>
-      <c r="D94" s="22" t="s">
+      <c r="E94" s="22" t="s">
         <v>340</v>
       </c>
-      <c r="E94" s="22" t="s">
-        <v>341</v>
+    </row>
+    <row r="95" spans="1:5">
+      <c r="A95" s="28">
+        <v>94</v>
+      </c>
+      <c r="B95" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="C95" s="29" t="s">
+        <v>351</v>
+      </c>
+      <c r="D95" s="27" t="s">
+        <v>355</v>
+      </c>
+      <c r="E95" s="27" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5">
+      <c r="A96">
+        <f>A95+1</f>
+        <v>95</v>
+      </c>
+      <c r="B96" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="C96" s="30" t="s">
+        <v>352</v>
+      </c>
+      <c r="D96" s="31" t="s">
+        <v>101</v>
+      </c>
+      <c r="E96" s="31" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5">
+      <c r="A97">
+        <f t="shared" ref="A97:A98" si="0">A96+1</f>
+        <v>96</v>
+      </c>
+      <c r="B97" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="C97" s="26" t="s">
+        <v>353</v>
+      </c>
+      <c r="D97" s="27" t="s">
+        <v>193</v>
+      </c>
+      <c r="E97" s="27" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5">
+      <c r="A98">
+        <f t="shared" si="0"/>
+        <v>97</v>
+      </c>
+      <c r="B98" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="C98" s="26" t="s">
+        <v>354</v>
+      </c>
+      <c r="D98" s="27" t="s">
+        <v>348</v>
+      </c>
+      <c r="E98" s="27" t="s">
+        <v>349</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
publica cambios de calendario 2026-04-30 13:34
</commit_message>
<xml_diff>
--- a/Template_Calendario_CCS_GPX.xlsx
+++ b/Template_Calendario_CCS_GPX.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cesarmora/Library/Mobile Documents/com~apple~CloudDocs/Personal/Ciclismo/Calendario/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0865E891-110F-BD41-8940-B74838D0B8F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A58F67AC-FF5A-B24A-BA5B-0140F4642702}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12200" yWindow="1420" windowWidth="20720" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12200" yWindow="780" windowWidth="20720" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template_Calendario_CCS" sheetId="1" r:id="rId1"/>
@@ -2109,16 +2109,16 @@
         <v>6</v>
       </c>
       <c r="C24" t="s">
-        <v>345</v>
+        <v>17</v>
       </c>
       <c r="D24" t="s">
-        <v>347</v>
+        <v>34</v>
       </c>
       <c r="E24" s="10" t="s">
         <v>41</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>346</v>
+        <v>48</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -2456,9 +2456,9 @@
     <hyperlink ref="E16" r:id="rId23" xr:uid="{35C172B7-7936-AF4E-B1C2-147C8E7867CA}"/>
     <hyperlink ref="E19" r:id="rId24" xr:uid="{08AE7119-345F-9D47-997F-67E247E970E5}"/>
     <hyperlink ref="E35" r:id="rId25" xr:uid="{13AFCAE5-A888-BD46-A83F-C77F11E366D7}"/>
-    <hyperlink ref="E24" r:id="rId26" xr:uid="{CF7403E1-E9E7-EC40-BE26-3A6B792A99C1}"/>
-    <hyperlink ref="E20" r:id="rId27" xr:uid="{8866888E-71DF-3944-9620-4E948829D43F}"/>
-    <hyperlink ref="E25" r:id="rId28" xr:uid="{F67F5632-1B2B-C049-8C5C-D8F9CF9A87E3}"/>
+    <hyperlink ref="E20" r:id="rId26" xr:uid="{8866888E-71DF-3944-9620-4E948829D43F}"/>
+    <hyperlink ref="E25" r:id="rId27" xr:uid="{F67F5632-1B2B-C049-8C5C-D8F9CF9A87E3}"/>
+    <hyperlink ref="E24" r:id="rId28" xr:uid="{F51A13EB-7897-0D42-A463-97945F82F47E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
publica cambios de calendario 2026-04-30 13:43
</commit_message>
<xml_diff>
--- a/Template_Calendario_CCS_GPX.xlsx
+++ b/Template_Calendario_CCS_GPX.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cesarmora/Library/Mobile Documents/com~apple~CloudDocs/Personal/Ciclismo/Calendario/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A58F67AC-FF5A-B24A-BA5B-0140F4642702}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{647B7200-F0ED-7F4F-9CA4-DCD88671F4CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="12200" yWindow="780" windowWidth="20720" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="359">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="358">
   <si>
     <t>Fecha</t>
   </si>
@@ -91,9 +91,6 @@
   </si>
   <si>
     <t>Vizcachas - Embalse el Yeso (Bis)</t>
-  </si>
-  <si>
-    <t>Viaje Colchagua: 3 dias</t>
   </si>
   <si>
     <t>Viña undurraga - Cuesta Chada (Bis)</t>
@@ -1646,19 +1643,19 @@
         <v>5</v>
       </c>
       <c r="G1" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="H1" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="I1" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="J1" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="J1" s="12" t="s">
+      <c r="K1" s="12" t="s">
         <v>46</v>
-      </c>
-      <c r="K1" s="12" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:11">
@@ -1672,13 +1669,13 @@
         <v>8</v>
       </c>
       <c r="D2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -1692,13 +1689,13 @@
         <v>9</v>
       </c>
       <c r="D3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -1712,13 +1709,13 @@
         <v>10</v>
       </c>
       <c r="D4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -1732,13 +1729,13 @@
         <v>11</v>
       </c>
       <c r="D5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -1752,13 +1749,13 @@
         <v>12</v>
       </c>
       <c r="D6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -1772,13 +1769,13 @@
         <v>13</v>
       </c>
       <c r="D7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -1792,13 +1789,13 @@
         <v>14</v>
       </c>
       <c r="D8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -1812,13 +1809,13 @@
         <v>15</v>
       </c>
       <c r="D9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -1829,16 +1826,16 @@
         <v>7</v>
       </c>
       <c r="C10" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="D10" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -1849,16 +1846,16 @@
         <v>7</v>
       </c>
       <c r="C11" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="D11" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -1872,13 +1869,13 @@
         <v>16</v>
       </c>
       <c r="D12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -1892,13 +1889,13 @@
         <v>17</v>
       </c>
       <c r="D13" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -1909,16 +1906,16 @@
         <v>6</v>
       </c>
       <c r="C14" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D14" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -1932,13 +1929,13 @@
         <v>18</v>
       </c>
       <c r="D15" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -1949,16 +1946,16 @@
         <v>6</v>
       </c>
       <c r="C16" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D16" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -1969,16 +1966,16 @@
         <v>6</v>
       </c>
       <c r="C17" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D17" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -1989,16 +1986,16 @@
         <v>6</v>
       </c>
       <c r="C18" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D18" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -2012,13 +2009,13 @@
         <v>11</v>
       </c>
       <c r="D19" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -2029,16 +2026,16 @@
         <v>6</v>
       </c>
       <c r="C20" t="s">
+        <v>342</v>
+      </c>
+      <c r="D20" t="s">
+        <v>29</v>
+      </c>
+      <c r="E20" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="F20" s="5" t="s">
         <v>343</v>
-      </c>
-      <c r="D20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E20" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="F20" s="5" t="s">
-        <v>344</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -2049,16 +2046,16 @@
         <v>7</v>
       </c>
       <c r="C21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D21" t="s">
-        <v>19</v>
+        <v>50</v>
       </c>
       <c r="E21" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -2069,16 +2066,16 @@
         <v>7</v>
       </c>
       <c r="C22" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D22" t="s">
-        <v>19</v>
+        <v>51</v>
       </c>
       <c r="E22" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -2089,16 +2086,16 @@
         <v>7</v>
       </c>
       <c r="C23" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D23" t="s">
-        <v>19</v>
+        <v>52</v>
       </c>
       <c r="E23" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -2112,13 +2109,13 @@
         <v>17</v>
       </c>
       <c r="D24" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -2129,16 +2126,16 @@
         <v>6</v>
       </c>
       <c r="C25" t="s">
+        <v>344</v>
+      </c>
+      <c r="D25" t="s">
+        <v>346</v>
+      </c>
+      <c r="E25" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="F25" s="5" t="s">
         <v>345</v>
-      </c>
-      <c r="D25" t="s">
-        <v>347</v>
-      </c>
-      <c r="E25" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="F25" s="5" t="s">
-        <v>346</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -2149,16 +2146,16 @@
         <v>6</v>
       </c>
       <c r="C26" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D26" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -2169,16 +2166,16 @@
         <v>6</v>
       </c>
       <c r="C27" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D27" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -2189,16 +2186,16 @@
         <v>6</v>
       </c>
       <c r="C28" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D28" t="s">
+        <v>39</v>
+      </c>
+      <c r="E28" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="E28" s="10" t="s">
-        <v>41</v>
-      </c>
       <c r="F28" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -2209,16 +2206,16 @@
         <v>6</v>
       </c>
       <c r="C29" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D29" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="30" spans="1:6">
@@ -2229,16 +2226,16 @@
         <v>6</v>
       </c>
       <c r="C30" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D30" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="31" spans="1:6">
@@ -2249,16 +2246,16 @@
         <v>7</v>
       </c>
       <c r="C31" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D31" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E31" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -2269,16 +2266,16 @@
         <v>7</v>
       </c>
       <c r="C32" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D32" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E32" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="33" spans="1:6">
@@ -2289,16 +2286,16 @@
         <v>7</v>
       </c>
       <c r="C33" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D33" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E33" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="34" spans="1:6">
@@ -2309,16 +2306,16 @@
         <v>6</v>
       </c>
       <c r="C34" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D34" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="35" spans="1:6">
@@ -2332,13 +2329,13 @@
         <v>9</v>
       </c>
       <c r="D35" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="36" spans="1:6">
@@ -2478,19 +2475,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="B1" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="C1" s="16" t="s">
         <v>77</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="D1" s="16" t="s">
         <v>78</v>
       </c>
-      <c r="D1" s="16" t="s">
+      <c r="E1" s="17" t="s">
         <v>79</v>
-      </c>
-      <c r="E1" s="17" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -2498,16 +2495,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="19" t="s">
+        <v>80</v>
+      </c>
+      <c r="C2" s="20" t="s">
         <v>81</v>
       </c>
-      <c r="C2" s="20" t="s">
+      <c r="D2" s="20" t="s">
         <v>82</v>
       </c>
-      <c r="D2" s="20" t="s">
+      <c r="E2" s="21" t="s">
         <v>83</v>
-      </c>
-      <c r="E2" s="21" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -2515,16 +2512,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C3" s="20" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="D3" s="20" t="s">
+      <c r="E3" s="21" t="s">
         <v>86</v>
-      </c>
-      <c r="E3" s="21" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -2532,16 +2529,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C4" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="D4" s="22" t="s">
         <v>88</v>
       </c>
-      <c r="D4" s="22" t="s">
+      <c r="E4" s="22" t="s">
         <v>89</v>
-      </c>
-      <c r="E4" s="22" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -2549,16 +2546,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C5" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="D5" s="22" t="s">
         <v>91</v>
       </c>
-      <c r="D5" s="22" t="s">
+      <c r="E5" s="22" t="s">
         <v>92</v>
-      </c>
-      <c r="E5" s="22" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -2566,16 +2563,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C6" s="20" t="s">
+        <v>93</v>
+      </c>
+      <c r="D6" s="22" t="s">
         <v>94</v>
       </c>
-      <c r="D6" s="22" t="s">
+      <c r="E6" s="22" t="s">
         <v>95</v>
-      </c>
-      <c r="E6" s="22" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -2583,16 +2580,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C7" s="20" t="s">
+        <v>96</v>
+      </c>
+      <c r="D7" s="20" t="s">
         <v>97</v>
       </c>
-      <c r="D7" s="20" t="s">
+      <c r="E7" s="20" t="s">
         <v>98</v>
-      </c>
-      <c r="E7" s="20" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -2600,16 +2597,16 @@
         <v>7</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C8" s="20" t="s">
+        <v>99</v>
+      </c>
+      <c r="D8" s="20" t="s">
         <v>100</v>
       </c>
-      <c r="D8" s="20" t="s">
+      <c r="E8" s="21" t="s">
         <v>101</v>
-      </c>
-      <c r="E8" s="21" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -2617,16 +2614,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C9" s="20" t="s">
+        <v>102</v>
+      </c>
+      <c r="D9" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="D9" s="20" t="s">
+      <c r="E9" s="21" t="s">
         <v>104</v>
-      </c>
-      <c r="E9" s="21" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -2634,16 +2631,16 @@
         <v>9</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C10" s="20" t="s">
+        <v>105</v>
+      </c>
+      <c r="D10" s="22" t="s">
         <v>106</v>
       </c>
-      <c r="D10" s="22" t="s">
+      <c r="E10" s="22" t="s">
         <v>107</v>
-      </c>
-      <c r="E10" s="22" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -2651,16 +2648,16 @@
         <v>10</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C11" s="20" t="s">
+        <v>108</v>
+      </c>
+      <c r="D11" s="22" t="s">
         <v>109</v>
       </c>
-      <c r="D11" s="22" t="s">
+      <c r="E11" s="22" t="s">
         <v>110</v>
-      </c>
-      <c r="E11" s="22" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -2668,16 +2665,16 @@
         <v>11</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C12" s="20" t="s">
+        <v>111</v>
+      </c>
+      <c r="D12" s="20" t="s">
         <v>112</v>
       </c>
-      <c r="D12" s="20" t="s">
+      <c r="E12" s="21" t="s">
         <v>113</v>
-      </c>
-      <c r="E12" s="21" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -2685,16 +2682,16 @@
         <v>12</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C13" s="20" t="s">
+        <v>114</v>
+      </c>
+      <c r="D13" s="20" t="s">
         <v>115</v>
       </c>
-      <c r="D13" s="20" t="s">
-        <v>116</v>
-      </c>
       <c r="E13" s="21" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -2702,16 +2699,16 @@
         <v>13</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C14" s="20" t="s">
+        <v>116</v>
+      </c>
+      <c r="D14" s="20" t="s">
         <v>117</v>
       </c>
-      <c r="D14" s="20" t="s">
+      <c r="E14" s="21" t="s">
         <v>118</v>
-      </c>
-      <c r="E14" s="21" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -2719,16 +2716,16 @@
         <v>14</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C15" s="20" t="s">
+        <v>119</v>
+      </c>
+      <c r="D15" s="20" t="s">
         <v>120</v>
       </c>
-      <c r="D15" s="20" t="s">
+      <c r="E15" s="21" t="s">
         <v>121</v>
-      </c>
-      <c r="E15" s="21" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -2736,16 +2733,16 @@
         <v>15</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C16" s="20" t="s">
+        <v>122</v>
+      </c>
+      <c r="D16" s="20" t="s">
         <v>123</v>
       </c>
-      <c r="D16" s="20" t="s">
+      <c r="E16" s="21" t="s">
         <v>124</v>
-      </c>
-      <c r="E16" s="21" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -2753,16 +2750,16 @@
         <v>16</v>
       </c>
       <c r="B17" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C17" s="20" t="s">
+        <v>125</v>
+      </c>
+      <c r="D17" s="20" t="s">
         <v>126</v>
       </c>
-      <c r="D17" s="20" t="s">
+      <c r="E17" s="21" t="s">
         <v>127</v>
-      </c>
-      <c r="E17" s="21" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -2770,16 +2767,16 @@
         <v>17</v>
       </c>
       <c r="B18" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C18" s="20" t="s">
+        <v>128</v>
+      </c>
+      <c r="D18" s="20" t="s">
         <v>129</v>
       </c>
-      <c r="D18" s="20" t="s">
+      <c r="E18" s="21" t="s">
         <v>130</v>
-      </c>
-      <c r="E18" s="21" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -2787,16 +2784,16 @@
         <v>18</v>
       </c>
       <c r="B19" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C19" s="20" t="s">
+        <v>131</v>
+      </c>
+      <c r="D19" s="20" t="s">
         <v>132</v>
       </c>
-      <c r="D19" s="20" t="s">
-        <v>133</v>
-      </c>
       <c r="E19" s="21" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -2804,16 +2801,16 @@
         <v>19</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C20" s="20" t="s">
+        <v>133</v>
+      </c>
+      <c r="D20" s="20" t="s">
         <v>134</v>
       </c>
-      <c r="D20" s="20" t="s">
+      <c r="E20" s="21" t="s">
         <v>135</v>
-      </c>
-      <c r="E20" s="21" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -2821,16 +2818,16 @@
         <v>20</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C21" s="20" t="s">
+        <v>136</v>
+      </c>
+      <c r="D21" s="22" t="s">
         <v>137</v>
       </c>
-      <c r="D21" s="22" t="s">
+      <c r="E21" s="22" t="s">
         <v>138</v>
-      </c>
-      <c r="E21" s="22" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -2838,16 +2835,16 @@
         <v>21</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C22" s="20" t="s">
+        <v>139</v>
+      </c>
+      <c r="D22" s="22" t="s">
         <v>140</v>
       </c>
-      <c r="D22" s="22" t="s">
+      <c r="E22" s="22" t="s">
         <v>141</v>
-      </c>
-      <c r="E22" s="22" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -2855,16 +2852,16 @@
         <v>22</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C23" s="20" t="s">
+        <v>142</v>
+      </c>
+      <c r="D23" s="20" t="s">
         <v>143</v>
       </c>
-      <c r="D23" s="20" t="s">
+      <c r="E23" s="21" t="s">
         <v>144</v>
-      </c>
-      <c r="E23" s="21" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -2872,16 +2869,16 @@
         <v>23</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C24" s="20" t="s">
+        <v>145</v>
+      </c>
+      <c r="D24" s="20" t="s">
         <v>146</v>
       </c>
-      <c r="D24" s="20" t="s">
+      <c r="E24" s="21" t="s">
         <v>147</v>
-      </c>
-      <c r="E24" s="21" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -2889,16 +2886,16 @@
         <v>24</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C25" s="20" t="s">
+        <v>148</v>
+      </c>
+      <c r="D25" s="20" t="s">
         <v>149</v>
       </c>
-      <c r="D25" s="20" t="s">
+      <c r="E25" s="21" t="s">
         <v>150</v>
-      </c>
-      <c r="E25" s="21" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -2906,16 +2903,16 @@
         <v>25</v>
       </c>
       <c r="B26" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C26" s="20" t="s">
+        <v>151</v>
+      </c>
+      <c r="D26" s="22" t="s">
         <v>152</v>
       </c>
-      <c r="D26" s="22" t="s">
+      <c r="E26" s="22" t="s">
         <v>153</v>
-      </c>
-      <c r="E26" s="22" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -2923,16 +2920,16 @@
         <v>26</v>
       </c>
       <c r="B27" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C27" s="20" t="s">
+        <v>154</v>
+      </c>
+      <c r="D27" s="20" t="s">
         <v>155</v>
       </c>
-      <c r="D27" s="20" t="s">
+      <c r="E27" s="21" t="s">
         <v>156</v>
-      </c>
-      <c r="E27" s="21" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -2940,16 +2937,16 @@
         <v>27</v>
       </c>
       <c r="B28" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C28" s="20" t="s">
+        <v>157</v>
+      </c>
+      <c r="D28" s="20" t="s">
         <v>158</v>
       </c>
-      <c r="D28" s="20" t="s">
+      <c r="E28" s="21" t="s">
         <v>159</v>
-      </c>
-      <c r="E28" s="21" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -2957,16 +2954,16 @@
         <v>28</v>
       </c>
       <c r="B29" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C29" s="20" t="s">
+        <v>160</v>
+      </c>
+      <c r="D29" s="20" t="s">
         <v>161</v>
       </c>
-      <c r="D29" s="20" t="s">
+      <c r="E29" s="21" t="s">
         <v>162</v>
-      </c>
-      <c r="E29" s="21" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="30" spans="1:5">
@@ -2974,16 +2971,16 @@
         <v>29</v>
       </c>
       <c r="B30" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C30" s="20" t="s">
+        <v>163</v>
+      </c>
+      <c r="D30" s="22" t="s">
         <v>164</v>
       </c>
-      <c r="D30" s="22" t="s">
+      <c r="E30" s="22" t="s">
         <v>165</v>
-      </c>
-      <c r="E30" s="22" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="31" spans="1:5">
@@ -2991,16 +2988,16 @@
         <v>30</v>
       </c>
       <c r="B31" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C31" s="20" t="s">
+        <v>166</v>
+      </c>
+      <c r="D31" s="20" t="s">
         <v>167</v>
       </c>
-      <c r="D31" s="20" t="s">
+      <c r="E31" s="21" t="s">
         <v>168</v>
-      </c>
-      <c r="E31" s="21" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="32" spans="1:5">
@@ -3008,16 +3005,16 @@
         <v>31</v>
       </c>
       <c r="B32" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C32" s="20" t="s">
+        <v>169</v>
+      </c>
+      <c r="D32" s="20" t="s">
         <v>170</v>
       </c>
-      <c r="D32" s="20" t="s">
+      <c r="E32" s="21" t="s">
         <v>171</v>
-      </c>
-      <c r="E32" s="21" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="33" spans="1:5">
@@ -3025,16 +3022,16 @@
         <v>32</v>
       </c>
       <c r="B33" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C33" s="20" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D33" s="20" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E33" s="21" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="34" spans="1:5">
@@ -3042,16 +3039,16 @@
         <v>33</v>
       </c>
       <c r="B34" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C34" s="20" t="s">
+        <v>173</v>
+      </c>
+      <c r="D34" s="20" t="s">
         <v>174</v>
       </c>
-      <c r="D34" s="20" t="s">
+      <c r="E34" s="21" t="s">
         <v>175</v>
-      </c>
-      <c r="E34" s="21" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="35" spans="1:5">
@@ -3059,16 +3056,16 @@
         <v>34</v>
       </c>
       <c r="B35" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C35" s="20" t="s">
+        <v>176</v>
+      </c>
+      <c r="D35" s="20" t="s">
         <v>177</v>
       </c>
-      <c r="D35" s="20" t="s">
+      <c r="E35" s="21" t="s">
         <v>178</v>
-      </c>
-      <c r="E35" s="21" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="36" spans="1:5">
@@ -3076,16 +3073,16 @@
         <v>35</v>
       </c>
       <c r="B36" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C36" s="20" t="s">
+        <v>179</v>
+      </c>
+      <c r="D36" s="20" t="s">
         <v>180</v>
       </c>
-      <c r="D36" s="20" t="s">
+      <c r="E36" s="21" t="s">
         <v>181</v>
-      </c>
-      <c r="E36" s="21" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="37" spans="1:5">
@@ -3093,16 +3090,16 @@
         <v>36</v>
       </c>
       <c r="B37" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C37" s="20" t="s">
+        <v>182</v>
+      </c>
+      <c r="D37" s="20" t="s">
         <v>183</v>
       </c>
-      <c r="D37" s="20" t="s">
+      <c r="E37" s="21" t="s">
         <v>184</v>
-      </c>
-      <c r="E37" s="21" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="38" spans="1:5">
@@ -3110,16 +3107,16 @@
         <v>37</v>
       </c>
       <c r="B38" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C38" s="20" t="s">
+        <v>185</v>
+      </c>
+      <c r="D38" s="20" t="s">
         <v>186</v>
       </c>
-      <c r="D38" s="20" t="s">
+      <c r="E38" s="21" t="s">
         <v>187</v>
-      </c>
-      <c r="E38" s="21" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="39" spans="1:5">
@@ -3127,16 +3124,16 @@
         <v>38</v>
       </c>
       <c r="B39" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C39" s="20" t="s">
+        <v>188</v>
+      </c>
+      <c r="D39" s="20" t="s">
         <v>189</v>
       </c>
-      <c r="D39" s="20" t="s">
+      <c r="E39" s="21" t="s">
         <v>190</v>
-      </c>
-      <c r="E39" s="21" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="40" spans="1:5">
@@ -3144,16 +3141,16 @@
         <v>39</v>
       </c>
       <c r="B40" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C40" s="20" t="s">
+        <v>191</v>
+      </c>
+      <c r="D40" s="20" t="s">
         <v>192</v>
       </c>
-      <c r="D40" s="20" t="s">
+      <c r="E40" s="21" t="s">
         <v>193</v>
-      </c>
-      <c r="E40" s="21" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="41" spans="1:5">
@@ -3161,16 +3158,16 @@
         <v>40</v>
       </c>
       <c r="B41" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C41" s="24" t="s">
+        <v>194</v>
+      </c>
+      <c r="D41" s="20" t="s">
         <v>195</v>
       </c>
-      <c r="D41" s="20" t="s">
+      <c r="E41" s="21" t="s">
         <v>196</v>
-      </c>
-      <c r="E41" s="21" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="42" spans="1:5">
@@ -3178,16 +3175,16 @@
         <v>41</v>
       </c>
       <c r="B42" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C42" s="20" t="s">
+        <v>197</v>
+      </c>
+      <c r="D42" s="22" t="s">
+        <v>180</v>
+      </c>
+      <c r="E42" s="22" t="s">
         <v>198</v>
-      </c>
-      <c r="D42" s="22" t="s">
-        <v>181</v>
-      </c>
-      <c r="E42" s="22" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="43" spans="1:5">
@@ -3195,16 +3192,16 @@
         <v>42</v>
       </c>
       <c r="B43" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C43" s="20" t="s">
+        <v>199</v>
+      </c>
+      <c r="D43" s="22" t="s">
         <v>200</v>
       </c>
-      <c r="D43" s="22" t="s">
+      <c r="E43" s="22" t="s">
         <v>201</v>
-      </c>
-      <c r="E43" s="22" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="44" spans="1:5">
@@ -3212,16 +3209,16 @@
         <v>43</v>
       </c>
       <c r="B44" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C44" s="20" t="s">
+        <v>202</v>
+      </c>
+      <c r="D44" s="20" t="s">
         <v>203</v>
       </c>
-      <c r="D44" s="20" t="s">
+      <c r="E44" s="21" t="s">
         <v>204</v>
-      </c>
-      <c r="E44" s="21" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="45" spans="1:5">
@@ -3229,16 +3226,16 @@
         <v>44</v>
       </c>
       <c r="B45" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C45" s="20" t="s">
+        <v>205</v>
+      </c>
+      <c r="D45" s="22" t="s">
         <v>206</v>
       </c>
-      <c r="D45" s="22" t="s">
+      <c r="E45" s="22" t="s">
         <v>207</v>
-      </c>
-      <c r="E45" s="22" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="46" spans="1:5">
@@ -3246,16 +3243,16 @@
         <v>45</v>
       </c>
       <c r="B46" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C46" s="23" t="s">
+        <v>208</v>
+      </c>
+      <c r="D46" s="20" t="s">
+        <v>134</v>
+      </c>
+      <c r="E46" s="21" t="s">
         <v>209</v>
-      </c>
-      <c r="D46" s="20" t="s">
-        <v>135</v>
-      </c>
-      <c r="E46" s="21" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="47" spans="1:5">
@@ -3263,16 +3260,16 @@
         <v>46</v>
       </c>
       <c r="B47" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C47" s="20" t="s">
+        <v>210</v>
+      </c>
+      <c r="D47" s="20" t="s">
         <v>211</v>
       </c>
-      <c r="D47" s="20" t="s">
+      <c r="E47" s="21" t="s">
         <v>212</v>
-      </c>
-      <c r="E47" s="21" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="48" spans="1:5">
@@ -3280,16 +3277,16 @@
         <v>47</v>
       </c>
       <c r="B48" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C48" s="20" t="s">
+        <v>213</v>
+      </c>
+      <c r="D48" s="20" t="s">
         <v>214</v>
       </c>
-      <c r="D48" s="20" t="s">
+      <c r="E48" s="21" t="s">
         <v>215</v>
-      </c>
-      <c r="E48" s="21" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="49" spans="1:5">
@@ -3297,16 +3294,16 @@
         <v>48</v>
       </c>
       <c r="B49" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C49" s="20" t="s">
+        <v>216</v>
+      </c>
+      <c r="D49" s="20" t="s">
+        <v>161</v>
+      </c>
+      <c r="E49" s="21" t="s">
         <v>217</v>
-      </c>
-      <c r="D49" s="20" t="s">
-        <v>162</v>
-      </c>
-      <c r="E49" s="21" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="50" spans="1:5">
@@ -3314,16 +3311,16 @@
         <v>49</v>
       </c>
       <c r="B50" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C50" s="20" t="s">
+        <v>218</v>
+      </c>
+      <c r="D50" s="22" t="s">
+        <v>100</v>
+      </c>
+      <c r="E50" s="22" t="s">
         <v>219</v>
-      </c>
-      <c r="D50" s="22" t="s">
-        <v>101</v>
-      </c>
-      <c r="E50" s="22" t="s">
-        <v>220</v>
       </c>
     </row>
     <row r="51" spans="1:5">
@@ -3331,16 +3328,16 @@
         <v>50</v>
       </c>
       <c r="B51" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C51" s="20" t="s">
+        <v>220</v>
+      </c>
+      <c r="D51" s="20" t="s">
         <v>221</v>
       </c>
-      <c r="D51" s="20" t="s">
+      <c r="E51" s="21" t="s">
         <v>222</v>
-      </c>
-      <c r="E51" s="21" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="52" spans="1:5">
@@ -3348,16 +3345,16 @@
         <v>51</v>
       </c>
       <c r="B52" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C52" s="20" t="s">
+        <v>223</v>
+      </c>
+      <c r="D52" s="20" t="s">
         <v>224</v>
       </c>
-      <c r="D52" s="20" t="s">
-        <v>225</v>
-      </c>
       <c r="E52" s="21" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="53" spans="1:5">
@@ -3365,16 +3362,16 @@
         <v>52</v>
       </c>
       <c r="B53" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C53" s="20" t="s">
+        <v>225</v>
+      </c>
+      <c r="D53" s="20" t="s">
         <v>226</v>
       </c>
-      <c r="D53" s="20" t="s">
+      <c r="E53" s="21" t="s">
         <v>227</v>
-      </c>
-      <c r="E53" s="21" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="54" spans="1:5">
@@ -3382,16 +3379,16 @@
         <v>53</v>
       </c>
       <c r="B54" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C54" s="20" t="s">
+        <v>228</v>
+      </c>
+      <c r="D54" s="20" t="s">
         <v>229</v>
       </c>
-      <c r="D54" s="20" t="s">
+      <c r="E54" s="21" t="s">
         <v>230</v>
-      </c>
-      <c r="E54" s="21" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="55" spans="1:5">
@@ -3399,16 +3396,16 @@
         <v>54</v>
       </c>
       <c r="B55" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C55" s="20" t="s">
+        <v>231</v>
+      </c>
+      <c r="D55" s="20" t="s">
         <v>232</v>
       </c>
-      <c r="D55" s="20" t="s">
+      <c r="E55" s="21" t="s">
         <v>233</v>
-      </c>
-      <c r="E55" s="21" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="56" spans="1:5">
@@ -3416,16 +3413,16 @@
         <v>55</v>
       </c>
       <c r="B56" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C56" s="20" t="s">
+        <v>234</v>
+      </c>
+      <c r="D56" s="22" t="s">
         <v>235</v>
       </c>
-      <c r="D56" s="22" t="s">
+      <c r="E56" s="22" t="s">
         <v>236</v>
-      </c>
-      <c r="E56" s="22" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="57" spans="1:5">
@@ -3433,16 +3430,16 @@
         <v>56</v>
       </c>
       <c r="B57" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C57" s="20" t="s">
+        <v>237</v>
+      </c>
+      <c r="D57" s="22" t="s">
         <v>238</v>
       </c>
-      <c r="D57" s="22" t="s">
+      <c r="E57" s="22" t="s">
         <v>239</v>
-      </c>
-      <c r="E57" s="22" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="58" spans="1:5">
@@ -3450,16 +3447,16 @@
         <v>57</v>
       </c>
       <c r="B58" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C58" s="20" t="s">
+        <v>240</v>
+      </c>
+      <c r="D58" s="20" t="s">
         <v>241</v>
       </c>
-      <c r="D58" s="20" t="s">
+      <c r="E58" s="21" t="s">
         <v>242</v>
-      </c>
-      <c r="E58" s="21" t="s">
-        <v>243</v>
       </c>
     </row>
     <row r="59" spans="1:5">
@@ -3467,16 +3464,16 @@
         <v>58</v>
       </c>
       <c r="B59" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C59" s="20" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="D59" s="22" t="s">
+        <v>243</v>
+      </c>
+      <c r="E59" s="22" t="s">
         <v>244</v>
-      </c>
-      <c r="E59" s="22" t="s">
-        <v>245</v>
       </c>
     </row>
     <row r="60" spans="1:5">
@@ -3484,16 +3481,16 @@
         <v>59</v>
       </c>
       <c r="B60" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C60" s="20" t="s">
+        <v>245</v>
+      </c>
+      <c r="D60" s="20" t="s">
         <v>246</v>
       </c>
-      <c r="D60" s="20" t="s">
+      <c r="E60" s="21" t="s">
         <v>247</v>
-      </c>
-      <c r="E60" s="21" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="61" spans="1:5">
@@ -3501,16 +3498,16 @@
         <v>60</v>
       </c>
       <c r="B61" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C61" s="20" t="s">
+        <v>248</v>
+      </c>
+      <c r="D61" s="20" t="s">
         <v>249</v>
       </c>
-      <c r="D61" s="20" t="s">
+      <c r="E61" s="21" t="s">
         <v>250</v>
-      </c>
-      <c r="E61" s="21" t="s">
-        <v>251</v>
       </c>
     </row>
     <row r="62" spans="1:5">
@@ -3518,16 +3515,16 @@
         <v>61</v>
       </c>
       <c r="B62" s="22" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C62" s="20" t="s">
+        <v>251</v>
+      </c>
+      <c r="D62" s="20" t="s">
+        <v>180</v>
+      </c>
+      <c r="E62" s="21" t="s">
         <v>252</v>
-      </c>
-      <c r="D62" s="20" t="s">
-        <v>181</v>
-      </c>
-      <c r="E62" s="21" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="63" spans="1:5">
@@ -3535,16 +3532,16 @@
         <v>62</v>
       </c>
       <c r="B63" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C63" s="20" t="s">
+        <v>253</v>
+      </c>
+      <c r="D63" s="20" t="s">
         <v>254</v>
       </c>
-      <c r="D63" s="20" t="s">
+      <c r="E63" s="21" t="s">
         <v>255</v>
-      </c>
-      <c r="E63" s="21" t="s">
-        <v>256</v>
       </c>
     </row>
     <row r="64" spans="1:5">
@@ -3552,16 +3549,16 @@
         <v>63</v>
       </c>
       <c r="B64" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C64" s="20" t="s">
+        <v>256</v>
+      </c>
+      <c r="D64" s="20" t="s">
         <v>257</v>
       </c>
-      <c r="D64" s="20" t="s">
+      <c r="E64" s="21" t="s">
         <v>258</v>
-      </c>
-      <c r="E64" s="21" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="65" spans="1:5">
@@ -3569,16 +3566,16 @@
         <v>64</v>
       </c>
       <c r="B65" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C65" s="20" t="s">
+        <v>259</v>
+      </c>
+      <c r="D65" s="20" t="s">
+        <v>85</v>
+      </c>
+      <c r="E65" s="21" t="s">
         <v>260</v>
-      </c>
-      <c r="D65" s="20" t="s">
-        <v>86</v>
-      </c>
-      <c r="E65" s="21" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="66" spans="1:5">
@@ -3586,16 +3583,16 @@
         <v>65</v>
       </c>
       <c r="B66" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C66" s="20">
         <v>132403031</v>
       </c>
       <c r="D66" s="20" t="s">
+        <v>261</v>
+      </c>
+      <c r="E66" s="21" t="s">
         <v>262</v>
-      </c>
-      <c r="E66" s="21" t="s">
-        <v>263</v>
       </c>
     </row>
     <row r="67" spans="1:5">
@@ -3603,16 +3600,16 @@
         <v>66</v>
       </c>
       <c r="B67" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C67" s="20" t="s">
+        <v>263</v>
+      </c>
+      <c r="D67" s="20" t="s">
         <v>264</v>
       </c>
-      <c r="D67" s="20" t="s">
+      <c r="E67" s="21" t="s">
         <v>265</v>
-      </c>
-      <c r="E67" s="21" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="68" spans="1:5">
@@ -3620,16 +3617,16 @@
         <v>67</v>
       </c>
       <c r="B68" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C68" s="20" t="s">
+        <v>266</v>
+      </c>
+      <c r="D68" s="20" t="s">
         <v>267</v>
       </c>
-      <c r="D68" s="20" t="s">
+      <c r="E68" s="21" t="s">
         <v>268</v>
-      </c>
-      <c r="E68" s="21" t="s">
-        <v>269</v>
       </c>
     </row>
     <row r="69" spans="1:5">
@@ -3637,16 +3634,16 @@
         <v>68</v>
       </c>
       <c r="B69" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C69" s="20" t="s">
+        <v>269</v>
+      </c>
+      <c r="D69" s="20" t="s">
         <v>270</v>
       </c>
-      <c r="D69" s="20" t="s">
+      <c r="E69" s="21" t="s">
         <v>271</v>
-      </c>
-      <c r="E69" s="21" t="s">
-        <v>272</v>
       </c>
     </row>
     <row r="70" spans="1:5">
@@ -3654,16 +3651,16 @@
         <v>69</v>
       </c>
       <c r="B70" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C70" s="20" t="s">
+        <v>272</v>
+      </c>
+      <c r="D70" s="22" t="s">
         <v>273</v>
       </c>
-      <c r="D70" s="22" t="s">
+      <c r="E70" s="22" t="s">
         <v>274</v>
-      </c>
-      <c r="E70" s="22" t="s">
-        <v>275</v>
       </c>
     </row>
     <row r="71" spans="1:5">
@@ -3671,16 +3668,16 @@
         <v>70</v>
       </c>
       <c r="B71" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C71" s="20" t="s">
+        <v>275</v>
+      </c>
+      <c r="D71" s="20" t="s">
         <v>276</v>
       </c>
-      <c r="D71" s="20" t="s">
+      <c r="E71" s="21" t="s">
         <v>277</v>
-      </c>
-      <c r="E71" s="21" t="s">
-        <v>278</v>
       </c>
     </row>
     <row r="72" spans="1:5">
@@ -3688,16 +3685,16 @@
         <v>71</v>
       </c>
       <c r="B72" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C72" s="20" t="s">
+        <v>278</v>
+      </c>
+      <c r="D72" s="22" t="s">
         <v>279</v>
       </c>
-      <c r="D72" s="22" t="s">
+      <c r="E72" s="22" t="s">
         <v>280</v>
-      </c>
-      <c r="E72" s="22" t="s">
-        <v>281</v>
       </c>
     </row>
     <row r="73" spans="1:5">
@@ -3705,16 +3702,16 @@
         <v>72</v>
       </c>
       <c r="B73" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C73" s="20" t="s">
+        <v>281</v>
+      </c>
+      <c r="D73" s="20" t="s">
         <v>282</v>
       </c>
-      <c r="D73" s="20" t="s">
+      <c r="E73" s="21" t="s">
         <v>283</v>
-      </c>
-      <c r="E73" s="21" t="s">
-        <v>284</v>
       </c>
     </row>
     <row r="74" spans="1:5">
@@ -3722,16 +3719,16 @@
         <v>73</v>
       </c>
       <c r="B74" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C74" s="20" t="s">
+        <v>284</v>
+      </c>
+      <c r="D74" s="20" t="s">
         <v>285</v>
       </c>
-      <c r="D74" s="20" t="s">
+      <c r="E74" s="21" t="s">
         <v>286</v>
-      </c>
-      <c r="E74" s="21" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="75" spans="1:5">
@@ -3739,16 +3736,16 @@
         <v>74</v>
       </c>
       <c r="B75" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C75" s="20" t="s">
+        <v>287</v>
+      </c>
+      <c r="D75" s="22" t="s">
+        <v>115</v>
+      </c>
+      <c r="E75" s="22" t="s">
         <v>288</v>
-      </c>
-      <c r="D75" s="22" t="s">
-        <v>116</v>
-      </c>
-      <c r="E75" s="22" t="s">
-        <v>289</v>
       </c>
     </row>
     <row r="76" spans="1:5">
@@ -3756,16 +3753,16 @@
         <v>75</v>
       </c>
       <c r="B76" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C76" s="20" t="s">
+        <v>289</v>
+      </c>
+      <c r="D76" s="22" t="s">
         <v>290</v>
       </c>
-      <c r="D76" s="22" t="s">
+      <c r="E76" s="22" t="s">
         <v>291</v>
-      </c>
-      <c r="E76" s="22" t="s">
-        <v>292</v>
       </c>
     </row>
     <row r="77" spans="1:5">
@@ -3773,16 +3770,16 @@
         <v>76</v>
       </c>
       <c r="B77" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C77" s="20" t="s">
+        <v>292</v>
+      </c>
+      <c r="D77" s="22" t="s">
         <v>293</v>
       </c>
-      <c r="D77" s="22" t="s">
+      <c r="E77" s="22" t="s">
         <v>294</v>
-      </c>
-      <c r="E77" s="22" t="s">
-        <v>295</v>
       </c>
     </row>
     <row r="78" spans="1:5">
@@ -3790,16 +3787,16 @@
         <v>77</v>
       </c>
       <c r="B78" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C78" s="20" t="s">
+        <v>295</v>
+      </c>
+      <c r="D78" s="22" t="s">
         <v>296</v>
       </c>
-      <c r="D78" s="22" t="s">
+      <c r="E78" s="22" t="s">
         <v>297</v>
-      </c>
-      <c r="E78" s="22" t="s">
-        <v>298</v>
       </c>
     </row>
     <row r="79" spans="1:5">
@@ -3807,16 +3804,16 @@
         <v>78</v>
       </c>
       <c r="B79" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C79" s="20" t="s">
+        <v>298</v>
+      </c>
+      <c r="D79" s="20" t="s">
+        <v>276</v>
+      </c>
+      <c r="E79" s="21" t="s">
         <v>299</v>
-      </c>
-      <c r="D79" s="20" t="s">
-        <v>277</v>
-      </c>
-      <c r="E79" s="21" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="80" spans="1:5">
@@ -3824,16 +3821,16 @@
         <v>79</v>
       </c>
       <c r="B80" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C80" s="20" t="s">
+        <v>300</v>
+      </c>
+      <c r="D80" s="22" t="s">
         <v>301</v>
       </c>
-      <c r="D80" s="22" t="s">
+      <c r="E80" s="22" t="s">
         <v>302</v>
-      </c>
-      <c r="E80" s="22" t="s">
-        <v>303</v>
       </c>
     </row>
     <row r="81" spans="1:5">
@@ -3841,16 +3838,16 @@
         <v>80</v>
       </c>
       <c r="B81" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C81" s="20" t="s">
+        <v>303</v>
+      </c>
+      <c r="D81" s="20" t="s">
         <v>304</v>
       </c>
-      <c r="D81" s="20" t="s">
+      <c r="E81" s="21" t="s">
         <v>305</v>
-      </c>
-      <c r="E81" s="21" t="s">
-        <v>306</v>
       </c>
     </row>
     <row r="82" spans="1:5">
@@ -3858,16 +3855,16 @@
         <v>81</v>
       </c>
       <c r="B82" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C82" s="20" t="s">
+        <v>306</v>
+      </c>
+      <c r="D82" s="20" t="s">
         <v>307</v>
       </c>
-      <c r="D82" s="20" t="s">
+      <c r="E82" s="21" t="s">
         <v>308</v>
-      </c>
-      <c r="E82" s="21" t="s">
-        <v>309</v>
       </c>
     </row>
     <row r="83" spans="1:5">
@@ -3875,16 +3872,16 @@
         <v>82</v>
       </c>
       <c r="B83" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C83" s="20" t="s">
+        <v>309</v>
+      </c>
+      <c r="D83" s="20" t="s">
         <v>310</v>
       </c>
-      <c r="D83" s="20" t="s">
+      <c r="E83" s="21" t="s">
         <v>311</v>
-      </c>
-      <c r="E83" s="21" t="s">
-        <v>312</v>
       </c>
     </row>
     <row r="84" spans="1:5">
@@ -3892,16 +3889,16 @@
         <v>83</v>
       </c>
       <c r="B84" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C84" s="20" t="s">
+        <v>312</v>
+      </c>
+      <c r="D84" s="20" t="s">
         <v>313</v>
       </c>
-      <c r="D84" s="20" t="s">
-        <v>314</v>
-      </c>
       <c r="E84" s="21" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="85" spans="1:5">
@@ -3909,16 +3906,16 @@
         <v>84</v>
       </c>
       <c r="B85" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C85" s="20" t="s">
+        <v>314</v>
+      </c>
+      <c r="D85" s="20" t="s">
         <v>315</v>
       </c>
-      <c r="D85" s="20" t="s">
+      <c r="E85" s="21" t="s">
         <v>316</v>
-      </c>
-      <c r="E85" s="21" t="s">
-        <v>317</v>
       </c>
     </row>
     <row r="86" spans="1:5">
@@ -3926,16 +3923,16 @@
         <v>85</v>
       </c>
       <c r="B86" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C86" s="20" t="s">
+        <v>317</v>
+      </c>
+      <c r="D86" s="20" t="s">
+        <v>304</v>
+      </c>
+      <c r="E86" s="21" t="s">
         <v>318</v>
-      </c>
-      <c r="D86" s="20" t="s">
-        <v>305</v>
-      </c>
-      <c r="E86" s="21" t="s">
-        <v>319</v>
       </c>
     </row>
     <row r="87" spans="1:5">
@@ -3943,16 +3940,16 @@
         <v>86</v>
       </c>
       <c r="B87" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C87" s="20" t="s">
+        <v>319</v>
+      </c>
+      <c r="D87" s="20" t="s">
         <v>320</v>
       </c>
-      <c r="D87" s="20" t="s">
+      <c r="E87" s="21" t="s">
         <v>321</v>
-      </c>
-      <c r="E87" s="21" t="s">
-        <v>322</v>
       </c>
     </row>
     <row r="88" spans="1:5">
@@ -3960,16 +3957,16 @@
         <v>87</v>
       </c>
       <c r="B88" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C88" s="20" t="s">
+        <v>322</v>
+      </c>
+      <c r="D88" s="20" t="s">
+        <v>307</v>
+      </c>
+      <c r="E88" s="21" t="s">
         <v>323</v>
-      </c>
-      <c r="D88" s="20" t="s">
-        <v>308</v>
-      </c>
-      <c r="E88" s="21" t="s">
-        <v>324</v>
       </c>
     </row>
     <row r="89" spans="1:5">
@@ -3977,16 +3974,16 @@
         <v>88</v>
       </c>
       <c r="B89" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C89" s="20" t="s">
+        <v>324</v>
+      </c>
+      <c r="D89" s="20" t="s">
+        <v>100</v>
+      </c>
+      <c r="E89" s="21" t="s">
         <v>325</v>
-      </c>
-      <c r="D89" s="20" t="s">
-        <v>101</v>
-      </c>
-      <c r="E89" s="21" t="s">
-        <v>326</v>
       </c>
     </row>
     <row r="90" spans="1:5">
@@ -3994,16 +3991,16 @@
         <v>89</v>
       </c>
       <c r="B90" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C90" s="20" t="s">
+        <v>326</v>
+      </c>
+      <c r="D90" s="20" t="s">
         <v>327</v>
       </c>
-      <c r="D90" s="20" t="s">
+      <c r="E90" s="21" t="s">
         <v>328</v>
-      </c>
-      <c r="E90" s="21" t="s">
-        <v>329</v>
       </c>
     </row>
     <row r="91" spans="1:5">
@@ -4011,16 +4008,16 @@
         <v>90</v>
       </c>
       <c r="B91" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C91" s="20" t="s">
+        <v>329</v>
+      </c>
+      <c r="D91" s="20" t="s">
         <v>330</v>
       </c>
-      <c r="D91" s="20" t="s">
+      <c r="E91" s="21" t="s">
         <v>331</v>
-      </c>
-      <c r="E91" s="21" t="s">
-        <v>332</v>
       </c>
     </row>
     <row r="92" spans="1:5">
@@ -4028,16 +4025,16 @@
         <v>91</v>
       </c>
       <c r="B92" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C92" s="20" t="s">
+        <v>332</v>
+      </c>
+      <c r="D92" s="20" t="s">
         <v>333</v>
       </c>
-      <c r="D92" s="20" t="s">
+      <c r="E92" s="21" t="s">
         <v>334</v>
-      </c>
-      <c r="E92" s="21" t="s">
-        <v>335</v>
       </c>
     </row>
     <row r="93" spans="1:5">
@@ -4045,16 +4042,16 @@
         <v>92</v>
       </c>
       <c r="B93" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C93" s="20" t="s">
+        <v>335</v>
+      </c>
+      <c r="D93" s="20" t="s">
+        <v>192</v>
+      </c>
+      <c r="E93" s="21" t="s">
         <v>336</v>
-      </c>
-      <c r="D93" s="20" t="s">
-        <v>193</v>
-      </c>
-      <c r="E93" s="21" t="s">
-        <v>337</v>
       </c>
     </row>
     <row r="94" spans="1:5">
@@ -4062,16 +4059,16 @@
         <v>93</v>
       </c>
       <c r="B94" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C94" s="20" t="s">
+        <v>337</v>
+      </c>
+      <c r="D94" s="22" t="s">
         <v>338</v>
       </c>
-      <c r="D94" s="22" t="s">
+      <c r="E94" s="22" t="s">
         <v>339</v>
-      </c>
-      <c r="E94" s="22" t="s">
-        <v>340</v>
       </c>
     </row>
     <row r="95" spans="1:5">
@@ -4079,16 +4076,16 @@
         <v>94</v>
       </c>
       <c r="B95" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C95" s="29" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="D95" s="27" t="s">
+        <v>354</v>
+      </c>
+      <c r="E95" s="27" t="s">
         <v>355</v>
-      </c>
-      <c r="E95" s="27" t="s">
-        <v>356</v>
       </c>
     </row>
     <row r="96" spans="1:5">
@@ -4097,16 +4094,16 @@
         <v>95</v>
       </c>
       <c r="B96" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C96" s="30" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="D96" s="31" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E96" s="31" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="97" spans="1:5">
@@ -4115,16 +4112,16 @@
         <v>96</v>
       </c>
       <c r="B97" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C97" s="26" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="D97" s="27" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E97" s="27" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="98" spans="1:5">
@@ -4133,16 +4130,16 @@
         <v>97</v>
       </c>
       <c r="B98" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C98" s="26" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="D98" s="27" t="s">
+        <v>347</v>
+      </c>
+      <c r="E98" s="27" t="s">
         <v>348</v>
-      </c>
-      <c r="E98" s="27" t="s">
-        <v>349</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
publica cambios de calendario 2026-05-26 22:02
</commit_message>
<xml_diff>
--- a/Template_Calendario_CCS_GPX.xlsx
+++ b/Template_Calendario_CCS_GPX.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cesarmora/Library/Mobile Documents/com~apple~CloudDocs/Personal/Ciclismo/Calendario/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{647B7200-F0ED-7F4F-9CA4-DCD88671F4CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3AB4338-7F25-EE41-BC68-1AC1B9534735}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12200" yWindow="780" windowWidth="20720" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12200" yWindow="780" windowWidth="20720" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template_Calendario_CCS" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="358">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="359">
   <si>
     <t>Fecha</t>
   </si>
@@ -489,9 +489,6 @@
     <t>Delporte</t>
   </si>
   <si>
-    <t>15720618-4</t>
-  </si>
-  <si>
     <t>José Ignacio</t>
   </si>
   <si>
@@ -555,27 +552,18 @@
     <t>7.546.124-0</t>
   </si>
   <si>
-    <t>25293314-k</t>
-  </si>
-  <si>
     <t>Oriana</t>
   </si>
   <si>
     <t>Gonzalez</t>
   </si>
   <si>
-    <t>13209775-5</t>
-  </si>
-  <si>
     <t>Mario</t>
   </si>
   <si>
     <t>González</t>
   </si>
   <si>
-    <t>7840203-2</t>
-  </si>
-  <si>
     <t xml:space="preserve">Pablo  </t>
   </si>
   <si>
@@ -591,18 +579,12 @@
     <t>Henriquez</t>
   </si>
   <si>
-    <t>15959545-5</t>
-  </si>
-  <si>
     <t>Felipe Ignacio</t>
   </si>
   <si>
     <t>Hernández</t>
   </si>
   <si>
-    <t>11741692-5</t>
-  </si>
-  <si>
     <t>Nolly</t>
   </si>
   <si>
@@ -642,9 +624,6 @@
     <t>Jiménez</t>
   </si>
   <si>
-    <t>8546622-4</t>
-  </si>
-  <si>
     <t>Eduardo</t>
   </si>
   <si>
@@ -660,15 +639,9 @@
     <t>kopplin</t>
   </si>
   <si>
-    <t>14148513-k</t>
-  </si>
-  <si>
     <t>Lalanne</t>
   </si>
   <si>
-    <t>11648183-9</t>
-  </si>
-  <si>
     <t>Francisca</t>
   </si>
   <si>
@@ -684,9 +657,6 @@
     <t>Leon</t>
   </si>
   <si>
-    <t>10522681-0</t>
-  </si>
-  <si>
     <t>Leria</t>
   </si>
   <si>
@@ -696,18 +666,12 @@
     <t>Leturia</t>
   </si>
   <si>
-    <t>16126127-0</t>
-  </si>
-  <si>
     <t xml:space="preserve">Alvaro </t>
   </si>
   <si>
     <t>López</t>
   </si>
   <si>
-    <t>8459653-1</t>
-  </si>
-  <si>
     <t xml:space="preserve">Ricardo </t>
   </si>
   <si>
@@ -720,18 +684,12 @@
     <t>Lyon</t>
   </si>
   <si>
-    <t>7212090-0</t>
-  </si>
-  <si>
     <t xml:space="preserve">Tomás </t>
   </si>
   <si>
     <t>Magallon</t>
   </si>
   <si>
-    <t>8713352-4</t>
-  </si>
-  <si>
     <t xml:space="preserve">Paolo </t>
   </si>
   <si>
@@ -756,9 +714,6 @@
     <t>Martínez</t>
   </si>
   <si>
-    <t>10548107-1</t>
-  </si>
-  <si>
     <t xml:space="preserve">Marcela </t>
   </si>
   <si>
@@ -780,24 +735,15 @@
     <t>Moller</t>
   </si>
   <si>
-    <t>7109273-9</t>
-  </si>
-  <si>
     <t xml:space="preserve">Ivana </t>
   </si>
   <si>
     <t>Morello</t>
   </si>
   <si>
-    <t>11836707-3</t>
-  </si>
-  <si>
     <t>Moreno</t>
   </si>
   <si>
-    <t>12928471-4</t>
-  </si>
-  <si>
     <t>Fernanda</t>
   </si>
   <si>
@@ -813,9 +759,6 @@
     <t>Munita</t>
   </si>
   <si>
-    <t>9976077-K</t>
-  </si>
-  <si>
     <t>Musalem</t>
   </si>
   <si>
@@ -834,18 +777,12 @@
     <t>Novoa</t>
   </si>
   <si>
-    <t>7250144-6</t>
-  </si>
-  <si>
     <t xml:space="preserve">Carlos </t>
   </si>
   <si>
     <t>Obaid</t>
   </si>
   <si>
-    <t>15661137-9</t>
-  </si>
-  <si>
     <t xml:space="preserve">Daniel </t>
   </si>
   <si>
@@ -879,9 +816,6 @@
     <t xml:space="preserve">Quevedo </t>
   </si>
   <si>
-    <t>7194204-K</t>
-  </si>
-  <si>
     <t xml:space="preserve">Karín </t>
   </si>
   <si>
@@ -945,18 +879,12 @@
     <t>Silva</t>
   </si>
   <si>
-    <t>23267753-8</t>
-  </si>
-  <si>
     <t>Pablo</t>
   </si>
   <si>
     <t>Soffiato</t>
   </si>
   <si>
-    <t>6902317-7</t>
-  </si>
-  <si>
     <t xml:space="preserve">Richard </t>
   </si>
   <si>
@@ -972,9 +900,6 @@
     <t>Torres</t>
   </si>
   <si>
-    <t>11391042-9</t>
-  </si>
-  <si>
     <t xml:space="preserve">Pedro Pablo </t>
   </si>
   <si>
@@ -1089,15 +1014,6 @@
     <t>10.160.334-2</t>
   </si>
   <si>
-    <t>8327118-3</t>
-  </si>
-  <si>
-    <t>12239638-K</t>
-  </si>
-  <si>
-    <t>27150755-0</t>
-  </si>
-  <si>
     <t>Álvaro</t>
   </si>
   <si>
@@ -1108,6 +1024,93 @@
   </si>
   <si>
     <t>Guajardo</t>
+  </si>
+  <si>
+    <t>13.240.303-1</t>
+  </si>
+  <si>
+    <t>7.212.090-0</t>
+  </si>
+  <si>
+    <t>8.546.622-4</t>
+  </si>
+  <si>
+    <t>14.148.513-k</t>
+  </si>
+  <si>
+    <t>11.741.692-5</t>
+  </si>
+  <si>
+    <t>15.720.618-4</t>
+  </si>
+  <si>
+    <t>25.293.314-k</t>
+  </si>
+  <si>
+    <t>13.209.775-5</t>
+  </si>
+  <si>
+    <t>7.840.203-2</t>
+  </si>
+  <si>
+    <t>15.959.545-5</t>
+  </si>
+  <si>
+    <t>11.648.183-9</t>
+  </si>
+  <si>
+    <t>10.522.681-0</t>
+  </si>
+  <si>
+    <t>16.126.127-0</t>
+  </si>
+  <si>
+    <t>8.459.653-1</t>
+  </si>
+  <si>
+    <t>8.713.352-4</t>
+  </si>
+  <si>
+    <t>10.548.107-1</t>
+  </si>
+  <si>
+    <t>7.109.273-9</t>
+  </si>
+  <si>
+    <t>11.836.707-3</t>
+  </si>
+  <si>
+    <t>12.928.471-4</t>
+  </si>
+  <si>
+    <t>9.976.077-K</t>
+  </si>
+  <si>
+    <t>7.250.144-6</t>
+  </si>
+  <si>
+    <t>15.661.137-9</t>
+  </si>
+  <si>
+    <t>7.194.204-K</t>
+  </si>
+  <si>
+    <t>23.267.753-8</t>
+  </si>
+  <si>
+    <t>6.902.317-7</t>
+  </si>
+  <si>
+    <t>11.391.042-9</t>
+  </si>
+  <si>
+    <t>8.327.118-3</t>
+  </si>
+  <si>
+    <t>12.239.638-K</t>
+  </si>
+  <si>
+    <t>27.150.755-0</t>
   </si>
 </sst>
 </file>
@@ -1826,10 +1829,10 @@
         <v>7</v>
       </c>
       <c r="C10" t="s">
-        <v>340</v>
+        <v>315</v>
       </c>
       <c r="D10" t="s">
-        <v>340</v>
+        <v>315</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>40</v>
@@ -1846,10 +1849,10 @@
         <v>7</v>
       </c>
       <c r="C11" t="s">
-        <v>340</v>
+        <v>315</v>
       </c>
       <c r="D11" t="s">
-        <v>340</v>
+        <v>315</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>40</v>
@@ -1906,7 +1909,7 @@
         <v>6</v>
       </c>
       <c r="C14" t="s">
-        <v>341</v>
+        <v>316</v>
       </c>
       <c r="D14" t="s">
         <v>34</v>
@@ -2026,7 +2029,7 @@
         <v>6</v>
       </c>
       <c r="C20" t="s">
-        <v>342</v>
+        <v>317</v>
       </c>
       <c r="D20" t="s">
         <v>29</v>
@@ -2035,7 +2038,7 @@
         <v>40</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>343</v>
+        <v>318</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -2126,16 +2129,16 @@
         <v>6</v>
       </c>
       <c r="C25" t="s">
-        <v>344</v>
+        <v>319</v>
       </c>
       <c r="D25" t="s">
-        <v>346</v>
+        <v>321</v>
       </c>
       <c r="E25" s="10" t="s">
         <v>40</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>345</v>
+        <v>320</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -2906,13 +2909,13 @@
         <v>80</v>
       </c>
       <c r="C26" s="20" t="s">
+        <v>335</v>
+      </c>
+      <c r="D26" s="22" t="s">
         <v>151</v>
       </c>
-      <c r="D26" s="22" t="s">
+      <c r="E26" s="22" t="s">
         <v>152</v>
-      </c>
-      <c r="E26" s="22" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -2923,13 +2926,13 @@
         <v>80</v>
       </c>
       <c r="C27" s="20" t="s">
+        <v>153</v>
+      </c>
+      <c r="D27" s="20" t="s">
         <v>154</v>
       </c>
-      <c r="D27" s="20" t="s">
+      <c r="E27" s="21" t="s">
         <v>155</v>
-      </c>
-      <c r="E27" s="21" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -2940,13 +2943,13 @@
         <v>80</v>
       </c>
       <c r="C28" s="20" t="s">
+        <v>156</v>
+      </c>
+      <c r="D28" s="20" t="s">
         <v>157</v>
       </c>
-      <c r="D28" s="20" t="s">
+      <c r="E28" s="21" t="s">
         <v>158</v>
-      </c>
-      <c r="E28" s="21" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -2957,13 +2960,13 @@
         <v>80</v>
       </c>
       <c r="C29" s="20" t="s">
+        <v>159</v>
+      </c>
+      <c r="D29" s="20" t="s">
         <v>160</v>
       </c>
-      <c r="D29" s="20" t="s">
+      <c r="E29" s="21" t="s">
         <v>161</v>
-      </c>
-      <c r="E29" s="21" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="30" spans="1:5">
@@ -2974,13 +2977,13 @@
         <v>80</v>
       </c>
       <c r="C30" s="20" t="s">
+        <v>162</v>
+      </c>
+      <c r="D30" s="22" t="s">
         <v>163</v>
       </c>
-      <c r="D30" s="22" t="s">
+      <c r="E30" s="22" t="s">
         <v>164</v>
-      </c>
-      <c r="E30" s="22" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="31" spans="1:5">
@@ -2991,13 +2994,13 @@
         <v>80</v>
       </c>
       <c r="C31" s="20" t="s">
+        <v>165</v>
+      </c>
+      <c r="D31" s="20" t="s">
         <v>166</v>
       </c>
-      <c r="D31" s="20" t="s">
+      <c r="E31" s="21" t="s">
         <v>167</v>
-      </c>
-      <c r="E31" s="21" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="32" spans="1:5">
@@ -3008,13 +3011,13 @@
         <v>80</v>
       </c>
       <c r="C32" s="20" t="s">
+        <v>168</v>
+      </c>
+      <c r="D32" s="20" t="s">
         <v>169</v>
       </c>
-      <c r="D32" s="20" t="s">
+      <c r="E32" s="21" t="s">
         <v>170</v>
-      </c>
-      <c r="E32" s="21" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="33" spans="1:5">
@@ -3025,13 +3028,13 @@
         <v>80</v>
       </c>
       <c r="C33" s="20" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D33" s="20" t="s">
         <v>143</v>
       </c>
       <c r="E33" s="21" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="34" spans="1:5">
@@ -3042,13 +3045,13 @@
         <v>80</v>
       </c>
       <c r="C34" s="20" t="s">
+        <v>336</v>
+      </c>
+      <c r="D34" s="20" t="s">
+        <v>172</v>
+      </c>
+      <c r="E34" s="21" t="s">
         <v>173</v>
-      </c>
-      <c r="D34" s="20" t="s">
-        <v>174</v>
-      </c>
-      <c r="E34" s="21" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="35" spans="1:5">
@@ -3059,13 +3062,13 @@
         <v>80</v>
       </c>
       <c r="C35" s="20" t="s">
-        <v>176</v>
+        <v>337</v>
       </c>
       <c r="D35" s="20" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="E35" s="21" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="36" spans="1:5">
@@ -3076,13 +3079,13 @@
         <v>80</v>
       </c>
       <c r="C36" s="20" t="s">
-        <v>179</v>
+        <v>338</v>
       </c>
       <c r="D36" s="20" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="E36" s="21" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
     </row>
     <row r="37" spans="1:5">
@@ -3093,13 +3096,13 @@
         <v>80</v>
       </c>
       <c r="C37" s="20" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D37" s="20" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="E37" s="21" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
     </row>
     <row r="38" spans="1:5">
@@ -3110,13 +3113,13 @@
         <v>80</v>
       </c>
       <c r="C38" s="20" t="s">
-        <v>185</v>
+        <v>339</v>
       </c>
       <c r="D38" s="20" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="E38" s="21" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
     </row>
     <row r="39" spans="1:5">
@@ -3127,13 +3130,13 @@
         <v>80</v>
       </c>
       <c r="C39" s="20" t="s">
-        <v>188</v>
+        <v>334</v>
       </c>
       <c r="D39" s="20" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="E39" s="21" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
     </row>
     <row r="40" spans="1:5">
@@ -3144,13 +3147,13 @@
         <v>80</v>
       </c>
       <c r="C40" s="20" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="D40" s="20" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="E40" s="21" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
     </row>
     <row r="41" spans="1:5">
@@ -3161,13 +3164,13 @@
         <v>80</v>
       </c>
       <c r="C41" s="24" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="D41" s="20" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="E41" s="21" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
     </row>
     <row r="42" spans="1:5">
@@ -3178,13 +3181,13 @@
         <v>80</v>
       </c>
       <c r="C42" s="20" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="D42" s="22" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="E42" s="22" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
     </row>
     <row r="43" spans="1:5">
@@ -3195,13 +3198,13 @@
         <v>80</v>
       </c>
       <c r="C43" s="20" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="D43" s="22" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="E43" s="22" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="44" spans="1:5">
@@ -3212,13 +3215,13 @@
         <v>80</v>
       </c>
       <c r="C44" s="20" t="s">
-        <v>202</v>
+        <v>332</v>
       </c>
       <c r="D44" s="20" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="E44" s="21" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
     </row>
     <row r="45" spans="1:5">
@@ -3229,13 +3232,13 @@
         <v>80</v>
       </c>
       <c r="C45" s="20" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="D45" s="22" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="E45" s="22" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
     </row>
     <row r="46" spans="1:5">
@@ -3246,13 +3249,13 @@
         <v>80</v>
       </c>
       <c r="C46" s="23" t="s">
-        <v>208</v>
+        <v>333</v>
       </c>
       <c r="D46" s="20" t="s">
         <v>134</v>
       </c>
       <c r="E46" s="21" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
     </row>
     <row r="47" spans="1:5">
@@ -3263,13 +3266,13 @@
         <v>80</v>
       </c>
       <c r="C47" s="20" t="s">
-        <v>210</v>
+        <v>340</v>
       </c>
       <c r="D47" s="20" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="E47" s="21" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
     </row>
     <row r="48" spans="1:5">
@@ -3280,13 +3283,13 @@
         <v>80</v>
       </c>
       <c r="C48" s="20" t="s">
-        <v>213</v>
+        <v>204</v>
       </c>
       <c r="D48" s="20" t="s">
-        <v>214</v>
+        <v>205</v>
       </c>
       <c r="E48" s="21" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
     </row>
     <row r="49" spans="1:5">
@@ -3297,13 +3300,13 @@
         <v>80</v>
       </c>
       <c r="C49" s="20" t="s">
-        <v>216</v>
+        <v>341</v>
       </c>
       <c r="D49" s="20" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E49" s="21" t="s">
-        <v>217</v>
+        <v>207</v>
       </c>
     </row>
     <row r="50" spans="1:5">
@@ -3314,13 +3317,13 @@
         <v>80</v>
       </c>
       <c r="C50" s="20" t="s">
-        <v>218</v>
+        <v>208</v>
       </c>
       <c r="D50" s="22" t="s">
         <v>100</v>
       </c>
       <c r="E50" s="22" t="s">
-        <v>219</v>
+        <v>209</v>
       </c>
     </row>
     <row r="51" spans="1:5">
@@ -3331,13 +3334,13 @@
         <v>80</v>
       </c>
       <c r="C51" s="20" t="s">
-        <v>220</v>
+        <v>342</v>
       </c>
       <c r="D51" s="20" t="s">
-        <v>221</v>
+        <v>210</v>
       </c>
       <c r="E51" s="21" t="s">
-        <v>222</v>
+        <v>211</v>
       </c>
     </row>
     <row r="52" spans="1:5">
@@ -3348,13 +3351,13 @@
         <v>80</v>
       </c>
       <c r="C52" s="20" t="s">
-        <v>223</v>
+        <v>343</v>
       </c>
       <c r="D52" s="20" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="E52" s="21" t="s">
-        <v>222</v>
+        <v>211</v>
       </c>
     </row>
     <row r="53" spans="1:5">
@@ -3365,13 +3368,13 @@
         <v>80</v>
       </c>
       <c r="C53" s="20" t="s">
-        <v>225</v>
+        <v>213</v>
       </c>
       <c r="D53" s="20" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="E53" s="21" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
     </row>
     <row r="54" spans="1:5">
@@ -3382,13 +3385,13 @@
         <v>80</v>
       </c>
       <c r="C54" s="20" t="s">
-        <v>228</v>
+        <v>331</v>
       </c>
       <c r="D54" s="20" t="s">
-        <v>229</v>
+        <v>216</v>
       </c>
       <c r="E54" s="21" t="s">
-        <v>230</v>
+        <v>217</v>
       </c>
     </row>
     <row r="55" spans="1:5">
@@ -3399,13 +3402,13 @@
         <v>80</v>
       </c>
       <c r="C55" s="20" t="s">
-        <v>231</v>
+        <v>344</v>
       </c>
       <c r="D55" s="20" t="s">
-        <v>232</v>
+        <v>218</v>
       </c>
       <c r="E55" s="21" t="s">
-        <v>233</v>
+        <v>219</v>
       </c>
     </row>
     <row r="56" spans="1:5">
@@ -3416,13 +3419,13 @@
         <v>80</v>
       </c>
       <c r="C56" s="20" t="s">
-        <v>234</v>
+        <v>220</v>
       </c>
       <c r="D56" s="22" t="s">
-        <v>235</v>
+        <v>221</v>
       </c>
       <c r="E56" s="22" t="s">
-        <v>236</v>
+        <v>222</v>
       </c>
     </row>
     <row r="57" spans="1:5">
@@ -3433,13 +3436,13 @@
         <v>80</v>
       </c>
       <c r="C57" s="20" t="s">
-        <v>237</v>
+        <v>223</v>
       </c>
       <c r="D57" s="22" t="s">
-        <v>238</v>
+        <v>224</v>
       </c>
       <c r="E57" s="22" t="s">
-        <v>239</v>
+        <v>225</v>
       </c>
     </row>
     <row r="58" spans="1:5">
@@ -3450,13 +3453,13 @@
         <v>80</v>
       </c>
       <c r="C58" s="20" t="s">
-        <v>240</v>
+        <v>345</v>
       </c>
       <c r="D58" s="20" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="E58" s="21" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
     </row>
     <row r="59" spans="1:5">
@@ -3467,13 +3470,13 @@
         <v>80</v>
       </c>
       <c r="C59" s="20" t="s">
-        <v>349</v>
+        <v>324</v>
       </c>
       <c r="D59" s="22" t="s">
-        <v>243</v>
+        <v>228</v>
       </c>
       <c r="E59" s="22" t="s">
-        <v>244</v>
+        <v>229</v>
       </c>
     </row>
     <row r="60" spans="1:5">
@@ -3484,13 +3487,13 @@
         <v>80</v>
       </c>
       <c r="C60" s="20" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="D60" s="20" t="s">
-        <v>246</v>
+        <v>231</v>
       </c>
       <c r="E60" s="21" t="s">
-        <v>247</v>
+        <v>232</v>
       </c>
     </row>
     <row r="61" spans="1:5">
@@ -3501,13 +3504,13 @@
         <v>80</v>
       </c>
       <c r="C61" s="20" t="s">
-        <v>248</v>
+        <v>346</v>
       </c>
       <c r="D61" s="20" t="s">
-        <v>249</v>
+        <v>233</v>
       </c>
       <c r="E61" s="21" t="s">
-        <v>250</v>
+        <v>234</v>
       </c>
     </row>
     <row r="62" spans="1:5">
@@ -3518,13 +3521,13 @@
         <v>80</v>
       </c>
       <c r="C62" s="20" t="s">
-        <v>251</v>
+        <v>347</v>
       </c>
       <c r="D62" s="20" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="E62" s="21" t="s">
-        <v>252</v>
+        <v>235</v>
       </c>
     </row>
     <row r="63" spans="1:5">
@@ -3535,13 +3538,13 @@
         <v>80</v>
       </c>
       <c r="C63" s="20" t="s">
-        <v>253</v>
+        <v>348</v>
       </c>
       <c r="D63" s="20" t="s">
-        <v>254</v>
+        <v>236</v>
       </c>
       <c r="E63" s="21" t="s">
-        <v>255</v>
+        <v>237</v>
       </c>
     </row>
     <row r="64" spans="1:5">
@@ -3552,13 +3555,13 @@
         <v>80</v>
       </c>
       <c r="C64" s="20" t="s">
-        <v>256</v>
+        <v>238</v>
       </c>
       <c r="D64" s="20" t="s">
-        <v>257</v>
+        <v>239</v>
       </c>
       <c r="E64" s="21" t="s">
-        <v>258</v>
+        <v>240</v>
       </c>
     </row>
     <row r="65" spans="1:5">
@@ -3569,13 +3572,13 @@
         <v>80</v>
       </c>
       <c r="C65" s="20" t="s">
-        <v>259</v>
+        <v>349</v>
       </c>
       <c r="D65" s="20" t="s">
         <v>85</v>
       </c>
       <c r="E65" s="21" t="s">
-        <v>260</v>
+        <v>241</v>
       </c>
     </row>
     <row r="66" spans="1:5">
@@ -3585,14 +3588,14 @@
       <c r="B66" s="19" t="s">
         <v>80</v>
       </c>
-      <c r="C66" s="20">
-        <v>132403031</v>
+      <c r="C66" s="20" t="s">
+        <v>330</v>
       </c>
       <c r="D66" s="20" t="s">
-        <v>261</v>
+        <v>242</v>
       </c>
       <c r="E66" s="21" t="s">
-        <v>262</v>
+        <v>243</v>
       </c>
     </row>
     <row r="67" spans="1:5">
@@ -3603,13 +3606,13 @@
         <v>80</v>
       </c>
       <c r="C67" s="20" t="s">
-        <v>263</v>
+        <v>244</v>
       </c>
       <c r="D67" s="20" t="s">
-        <v>264</v>
+        <v>245</v>
       </c>
       <c r="E67" s="21" t="s">
-        <v>265</v>
+        <v>246</v>
       </c>
     </row>
     <row r="68" spans="1:5">
@@ -3620,13 +3623,13 @@
         <v>80</v>
       </c>
       <c r="C68" s="20" t="s">
-        <v>266</v>
+        <v>350</v>
       </c>
       <c r="D68" s="20" t="s">
-        <v>267</v>
+        <v>247</v>
       </c>
       <c r="E68" s="21" t="s">
-        <v>268</v>
+        <v>248</v>
       </c>
     </row>
     <row r="69" spans="1:5">
@@ -3637,13 +3640,13 @@
         <v>80</v>
       </c>
       <c r="C69" s="20" t="s">
-        <v>269</v>
+        <v>351</v>
       </c>
       <c r="D69" s="20" t="s">
-        <v>270</v>
+        <v>249</v>
       </c>
       <c r="E69" s="21" t="s">
-        <v>271</v>
+        <v>250</v>
       </c>
     </row>
     <row r="70" spans="1:5">
@@ -3654,13 +3657,13 @@
         <v>80</v>
       </c>
       <c r="C70" s="20" t="s">
-        <v>272</v>
+        <v>251</v>
       </c>
       <c r="D70" s="22" t="s">
-        <v>273</v>
+        <v>252</v>
       </c>
       <c r="E70" s="22" t="s">
-        <v>274</v>
+        <v>253</v>
       </c>
     </row>
     <row r="71" spans="1:5">
@@ -3671,13 +3674,13 @@
         <v>80</v>
       </c>
       <c r="C71" s="20" t="s">
-        <v>275</v>
+        <v>254</v>
       </c>
       <c r="D71" s="20" t="s">
-        <v>276</v>
+        <v>255</v>
       </c>
       <c r="E71" s="21" t="s">
-        <v>277</v>
+        <v>256</v>
       </c>
     </row>
     <row r="72" spans="1:5">
@@ -3688,13 +3691,13 @@
         <v>80</v>
       </c>
       <c r="C72" s="20" t="s">
-        <v>278</v>
+        <v>257</v>
       </c>
       <c r="D72" s="22" t="s">
-        <v>279</v>
+        <v>258</v>
       </c>
       <c r="E72" s="22" t="s">
-        <v>280</v>
+        <v>259</v>
       </c>
     </row>
     <row r="73" spans="1:5">
@@ -3705,13 +3708,13 @@
         <v>80</v>
       </c>
       <c r="C73" s="20" t="s">
-        <v>281</v>
+        <v>352</v>
       </c>
       <c r="D73" s="20" t="s">
-        <v>282</v>
+        <v>260</v>
       </c>
       <c r="E73" s="21" t="s">
-        <v>283</v>
+        <v>261</v>
       </c>
     </row>
     <row r="74" spans="1:5">
@@ -3722,13 +3725,13 @@
         <v>80</v>
       </c>
       <c r="C74" s="20" t="s">
-        <v>284</v>
+        <v>262</v>
       </c>
       <c r="D74" s="20" t="s">
-        <v>285</v>
+        <v>263</v>
       </c>
       <c r="E74" s="21" t="s">
-        <v>286</v>
+        <v>264</v>
       </c>
     </row>
     <row r="75" spans="1:5">
@@ -3739,13 +3742,13 @@
         <v>80</v>
       </c>
       <c r="C75" s="20" t="s">
-        <v>287</v>
+        <v>265</v>
       </c>
       <c r="D75" s="22" t="s">
         <v>115</v>
       </c>
       <c r="E75" s="22" t="s">
-        <v>288</v>
+        <v>266</v>
       </c>
     </row>
     <row r="76" spans="1:5">
@@ -3756,13 +3759,13 @@
         <v>80</v>
       </c>
       <c r="C76" s="20" t="s">
-        <v>289</v>
+        <v>267</v>
       </c>
       <c r="D76" s="22" t="s">
-        <v>290</v>
+        <v>268</v>
       </c>
       <c r="E76" s="22" t="s">
-        <v>291</v>
+        <v>269</v>
       </c>
     </row>
     <row r="77" spans="1:5">
@@ -3773,13 +3776,13 @@
         <v>80</v>
       </c>
       <c r="C77" s="20" t="s">
-        <v>292</v>
+        <v>270</v>
       </c>
       <c r="D77" s="22" t="s">
-        <v>293</v>
+        <v>271</v>
       </c>
       <c r="E77" s="22" t="s">
-        <v>294</v>
+        <v>272</v>
       </c>
     </row>
     <row r="78" spans="1:5">
@@ -3790,13 +3793,13 @@
         <v>80</v>
       </c>
       <c r="C78" s="20" t="s">
-        <v>295</v>
+        <v>273</v>
       </c>
       <c r="D78" s="22" t="s">
-        <v>296</v>
+        <v>274</v>
       </c>
       <c r="E78" s="22" t="s">
-        <v>297</v>
+        <v>275</v>
       </c>
     </row>
     <row r="79" spans="1:5">
@@ -3807,13 +3810,13 @@
         <v>80</v>
       </c>
       <c r="C79" s="20" t="s">
-        <v>298</v>
+        <v>276</v>
       </c>
       <c r="D79" s="20" t="s">
-        <v>276</v>
+        <v>255</v>
       </c>
       <c r="E79" s="21" t="s">
-        <v>299</v>
+        <v>277</v>
       </c>
     </row>
     <row r="80" spans="1:5">
@@ -3824,13 +3827,13 @@
         <v>80</v>
       </c>
       <c r="C80" s="20" t="s">
-        <v>300</v>
+        <v>278</v>
       </c>
       <c r="D80" s="22" t="s">
-        <v>301</v>
+        <v>279</v>
       </c>
       <c r="E80" s="22" t="s">
-        <v>302</v>
+        <v>280</v>
       </c>
     </row>
     <row r="81" spans="1:5">
@@ -3841,13 +3844,13 @@
         <v>80</v>
       </c>
       <c r="C81" s="20" t="s">
-        <v>303</v>
+        <v>353</v>
       </c>
       <c r="D81" s="20" t="s">
-        <v>304</v>
+        <v>281</v>
       </c>
       <c r="E81" s="21" t="s">
-        <v>305</v>
+        <v>282</v>
       </c>
     </row>
     <row r="82" spans="1:5">
@@ -3858,13 +3861,13 @@
         <v>80</v>
       </c>
       <c r="C82" s="20" t="s">
-        <v>306</v>
+        <v>354</v>
       </c>
       <c r="D82" s="20" t="s">
-        <v>307</v>
+        <v>283</v>
       </c>
       <c r="E82" s="21" t="s">
-        <v>308</v>
+        <v>284</v>
       </c>
     </row>
     <row r="83" spans="1:5">
@@ -3875,13 +3878,13 @@
         <v>80</v>
       </c>
       <c r="C83" s="20" t="s">
-        <v>309</v>
+        <v>285</v>
       </c>
       <c r="D83" s="20" t="s">
-        <v>310</v>
+        <v>286</v>
       </c>
       <c r="E83" s="21" t="s">
-        <v>311</v>
+        <v>287</v>
       </c>
     </row>
     <row r="84" spans="1:5">
@@ -3892,13 +3895,13 @@
         <v>80</v>
       </c>
       <c r="C84" s="20" t="s">
-        <v>312</v>
+        <v>355</v>
       </c>
       <c r="D84" s="20" t="s">
-        <v>313</v>
+        <v>288</v>
       </c>
       <c r="E84" s="21" t="s">
-        <v>311</v>
+        <v>287</v>
       </c>
     </row>
     <row r="85" spans="1:5">
@@ -3909,13 +3912,13 @@
         <v>80</v>
       </c>
       <c r="C85" s="20" t="s">
-        <v>314</v>
+        <v>289</v>
       </c>
       <c r="D85" s="20" t="s">
-        <v>315</v>
+        <v>290</v>
       </c>
       <c r="E85" s="21" t="s">
-        <v>316</v>
+        <v>291</v>
       </c>
     </row>
     <row r="86" spans="1:5">
@@ -3926,13 +3929,13 @@
         <v>80</v>
       </c>
       <c r="C86" s="20" t="s">
-        <v>317</v>
+        <v>292</v>
       </c>
       <c r="D86" s="20" t="s">
-        <v>304</v>
+        <v>281</v>
       </c>
       <c r="E86" s="21" t="s">
-        <v>318</v>
+        <v>293</v>
       </c>
     </row>
     <row r="87" spans="1:5">
@@ -3943,13 +3946,13 @@
         <v>80</v>
       </c>
       <c r="C87" s="20" t="s">
-        <v>319</v>
+        <v>294</v>
       </c>
       <c r="D87" s="20" t="s">
-        <v>320</v>
+        <v>295</v>
       </c>
       <c r="E87" s="21" t="s">
-        <v>321</v>
+        <v>296</v>
       </c>
     </row>
     <row r="88" spans="1:5">
@@ -3960,13 +3963,13 @@
         <v>80</v>
       </c>
       <c r="C88" s="20" t="s">
-        <v>322</v>
+        <v>297</v>
       </c>
       <c r="D88" s="20" t="s">
-        <v>307</v>
+        <v>283</v>
       </c>
       <c r="E88" s="21" t="s">
-        <v>323</v>
+        <v>298</v>
       </c>
     </row>
     <row r="89" spans="1:5">
@@ -3977,13 +3980,13 @@
         <v>80</v>
       </c>
       <c r="C89" s="20" t="s">
-        <v>324</v>
+        <v>299</v>
       </c>
       <c r="D89" s="20" t="s">
         <v>100</v>
       </c>
       <c r="E89" s="21" t="s">
-        <v>325</v>
+        <v>300</v>
       </c>
     </row>
     <row r="90" spans="1:5">
@@ -3994,13 +3997,13 @@
         <v>80</v>
       </c>
       <c r="C90" s="20" t="s">
-        <v>326</v>
+        <v>301</v>
       </c>
       <c r="D90" s="20" t="s">
-        <v>327</v>
+        <v>302</v>
       </c>
       <c r="E90" s="21" t="s">
-        <v>328</v>
+        <v>303</v>
       </c>
     </row>
     <row r="91" spans="1:5">
@@ -4011,13 +4014,13 @@
         <v>80</v>
       </c>
       <c r="C91" s="20" t="s">
-        <v>329</v>
+        <v>304</v>
       </c>
       <c r="D91" s="20" t="s">
-        <v>330</v>
+        <v>305</v>
       </c>
       <c r="E91" s="21" t="s">
-        <v>331</v>
+        <v>306</v>
       </c>
     </row>
     <row r="92" spans="1:5">
@@ -4028,13 +4031,13 @@
         <v>80</v>
       </c>
       <c r="C92" s="20" t="s">
-        <v>332</v>
+        <v>307</v>
       </c>
       <c r="D92" s="20" t="s">
-        <v>333</v>
+        <v>308</v>
       </c>
       <c r="E92" s="21" t="s">
-        <v>334</v>
+        <v>309</v>
       </c>
     </row>
     <row r="93" spans="1:5">
@@ -4045,13 +4048,13 @@
         <v>80</v>
       </c>
       <c r="C93" s="20" t="s">
-        <v>335</v>
+        <v>310</v>
       </c>
       <c r="D93" s="20" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="E93" s="21" t="s">
-        <v>336</v>
+        <v>311</v>
       </c>
     </row>
     <row r="94" spans="1:5">
@@ -4062,13 +4065,13 @@
         <v>80</v>
       </c>
       <c r="C94" s="20" t="s">
-        <v>337</v>
+        <v>312</v>
       </c>
       <c r="D94" s="22" t="s">
-        <v>338</v>
+        <v>313</v>
       </c>
       <c r="E94" s="22" t="s">
-        <v>339</v>
+        <v>314</v>
       </c>
     </row>
     <row r="95" spans="1:5">
@@ -4079,13 +4082,13 @@
         <v>80</v>
       </c>
       <c r="C95" s="29" t="s">
-        <v>350</v>
+        <v>325</v>
       </c>
       <c r="D95" s="27" t="s">
-        <v>354</v>
+        <v>326</v>
       </c>
       <c r="E95" s="27" t="s">
-        <v>355</v>
+        <v>327</v>
       </c>
     </row>
     <row r="96" spans="1:5">
@@ -4097,13 +4100,13 @@
         <v>80</v>
       </c>
       <c r="C96" s="30" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
       <c r="D96" s="31" t="s">
         <v>100</v>
       </c>
       <c r="E96" s="31" t="s">
-        <v>356</v>
+        <v>328</v>
       </c>
     </row>
     <row r="97" spans="1:5">
@@ -4115,13 +4118,13 @@
         <v>80</v>
       </c>
       <c r="C97" s="26" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
       <c r="D97" s="27" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="E97" s="27" t="s">
-        <v>357</v>
+        <v>329</v>
       </c>
     </row>
     <row r="98" spans="1:5">
@@ -4133,13 +4136,13 @@
         <v>80</v>
       </c>
       <c r="C98" s="26" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
       <c r="D98" s="27" t="s">
-        <v>347</v>
+        <v>322</v>
       </c>
       <c r="E98" s="27" t="s">
-        <v>348</v>
+        <v>323</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
publica cambios de calendario 2026-06-04 19:48
</commit_message>
<xml_diff>
--- a/Template_Calendario_CCS_GPX.xlsx
+++ b/Template_Calendario_CCS_GPX.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cesarmora/Library/Mobile Documents/com~apple~CloudDocs/Personal/Ciclismo/Calendario/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3AB4338-7F25-EE41-BC68-1AC1B9534735}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CF34706-A0B3-594E-AB01-24E903B5AB34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12200" yWindow="780" windowWidth="20720" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12200" yWindow="780" windowWidth="20720" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template_Calendario_CCS" sheetId="1" r:id="rId1"/>
@@ -108,9 +108,6 @@
     <t>Lo Prado - Cuesta Ibacache (Bis)</t>
   </si>
   <si>
-    <t>La Dormida - Chacabuco</t>
-  </si>
-  <si>
     <t>Coda - Las Dichas - Tunquén</t>
   </si>
   <si>
@@ -153,9 +150,6 @@
     <t>Lo Prado</t>
   </si>
   <si>
-    <t>La Dormida</t>
-  </si>
-  <si>
     <t>Strava</t>
   </si>
   <si>
@@ -1111,6 +1105,12 @@
   </si>
   <si>
     <t>27.150.755-0</t>
+  </si>
+  <si>
+    <t>Base Chacabuco - Cuesta La Dormida - Cuesta Chacabuco</t>
+  </si>
+  <si>
+    <t>Base Chacabuco</t>
   </si>
 </sst>
 </file>
@@ -1611,7 +1611,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K46"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -1646,19 +1646,19 @@
         <v>5</v>
       </c>
       <c r="G1" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="I1" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="J1" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="K1" s="12" t="s">
         <v>44</v>
-      </c>
-      <c r="J1" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="K1" s="12" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:11">
@@ -1672,13 +1672,13 @@
         <v>8</v>
       </c>
       <c r="D2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -1692,13 +1692,13 @@
         <v>9</v>
       </c>
       <c r="D3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -1712,13 +1712,13 @@
         <v>10</v>
       </c>
       <c r="D4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -1732,13 +1732,13 @@
         <v>11</v>
       </c>
       <c r="D5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -1752,13 +1752,13 @@
         <v>12</v>
       </c>
       <c r="D6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -1772,13 +1772,13 @@
         <v>13</v>
       </c>
       <c r="D7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -1792,13 +1792,13 @@
         <v>14</v>
       </c>
       <c r="D8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -1812,13 +1812,13 @@
         <v>15</v>
       </c>
       <c r="D9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -1829,16 +1829,16 @@
         <v>7</v>
       </c>
       <c r="C10" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="D10" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -1849,16 +1849,16 @@
         <v>7</v>
       </c>
       <c r="C11" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="D11" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -1872,13 +1872,13 @@
         <v>16</v>
       </c>
       <c r="D12" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -1892,13 +1892,13 @@
         <v>17</v>
       </c>
       <c r="D13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -1909,16 +1909,16 @@
         <v>6</v>
       </c>
       <c r="C14" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="D14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -1932,13 +1932,13 @@
         <v>18</v>
       </c>
       <c r="D15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -1949,16 +1949,16 @@
         <v>6</v>
       </c>
       <c r="C16" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D16" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -1972,13 +1972,13 @@
         <v>19</v>
       </c>
       <c r="D17" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -1992,13 +1992,13 @@
         <v>20</v>
       </c>
       <c r="D18" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -2012,13 +2012,13 @@
         <v>11</v>
       </c>
       <c r="D19" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -2029,16 +2029,16 @@
         <v>6</v>
       </c>
       <c r="C20" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="D20" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -2049,16 +2049,16 @@
         <v>7</v>
       </c>
       <c r="C21" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D21" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E21" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -2069,16 +2069,16 @@
         <v>7</v>
       </c>
       <c r="C22" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D22" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E22" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -2089,16 +2089,16 @@
         <v>7</v>
       </c>
       <c r="C23" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D23" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E23" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -2112,13 +2112,13 @@
         <v>17</v>
       </c>
       <c r="D24" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -2129,16 +2129,16 @@
         <v>6</v>
       </c>
       <c r="C25" t="s">
+        <v>317</v>
+      </c>
+      <c r="D25" t="s">
         <v>319</v>
       </c>
-      <c r="D25" t="s">
-        <v>321</v>
-      </c>
       <c r="E25" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -2152,13 +2152,13 @@
         <v>22</v>
       </c>
       <c r="D26" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -2172,13 +2172,13 @@
         <v>23</v>
       </c>
       <c r="D27" t="s">
+        <v>37</v>
+      </c>
+      <c r="E27" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="E27" s="10" t="s">
-        <v>40</v>
-      </c>
       <c r="F27" s="5" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -2189,16 +2189,16 @@
         <v>6</v>
       </c>
       <c r="C28" t="s">
-        <v>24</v>
+        <v>357</v>
       </c>
       <c r="D28" t="s">
-        <v>39</v>
+        <v>358</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -2209,16 +2209,16 @@
         <v>6</v>
       </c>
       <c r="C29" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D29" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="30" spans="1:6">
@@ -2229,16 +2229,16 @@
         <v>6</v>
       </c>
       <c r="C30" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D30" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="31" spans="1:6">
@@ -2249,16 +2249,16 @@
         <v>7</v>
       </c>
       <c r="C31" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D31" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E31" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -2269,16 +2269,16 @@
         <v>7</v>
       </c>
       <c r="C32" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D32" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E32" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="33" spans="1:6">
@@ -2289,16 +2289,16 @@
         <v>7</v>
       </c>
       <c r="C33" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D33" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E33" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="34" spans="1:6">
@@ -2312,13 +2312,13 @@
         <v>21</v>
       </c>
       <c r="D34" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="35" spans="1:6">
@@ -2332,13 +2332,13 @@
         <v>9</v>
       </c>
       <c r="D35" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="36" spans="1:6">
@@ -2467,7 +2467,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B1CA8C7-05A5-DA44-B969-9E41B832BB96}">
   <dimension ref="A1:E98"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="7.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.6640625" bestFit="1" customWidth="1"/>
@@ -2478,19 +2478,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="B1" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="C1" s="16" t="s">
         <v>75</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="D1" s="16" t="s">
         <v>76</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="E1" s="17" t="s">
         <v>77</v>
-      </c>
-      <c r="D1" s="16" t="s">
-        <v>78</v>
-      </c>
-      <c r="E1" s="17" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -2498,16 +2498,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="C2" s="20" t="s">
+        <v>79</v>
+      </c>
+      <c r="D2" s="20" t="s">
         <v>80</v>
       </c>
-      <c r="C2" s="20" t="s">
+      <c r="E2" s="21" t="s">
         <v>81</v>
-      </c>
-      <c r="D2" s="20" t="s">
-        <v>82</v>
-      </c>
-      <c r="E2" s="21" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -2515,16 +2515,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C3" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="D3" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="E3" s="21" t="s">
         <v>84</v>
-      </c>
-      <c r="D3" s="20" t="s">
-        <v>85</v>
-      </c>
-      <c r="E3" s="21" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -2532,16 +2532,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C4" s="20" t="s">
+        <v>85</v>
+      </c>
+      <c r="D4" s="22" t="s">
+        <v>86</v>
+      </c>
+      <c r="E4" s="22" t="s">
         <v>87</v>
-      </c>
-      <c r="D4" s="22" t="s">
-        <v>88</v>
-      </c>
-      <c r="E4" s="22" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -2549,16 +2549,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C5" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="D5" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="E5" s="22" t="s">
         <v>90</v>
-      </c>
-      <c r="D5" s="22" t="s">
-        <v>91</v>
-      </c>
-      <c r="E5" s="22" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -2566,16 +2566,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C6" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="D6" s="22" t="s">
+        <v>92</v>
+      </c>
+      <c r="E6" s="22" t="s">
         <v>93</v>
-      </c>
-      <c r="D6" s="22" t="s">
-        <v>94</v>
-      </c>
-      <c r="E6" s="22" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -2583,16 +2583,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C7" s="20" t="s">
+        <v>94</v>
+      </c>
+      <c r="D7" s="20" t="s">
+        <v>95</v>
+      </c>
+      <c r="E7" s="20" t="s">
         <v>96</v>
-      </c>
-      <c r="D7" s="20" t="s">
-        <v>97</v>
-      </c>
-      <c r="E7" s="20" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -2600,16 +2600,16 @@
         <v>7</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C8" s="20" t="s">
+        <v>97</v>
+      </c>
+      <c r="D8" s="20" t="s">
+        <v>98</v>
+      </c>
+      <c r="E8" s="21" t="s">
         <v>99</v>
-      </c>
-      <c r="D8" s="20" t="s">
-        <v>100</v>
-      </c>
-      <c r="E8" s="21" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -2617,16 +2617,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C9" s="20" t="s">
+        <v>100</v>
+      </c>
+      <c r="D9" s="20" t="s">
+        <v>101</v>
+      </c>
+      <c r="E9" s="21" t="s">
         <v>102</v>
-      </c>
-      <c r="D9" s="20" t="s">
-        <v>103</v>
-      </c>
-      <c r="E9" s="21" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -2634,16 +2634,16 @@
         <v>9</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C10" s="20" t="s">
+        <v>103</v>
+      </c>
+      <c r="D10" s="22" t="s">
+        <v>104</v>
+      </c>
+      <c r="E10" s="22" t="s">
         <v>105</v>
-      </c>
-      <c r="D10" s="22" t="s">
-        <v>106</v>
-      </c>
-      <c r="E10" s="22" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -2651,16 +2651,16 @@
         <v>10</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C11" s="20" t="s">
+        <v>106</v>
+      </c>
+      <c r="D11" s="22" t="s">
+        <v>107</v>
+      </c>
+      <c r="E11" s="22" t="s">
         <v>108</v>
-      </c>
-      <c r="D11" s="22" t="s">
-        <v>109</v>
-      </c>
-      <c r="E11" s="22" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -2668,16 +2668,16 @@
         <v>11</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C12" s="20" t="s">
+        <v>109</v>
+      </c>
+      <c r="D12" s="20" t="s">
+        <v>110</v>
+      </c>
+      <c r="E12" s="21" t="s">
         <v>111</v>
-      </c>
-      <c r="D12" s="20" t="s">
-        <v>112</v>
-      </c>
-      <c r="E12" s="21" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -2685,16 +2685,16 @@
         <v>12</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C13" s="20" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D13" s="20" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -2702,16 +2702,16 @@
         <v>13</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C14" s="20" t="s">
+        <v>114</v>
+      </c>
+      <c r="D14" s="20" t="s">
+        <v>115</v>
+      </c>
+      <c r="E14" s="21" t="s">
         <v>116</v>
-      </c>
-      <c r="D14" s="20" t="s">
-        <v>117</v>
-      </c>
-      <c r="E14" s="21" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -2719,16 +2719,16 @@
         <v>14</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C15" s="20" t="s">
+        <v>117</v>
+      </c>
+      <c r="D15" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="E15" s="21" t="s">
         <v>119</v>
-      </c>
-      <c r="D15" s="20" t="s">
-        <v>120</v>
-      </c>
-      <c r="E15" s="21" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -2736,16 +2736,16 @@
         <v>15</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C16" s="20" t="s">
+        <v>120</v>
+      </c>
+      <c r="D16" s="20" t="s">
+        <v>121</v>
+      </c>
+      <c r="E16" s="21" t="s">
         <v>122</v>
-      </c>
-      <c r="D16" s="20" t="s">
-        <v>123</v>
-      </c>
-      <c r="E16" s="21" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -2753,16 +2753,16 @@
         <v>16</v>
       </c>
       <c r="B17" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C17" s="20" t="s">
+        <v>123</v>
+      </c>
+      <c r="D17" s="20" t="s">
+        <v>124</v>
+      </c>
+      <c r="E17" s="21" t="s">
         <v>125</v>
-      </c>
-      <c r="D17" s="20" t="s">
-        <v>126</v>
-      </c>
-      <c r="E17" s="21" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -2770,16 +2770,16 @@
         <v>17</v>
       </c>
       <c r="B18" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C18" s="20" t="s">
+        <v>126</v>
+      </c>
+      <c r="D18" s="20" t="s">
+        <v>127</v>
+      </c>
+      <c r="E18" s="21" t="s">
         <v>128</v>
-      </c>
-      <c r="D18" s="20" t="s">
-        <v>129</v>
-      </c>
-      <c r="E18" s="21" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -2787,16 +2787,16 @@
         <v>18</v>
       </c>
       <c r="B19" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C19" s="20" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D19" s="20" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="E19" s="21" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -2804,16 +2804,16 @@
         <v>19</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C20" s="20" t="s">
+        <v>131</v>
+      </c>
+      <c r="D20" s="20" t="s">
+        <v>132</v>
+      </c>
+      <c r="E20" s="21" t="s">
         <v>133</v>
-      </c>
-      <c r="D20" s="20" t="s">
-        <v>134</v>
-      </c>
-      <c r="E20" s="21" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -2821,16 +2821,16 @@
         <v>20</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C21" s="20" t="s">
+        <v>134</v>
+      </c>
+      <c r="D21" s="22" t="s">
+        <v>135</v>
+      </c>
+      <c r="E21" s="22" t="s">
         <v>136</v>
-      </c>
-      <c r="D21" s="22" t="s">
-        <v>137</v>
-      </c>
-      <c r="E21" s="22" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -2838,16 +2838,16 @@
         <v>21</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C22" s="20" t="s">
+        <v>137</v>
+      </c>
+      <c r="D22" s="22" t="s">
+        <v>138</v>
+      </c>
+      <c r="E22" s="22" t="s">
         <v>139</v>
-      </c>
-      <c r="D22" s="22" t="s">
-        <v>140</v>
-      </c>
-      <c r="E22" s="22" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -2855,16 +2855,16 @@
         <v>22</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C23" s="20" t="s">
+        <v>140</v>
+      </c>
+      <c r="D23" s="20" t="s">
+        <v>141</v>
+      </c>
+      <c r="E23" s="21" t="s">
         <v>142</v>
-      </c>
-      <c r="D23" s="20" t="s">
-        <v>143</v>
-      </c>
-      <c r="E23" s="21" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -2872,16 +2872,16 @@
         <v>23</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C24" s="20" t="s">
+        <v>143</v>
+      </c>
+      <c r="D24" s="20" t="s">
+        <v>144</v>
+      </c>
+      <c r="E24" s="21" t="s">
         <v>145</v>
-      </c>
-      <c r="D24" s="20" t="s">
-        <v>146</v>
-      </c>
-      <c r="E24" s="21" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -2889,16 +2889,16 @@
         <v>24</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C25" s="20" t="s">
+        <v>146</v>
+      </c>
+      <c r="D25" s="20" t="s">
+        <v>147</v>
+      </c>
+      <c r="E25" s="21" t="s">
         <v>148</v>
-      </c>
-      <c r="D25" s="20" t="s">
-        <v>149</v>
-      </c>
-      <c r="E25" s="21" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -2906,16 +2906,16 @@
         <v>25</v>
       </c>
       <c r="B26" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C26" s="20" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="D26" s="22" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E26" s="22" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -2923,16 +2923,16 @@
         <v>26</v>
       </c>
       <c r="B27" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C27" s="20" t="s">
+        <v>151</v>
+      </c>
+      <c r="D27" s="20" t="s">
+        <v>152</v>
+      </c>
+      <c r="E27" s="21" t="s">
         <v>153</v>
-      </c>
-      <c r="D27" s="20" t="s">
-        <v>154</v>
-      </c>
-      <c r="E27" s="21" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -2940,16 +2940,16 @@
         <v>27</v>
       </c>
       <c r="B28" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C28" s="20" t="s">
+        <v>154</v>
+      </c>
+      <c r="D28" s="20" t="s">
+        <v>155</v>
+      </c>
+      <c r="E28" s="21" t="s">
         <v>156</v>
-      </c>
-      <c r="D28" s="20" t="s">
-        <v>157</v>
-      </c>
-      <c r="E28" s="21" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -2957,16 +2957,16 @@
         <v>28</v>
       </c>
       <c r="B29" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C29" s="20" t="s">
+        <v>157</v>
+      </c>
+      <c r="D29" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E29" s="21" t="s">
         <v>159</v>
-      </c>
-      <c r="D29" s="20" t="s">
-        <v>160</v>
-      </c>
-      <c r="E29" s="21" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="30" spans="1:5">
@@ -2974,16 +2974,16 @@
         <v>29</v>
       </c>
       <c r="B30" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C30" s="20" t="s">
+        <v>160</v>
+      </c>
+      <c r="D30" s="22" t="s">
+        <v>161</v>
+      </c>
+      <c r="E30" s="22" t="s">
         <v>162</v>
-      </c>
-      <c r="D30" s="22" t="s">
-        <v>163</v>
-      </c>
-      <c r="E30" s="22" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="31" spans="1:5">
@@ -2991,16 +2991,16 @@
         <v>30</v>
       </c>
       <c r="B31" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C31" s="20" t="s">
+        <v>163</v>
+      </c>
+      <c r="D31" s="20" t="s">
+        <v>164</v>
+      </c>
+      <c r="E31" s="21" t="s">
         <v>165</v>
-      </c>
-      <c r="D31" s="20" t="s">
-        <v>166</v>
-      </c>
-      <c r="E31" s="21" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="32" spans="1:5">
@@ -3008,16 +3008,16 @@
         <v>31</v>
       </c>
       <c r="B32" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C32" s="20" t="s">
+        <v>166</v>
+      </c>
+      <c r="D32" s="20" t="s">
+        <v>167</v>
+      </c>
+      <c r="E32" s="21" t="s">
         <v>168</v>
-      </c>
-      <c r="D32" s="20" t="s">
-        <v>169</v>
-      </c>
-      <c r="E32" s="21" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="33" spans="1:5">
@@ -3025,16 +3025,16 @@
         <v>32</v>
       </c>
       <c r="B33" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C33" s="20" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D33" s="20" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="E33" s="21" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="34" spans="1:5">
@@ -3042,16 +3042,16 @@
         <v>33</v>
       </c>
       <c r="B34" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C34" s="20" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="D34" s="20" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E34" s="21" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="35" spans="1:5">
@@ -3059,16 +3059,16 @@
         <v>34</v>
       </c>
       <c r="B35" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C35" s="20" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="D35" s="20" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E35" s="21" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="36" spans="1:5">
@@ -3076,16 +3076,16 @@
         <v>35</v>
       </c>
       <c r="B36" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C36" s="20" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="D36" s="20" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="E36" s="21" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="37" spans="1:5">
@@ -3093,16 +3093,16 @@
         <v>36</v>
       </c>
       <c r="B37" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C37" s="20" t="s">
+        <v>176</v>
+      </c>
+      <c r="D37" s="20" t="s">
+        <v>177</v>
+      </c>
+      <c r="E37" s="21" t="s">
         <v>178</v>
-      </c>
-      <c r="D37" s="20" t="s">
-        <v>179</v>
-      </c>
-      <c r="E37" s="21" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="38" spans="1:5">
@@ -3110,16 +3110,16 @@
         <v>37</v>
       </c>
       <c r="B38" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C38" s="20" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="D38" s="20" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="E38" s="21" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="39" spans="1:5">
@@ -3127,16 +3127,16 @@
         <v>38</v>
       </c>
       <c r="B39" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C39" s="20" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="D39" s="20" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="E39" s="21" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="40" spans="1:5">
@@ -3144,16 +3144,16 @@
         <v>39</v>
       </c>
       <c r="B40" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C40" s="20" t="s">
+        <v>183</v>
+      </c>
+      <c r="D40" s="20" t="s">
+        <v>184</v>
+      </c>
+      <c r="E40" s="21" t="s">
         <v>185</v>
-      </c>
-      <c r="D40" s="20" t="s">
-        <v>186</v>
-      </c>
-      <c r="E40" s="21" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="41" spans="1:5">
@@ -3161,16 +3161,16 @@
         <v>40</v>
       </c>
       <c r="B41" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C41" s="24" t="s">
+        <v>186</v>
+      </c>
+      <c r="D41" s="20" t="s">
+        <v>187</v>
+      </c>
+      <c r="E41" s="21" t="s">
         <v>188</v>
-      </c>
-      <c r="D41" s="20" t="s">
-        <v>189</v>
-      </c>
-      <c r="E41" s="21" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="42" spans="1:5">
@@ -3178,16 +3178,16 @@
         <v>41</v>
       </c>
       <c r="B42" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C42" s="20" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D42" s="22" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="E42" s="22" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
     </row>
     <row r="43" spans="1:5">
@@ -3195,16 +3195,16 @@
         <v>42</v>
       </c>
       <c r="B43" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C43" s="20" t="s">
+        <v>191</v>
+      </c>
+      <c r="D43" s="22" t="s">
+        <v>192</v>
+      </c>
+      <c r="E43" s="22" t="s">
         <v>193</v>
-      </c>
-      <c r="D43" s="22" t="s">
-        <v>194</v>
-      </c>
-      <c r="E43" s="22" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="44" spans="1:5">
@@ -3212,16 +3212,16 @@
         <v>43</v>
       </c>
       <c r="B44" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C44" s="20" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="D44" s="20" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="E44" s="21" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
     </row>
     <row r="45" spans="1:5">
@@ -3229,16 +3229,16 @@
         <v>44</v>
       </c>
       <c r="B45" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C45" s="20" t="s">
+        <v>196</v>
+      </c>
+      <c r="D45" s="22" t="s">
+        <v>197</v>
+      </c>
+      <c r="E45" s="22" t="s">
         <v>198</v>
-      </c>
-      <c r="D45" s="22" t="s">
-        <v>199</v>
-      </c>
-      <c r="E45" s="22" t="s">
-        <v>200</v>
       </c>
     </row>
     <row r="46" spans="1:5">
@@ -3246,16 +3246,16 @@
         <v>45</v>
       </c>
       <c r="B46" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C46" s="23" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="D46" s="20" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E46" s="21" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
     </row>
     <row r="47" spans="1:5">
@@ -3263,16 +3263,16 @@
         <v>46</v>
       </c>
       <c r="B47" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C47" s="20" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="D47" s="20" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="E47" s="21" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
     </row>
     <row r="48" spans="1:5">
@@ -3280,16 +3280,16 @@
         <v>47</v>
       </c>
       <c r="B48" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C48" s="20" t="s">
+        <v>202</v>
+      </c>
+      <c r="D48" s="20" t="s">
+        <v>203</v>
+      </c>
+      <c r="E48" s="21" t="s">
         <v>204</v>
-      </c>
-      <c r="D48" s="20" t="s">
-        <v>205</v>
-      </c>
-      <c r="E48" s="21" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="49" spans="1:5">
@@ -3297,16 +3297,16 @@
         <v>48</v>
       </c>
       <c r="B49" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C49" s="20" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="D49" s="20" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="E49" s="21" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="50" spans="1:5">
@@ -3314,16 +3314,16 @@
         <v>49</v>
       </c>
       <c r="B50" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C50" s="20" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="D50" s="22" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E50" s="22" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
     </row>
     <row r="51" spans="1:5">
@@ -3331,16 +3331,16 @@
         <v>50</v>
       </c>
       <c r="B51" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C51" s="20" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="D51" s="20" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E51" s="21" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
     </row>
     <row r="52" spans="1:5">
@@ -3348,16 +3348,16 @@
         <v>51</v>
       </c>
       <c r="B52" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C52" s="20" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="D52" s="20" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="E52" s="21" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
     </row>
     <row r="53" spans="1:5">
@@ -3365,16 +3365,16 @@
         <v>52</v>
       </c>
       <c r="B53" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C53" s="20" t="s">
+        <v>211</v>
+      </c>
+      <c r="D53" s="20" t="s">
+        <v>212</v>
+      </c>
+      <c r="E53" s="21" t="s">
         <v>213</v>
-      </c>
-      <c r="D53" s="20" t="s">
-        <v>214</v>
-      </c>
-      <c r="E53" s="21" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="54" spans="1:5">
@@ -3382,16 +3382,16 @@
         <v>53</v>
       </c>
       <c r="B54" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C54" s="20" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="D54" s="20" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="E54" s="21" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="55" spans="1:5">
@@ -3399,16 +3399,16 @@
         <v>54</v>
       </c>
       <c r="B55" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C55" s="20" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="D55" s="20" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="E55" s="21" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
     </row>
     <row r="56" spans="1:5">
@@ -3416,16 +3416,16 @@
         <v>55</v>
       </c>
       <c r="B56" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C56" s="20" t="s">
+        <v>218</v>
+      </c>
+      <c r="D56" s="22" t="s">
+        <v>219</v>
+      </c>
+      <c r="E56" s="22" t="s">
         <v>220</v>
-      </c>
-      <c r="D56" s="22" t="s">
-        <v>221</v>
-      </c>
-      <c r="E56" s="22" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="57" spans="1:5">
@@ -3433,16 +3433,16 @@
         <v>56</v>
       </c>
       <c r="B57" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C57" s="20" t="s">
+        <v>221</v>
+      </c>
+      <c r="D57" s="22" t="s">
+        <v>222</v>
+      </c>
+      <c r="E57" s="22" t="s">
         <v>223</v>
-      </c>
-      <c r="D57" s="22" t="s">
-        <v>224</v>
-      </c>
-      <c r="E57" s="22" t="s">
-        <v>225</v>
       </c>
     </row>
     <row r="58" spans="1:5">
@@ -3450,16 +3450,16 @@
         <v>57</v>
       </c>
       <c r="B58" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C58" s="20" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="D58" s="20" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="E58" s="21" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
     </row>
     <row r="59" spans="1:5">
@@ -3467,16 +3467,16 @@
         <v>58</v>
       </c>
       <c r="B59" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C59" s="20" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="D59" s="22" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="E59" s="22" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="60" spans="1:5">
@@ -3484,16 +3484,16 @@
         <v>59</v>
       </c>
       <c r="B60" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C60" s="20" t="s">
+        <v>228</v>
+      </c>
+      <c r="D60" s="20" t="s">
+        <v>229</v>
+      </c>
+      <c r="E60" s="21" t="s">
         <v>230</v>
-      </c>
-      <c r="D60" s="20" t="s">
-        <v>231</v>
-      </c>
-      <c r="E60" s="21" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="61" spans="1:5">
@@ -3501,16 +3501,16 @@
         <v>60</v>
       </c>
       <c r="B61" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C61" s="20" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="D61" s="20" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E61" s="21" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
     <row r="62" spans="1:5">
@@ -3518,16 +3518,16 @@
         <v>61</v>
       </c>
       <c r="B62" s="22" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C62" s="20" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="D62" s="20" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="E62" s="21" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
     </row>
     <row r="63" spans="1:5">
@@ -3535,16 +3535,16 @@
         <v>62</v>
       </c>
       <c r="B63" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C63" s="20" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="D63" s="20" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="E63" s="21" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
     </row>
     <row r="64" spans="1:5">
@@ -3552,16 +3552,16 @@
         <v>63</v>
       </c>
       <c r="B64" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C64" s="20" t="s">
+        <v>236</v>
+      </c>
+      <c r="D64" s="20" t="s">
+        <v>237</v>
+      </c>
+      <c r="E64" s="21" t="s">
         <v>238</v>
-      </c>
-      <c r="D64" s="20" t="s">
-        <v>239</v>
-      </c>
-      <c r="E64" s="21" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="65" spans="1:5">
@@ -3569,16 +3569,16 @@
         <v>64</v>
       </c>
       <c r="B65" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C65" s="20" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="D65" s="20" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E65" s="21" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="66" spans="1:5">
@@ -3586,16 +3586,16 @@
         <v>65</v>
       </c>
       <c r="B66" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C66" s="20" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="D66" s="20" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="E66" s="21" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="67" spans="1:5">
@@ -3603,16 +3603,16 @@
         <v>66</v>
       </c>
       <c r="B67" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C67" s="20" t="s">
+        <v>242</v>
+      </c>
+      <c r="D67" s="20" t="s">
+        <v>243</v>
+      </c>
+      <c r="E67" s="21" t="s">
         <v>244</v>
-      </c>
-      <c r="D67" s="20" t="s">
-        <v>245</v>
-      </c>
-      <c r="E67" s="21" t="s">
-        <v>246</v>
       </c>
     </row>
     <row r="68" spans="1:5">
@@ -3620,16 +3620,16 @@
         <v>67</v>
       </c>
       <c r="B68" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C68" s="20" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="D68" s="20" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="E68" s="21" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
     </row>
     <row r="69" spans="1:5">
@@ -3637,16 +3637,16 @@
         <v>68</v>
       </c>
       <c r="B69" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C69" s="20" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="D69" s="20" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="E69" s="21" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="70" spans="1:5">
@@ -3654,16 +3654,16 @@
         <v>69</v>
       </c>
       <c r="B70" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C70" s="20" t="s">
+        <v>249</v>
+      </c>
+      <c r="D70" s="22" t="s">
+        <v>250</v>
+      </c>
+      <c r="E70" s="22" t="s">
         <v>251</v>
-      </c>
-      <c r="D70" s="22" t="s">
-        <v>252</v>
-      </c>
-      <c r="E70" s="22" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="71" spans="1:5">
@@ -3671,16 +3671,16 @@
         <v>70</v>
       </c>
       <c r="B71" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C71" s="20" t="s">
+        <v>252</v>
+      </c>
+      <c r="D71" s="20" t="s">
+        <v>253</v>
+      </c>
+      <c r="E71" s="21" t="s">
         <v>254</v>
-      </c>
-      <c r="D71" s="20" t="s">
-        <v>255</v>
-      </c>
-      <c r="E71" s="21" t="s">
-        <v>256</v>
       </c>
     </row>
     <row r="72" spans="1:5">
@@ -3688,16 +3688,16 @@
         <v>71</v>
       </c>
       <c r="B72" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C72" s="20" t="s">
+        <v>255</v>
+      </c>
+      <c r="D72" s="22" t="s">
+        <v>256</v>
+      </c>
+      <c r="E72" s="22" t="s">
         <v>257</v>
-      </c>
-      <c r="D72" s="22" t="s">
-        <v>258</v>
-      </c>
-      <c r="E72" s="22" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="73" spans="1:5">
@@ -3705,16 +3705,16 @@
         <v>72</v>
       </c>
       <c r="B73" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C73" s="20" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="D73" s="20" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="E73" s="21" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="74" spans="1:5">
@@ -3722,16 +3722,16 @@
         <v>73</v>
       </c>
       <c r="B74" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C74" s="20" t="s">
+        <v>260</v>
+      </c>
+      <c r="D74" s="20" t="s">
+        <v>261</v>
+      </c>
+      <c r="E74" s="21" t="s">
         <v>262</v>
-      </c>
-      <c r="D74" s="20" t="s">
-        <v>263</v>
-      </c>
-      <c r="E74" s="21" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="75" spans="1:5">
@@ -3739,16 +3739,16 @@
         <v>74</v>
       </c>
       <c r="B75" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C75" s="20" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="D75" s="22" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E75" s="22" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
     </row>
     <row r="76" spans="1:5">
@@ -3756,16 +3756,16 @@
         <v>75</v>
       </c>
       <c r="B76" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C76" s="20" t="s">
+        <v>265</v>
+      </c>
+      <c r="D76" s="22" t="s">
+        <v>266</v>
+      </c>
+      <c r="E76" s="22" t="s">
         <v>267</v>
-      </c>
-      <c r="D76" s="22" t="s">
-        <v>268</v>
-      </c>
-      <c r="E76" s="22" t="s">
-        <v>269</v>
       </c>
     </row>
     <row r="77" spans="1:5">
@@ -3773,16 +3773,16 @@
         <v>76</v>
       </c>
       <c r="B77" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C77" s="20" t="s">
+        <v>268</v>
+      </c>
+      <c r="D77" s="22" t="s">
+        <v>269</v>
+      </c>
+      <c r="E77" s="22" t="s">
         <v>270</v>
-      </c>
-      <c r="D77" s="22" t="s">
-        <v>271</v>
-      </c>
-      <c r="E77" s="22" t="s">
-        <v>272</v>
       </c>
     </row>
     <row r="78" spans="1:5">
@@ -3790,16 +3790,16 @@
         <v>77</v>
       </c>
       <c r="B78" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C78" s="20" t="s">
+        <v>271</v>
+      </c>
+      <c r="D78" s="22" t="s">
+        <v>272</v>
+      </c>
+      <c r="E78" s="22" t="s">
         <v>273</v>
-      </c>
-      <c r="D78" s="22" t="s">
-        <v>274</v>
-      </c>
-      <c r="E78" s="22" t="s">
-        <v>275</v>
       </c>
     </row>
     <row r="79" spans="1:5">
@@ -3807,16 +3807,16 @@
         <v>78</v>
       </c>
       <c r="B79" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C79" s="20" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="D79" s="20" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="E79" s="21" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
     </row>
     <row r="80" spans="1:5">
@@ -3824,16 +3824,16 @@
         <v>79</v>
       </c>
       <c r="B80" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C80" s="20" t="s">
+        <v>276</v>
+      </c>
+      <c r="D80" s="22" t="s">
+        <v>277</v>
+      </c>
+      <c r="E80" s="22" t="s">
         <v>278</v>
-      </c>
-      <c r="D80" s="22" t="s">
-        <v>279</v>
-      </c>
-      <c r="E80" s="22" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="81" spans="1:5">
@@ -3841,16 +3841,16 @@
         <v>80</v>
       </c>
       <c r="B81" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C81" s="20" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="D81" s="20" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="E81" s="21" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
     </row>
     <row r="82" spans="1:5">
@@ -3858,16 +3858,16 @@
         <v>81</v>
       </c>
       <c r="B82" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C82" s="20" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="D82" s="20" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="E82" s="21" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
     </row>
     <row r="83" spans="1:5">
@@ -3875,16 +3875,16 @@
         <v>82</v>
       </c>
       <c r="B83" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C83" s="20" t="s">
+        <v>283</v>
+      </c>
+      <c r="D83" s="20" t="s">
+        <v>284</v>
+      </c>
+      <c r="E83" s="21" t="s">
         <v>285</v>
-      </c>
-      <c r="D83" s="20" t="s">
-        <v>286</v>
-      </c>
-      <c r="E83" s="21" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="84" spans="1:5">
@@ -3892,16 +3892,16 @@
         <v>83</v>
       </c>
       <c r="B84" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C84" s="20" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="D84" s="20" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="E84" s="21" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
     </row>
     <row r="85" spans="1:5">
@@ -3909,16 +3909,16 @@
         <v>84</v>
       </c>
       <c r="B85" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C85" s="20" t="s">
+        <v>287</v>
+      </c>
+      <c r="D85" s="20" t="s">
+        <v>288</v>
+      </c>
+      <c r="E85" s="21" t="s">
         <v>289</v>
-      </c>
-      <c r="D85" s="20" t="s">
-        <v>290</v>
-      </c>
-      <c r="E85" s="21" t="s">
-        <v>291</v>
       </c>
     </row>
     <row r="86" spans="1:5">
@@ -3926,16 +3926,16 @@
         <v>85</v>
       </c>
       <c r="B86" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C86" s="20" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="D86" s="20" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="E86" s="21" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
     </row>
     <row r="87" spans="1:5">
@@ -3943,16 +3943,16 @@
         <v>86</v>
       </c>
       <c r="B87" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C87" s="20" t="s">
+        <v>292</v>
+      </c>
+      <c r="D87" s="20" t="s">
+        <v>293</v>
+      </c>
+      <c r="E87" s="21" t="s">
         <v>294</v>
-      </c>
-      <c r="D87" s="20" t="s">
-        <v>295</v>
-      </c>
-      <c r="E87" s="21" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="88" spans="1:5">
@@ -3960,16 +3960,16 @@
         <v>87</v>
       </c>
       <c r="B88" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C88" s="20" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="D88" s="20" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="E88" s="21" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="89" spans="1:5">
@@ -3977,16 +3977,16 @@
         <v>88</v>
       </c>
       <c r="B89" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C89" s="20" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="D89" s="20" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E89" s="21" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="90" spans="1:5">
@@ -3994,16 +3994,16 @@
         <v>89</v>
       </c>
       <c r="B90" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C90" s="20" t="s">
+        <v>299</v>
+      </c>
+      <c r="D90" s="20" t="s">
+        <v>300</v>
+      </c>
+      <c r="E90" s="21" t="s">
         <v>301</v>
-      </c>
-      <c r="D90" s="20" t="s">
-        <v>302</v>
-      </c>
-      <c r="E90" s="21" t="s">
-        <v>303</v>
       </c>
     </row>
     <row r="91" spans="1:5">
@@ -4011,16 +4011,16 @@
         <v>90</v>
       </c>
       <c r="B91" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C91" s="20" t="s">
+        <v>302</v>
+      </c>
+      <c r="D91" s="20" t="s">
+        <v>303</v>
+      </c>
+      <c r="E91" s="21" t="s">
         <v>304</v>
-      </c>
-      <c r="D91" s="20" t="s">
-        <v>305</v>
-      </c>
-      <c r="E91" s="21" t="s">
-        <v>306</v>
       </c>
     </row>
     <row r="92" spans="1:5">
@@ -4028,16 +4028,16 @@
         <v>91</v>
       </c>
       <c r="B92" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C92" s="20" t="s">
+        <v>305</v>
+      </c>
+      <c r="D92" s="20" t="s">
+        <v>306</v>
+      </c>
+      <c r="E92" s="21" t="s">
         <v>307</v>
-      </c>
-      <c r="D92" s="20" t="s">
-        <v>308</v>
-      </c>
-      <c r="E92" s="21" t="s">
-        <v>309</v>
       </c>
     </row>
     <row r="93" spans="1:5">
@@ -4045,16 +4045,16 @@
         <v>92</v>
       </c>
       <c r="B93" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C93" s="20" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="D93" s="20" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="E93" s="21" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
     </row>
     <row r="94" spans="1:5">
@@ -4062,16 +4062,16 @@
         <v>93</v>
       </c>
       <c r="B94" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C94" s="20" t="s">
+        <v>310</v>
+      </c>
+      <c r="D94" s="22" t="s">
+        <v>311</v>
+      </c>
+      <c r="E94" s="22" t="s">
         <v>312</v>
-      </c>
-      <c r="D94" s="22" t="s">
-        <v>313</v>
-      </c>
-      <c r="E94" s="22" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="95" spans="1:5">
@@ -4079,16 +4079,16 @@
         <v>94</v>
       </c>
       <c r="B95" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C95" s="29" t="s">
+        <v>323</v>
+      </c>
+      <c r="D95" s="27" t="s">
+        <v>324</v>
+      </c>
+      <c r="E95" s="27" t="s">
         <v>325</v>
-      </c>
-      <c r="D95" s="27" t="s">
-        <v>326</v>
-      </c>
-      <c r="E95" s="27" t="s">
-        <v>327</v>
       </c>
     </row>
     <row r="96" spans="1:5">
@@ -4097,16 +4097,16 @@
         <v>95</v>
       </c>
       <c r="B96" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C96" s="30" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="D96" s="31" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E96" s="31" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
     </row>
     <row r="97" spans="1:5">
@@ -4115,16 +4115,16 @@
         <v>96</v>
       </c>
       <c r="B97" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C97" s="26" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="D97" s="27" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="E97" s="27" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="98" spans="1:5">
@@ -4133,16 +4133,16 @@
         <v>97</v>
       </c>
       <c r="B98" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C98" s="26" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="D98" s="27" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="E98" s="27" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
agrega 3 links de Strava por ruta (niveles R/M/C)
- Excel con columnas R/M/C (Ristretto/Macchiato/Capuccino), un link por grupo
- backend: extractStravaLink lee R/M/C; M y C caen a R si aun no tienen su URL propia
  (hoy clonadas con formula =E2, que no arrastra el hipervinculo)
- frontend: buildStravaButtons muestra 3 botones en tabla, tarjetas y etapas
- regenera datos: 53 rutas con R/M/C, 14 sin (viajes/eventos sin Strava)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Template_Calendario_CCS_GPX.xlsx
+++ b/Template_Calendario_CCS_GPX.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cesarmora/Library/Mobile Documents/com~apple~CloudDocs/Personal/Ciclismo/Calendario/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8816E816-65EE-3B4C-8B39-CF9EE9D2A8C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A23A874-A946-6244-AD08-7401901FEE09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Usuarios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Template_Calendario_CCS!$A$1:$K$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Template_Calendario_CCS!$A$1:$M$68</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="739" uniqueCount="376">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="741" uniqueCount="378">
   <si>
     <t>Fecha</t>
   </si>
@@ -51,9 +51,6 @@
     <t>Inicio</t>
   </si>
   <si>
-    <t>Link Strava</t>
-  </si>
-  <si>
     <t>Archivo GPX</t>
   </si>
   <si>
@@ -1165,6 +1162,15 @@
   </si>
   <si>
     <t>Aurora - Chorombo Alto - Mallarauco - Barriga - Aurora</t>
+  </si>
+  <si>
+    <t>R</t>
+  </si>
+  <si>
+    <t>M</t>
+  </si>
+  <si>
+    <t>C</t>
   </si>
 </sst>
 </file>
@@ -1656,23 +1662,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K68"/>
+  <dimension ref="A1:M68"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14" style="6" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
     <col min="3" max="3" width="66.83203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="24" customWidth="1"/>
-    <col min="5" max="5" width="48.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="49.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.83203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.83203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="23.5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="49.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.83203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.83203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="23.5" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="37.25" customHeight="1">
+    <row r="1" spans="1:13" ht="37.25" customHeight="1">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -1686,1365 +1692,1907 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>375</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>376</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="8" t="s">
+      <c r="I1" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="J1" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="K1" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="L1" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="J1" s="9" t="s">
+      <c r="M1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="K1" s="9" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11">
+    </row>
+    <row r="2" spans="1:13">
       <c r="A2" s="6">
         <v>46025</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11">
+        <v>36</v>
+      </c>
+      <c r="F2" s="7" t="str">
+        <f>E2</f>
+        <v>Strava</v>
+      </c>
+      <c r="G2" s="7" t="str">
+        <f>F2</f>
+        <v>Strava</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
       <c r="A3" s="6">
         <v>46032</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11">
+        <v>36</v>
+      </c>
+      <c r="F3" s="7" t="str">
+        <f t="shared" ref="F3:G3" si="0">E3</f>
+        <v>Strava</v>
+      </c>
+      <c r="G3" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>Strava</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
       <c r="A4" s="6">
         <v>46039</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11">
+        <v>36</v>
+      </c>
+      <c r="F4" s="7" t="str">
+        <f t="shared" ref="F4:G4" si="1">E4</f>
+        <v>Strava</v>
+      </c>
+      <c r="G4" s="7" t="str">
+        <f t="shared" si="1"/>
+        <v>Strava</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
       <c r="A5" s="6">
         <v>46046</v>
       </c>
       <c r="B5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11">
+        <v>36</v>
+      </c>
+      <c r="F5" s="7" t="str">
+        <f t="shared" ref="F5:G5" si="2">E5</f>
+        <v>Strava</v>
+      </c>
+      <c r="G5" s="7" t="str">
+        <f t="shared" si="2"/>
+        <v>Strava</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
       <c r="A6" s="6">
         <v>46053</v>
       </c>
       <c r="B6" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11">
+        <v>36</v>
+      </c>
+      <c r="F6" s="7" t="str">
+        <f t="shared" ref="F6:G6" si="3">E6</f>
+        <v>Strava</v>
+      </c>
+      <c r="G6" s="7" t="str">
+        <f t="shared" si="3"/>
+        <v>Strava</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
       <c r="A7" s="6">
         <v>46060</v>
       </c>
       <c r="B7" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11">
+        <v>36</v>
+      </c>
+      <c r="F7" s="7" t="str">
+        <f t="shared" ref="F7:G7" si="4">E7</f>
+        <v>Strava</v>
+      </c>
+      <c r="G7" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>Strava</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
       <c r="A8" s="6">
         <v>46067</v>
       </c>
       <c r="B8" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D8" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11">
+        <v>36</v>
+      </c>
+      <c r="F8" s="7" t="str">
+        <f t="shared" ref="F8:G8" si="5">E8</f>
+        <v>Strava</v>
+      </c>
+      <c r="G8" s="7" t="str">
+        <f t="shared" si="5"/>
+        <v>Strava</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
       <c r="A9" s="6">
         <v>46074</v>
       </c>
       <c r="B9" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11">
+        <v>36</v>
+      </c>
+      <c r="F9" s="7" t="str">
+        <f t="shared" ref="F9:G9" si="6">E9</f>
+        <v>Strava</v>
+      </c>
+      <c r="G9" s="7" t="str">
+        <f t="shared" si="6"/>
+        <v>Strava</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
       <c r="A10" s="6">
         <v>46080</v>
       </c>
       <c r="B10" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D10" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11">
+        <v>36</v>
+      </c>
+      <c r="F10" s="7" t="str">
+        <f t="shared" ref="F10:G10" si="7">E10</f>
+        <v>Strava</v>
+      </c>
+      <c r="G10" s="7" t="str">
+        <f t="shared" si="7"/>
+        <v>Strava</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13">
       <c r="A11" s="6">
         <v>46081</v>
       </c>
       <c r="B11" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C11" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D11" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11">
+        <v>36</v>
+      </c>
+      <c r="F11" s="7" t="str">
+        <f t="shared" ref="F11:G11" si="8">E11</f>
+        <v>Strava</v>
+      </c>
+      <c r="G11" s="7" t="str">
+        <f t="shared" si="8"/>
+        <v>Strava</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13">
       <c r="A12" s="6">
         <v>46088</v>
       </c>
       <c r="B12" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C12" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11">
+        <v>36</v>
+      </c>
+      <c r="F12" s="7" t="str">
+        <f t="shared" ref="F12:G12" si="9">E12</f>
+        <v>Strava</v>
+      </c>
+      <c r="G12" s="7" t="str">
+        <f t="shared" si="9"/>
+        <v>Strava</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13">
       <c r="A13" s="6">
         <v>46095</v>
       </c>
       <c r="B13" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C13" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11">
+        <v>36</v>
+      </c>
+      <c r="F13" s="7" t="str">
+        <f t="shared" ref="F13:G13" si="10">E13</f>
+        <v>Strava</v>
+      </c>
+      <c r="G13" s="7" t="str">
+        <f t="shared" si="10"/>
+        <v>Strava</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13">
       <c r="A14" s="6">
         <v>46102</v>
       </c>
       <c r="B14" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C14" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D14" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11">
+        <v>36</v>
+      </c>
+      <c r="F14" s="7" t="str">
+        <f t="shared" ref="F14:G14" si="11">E14</f>
+        <v>Strava</v>
+      </c>
+      <c r="G14" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v>Strava</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13">
       <c r="A15" s="6">
         <v>46109</v>
       </c>
       <c r="B15" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C15" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D15" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11">
+        <v>36</v>
+      </c>
+      <c r="F15" s="7" t="str">
+        <f t="shared" ref="F15:G15" si="12">E15</f>
+        <v>Strava</v>
+      </c>
+      <c r="G15" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>Strava</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13">
       <c r="A16" s="6">
         <v>45750</v>
       </c>
       <c r="B16" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C16" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6">
+        <v>36</v>
+      </c>
+      <c r="F16" s="7" t="str">
+        <f t="shared" ref="F16:G16" si="13">E16</f>
+        <v>Strava</v>
+      </c>
+      <c r="G16" s="7" t="str">
+        <f t="shared" si="13"/>
+        <v>Strava</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8">
       <c r="A17" s="6">
         <v>46123</v>
       </c>
       <c r="B17" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C17" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D17" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F17" s="4" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6">
+        <v>36</v>
+      </c>
+      <c r="F17" s="7" t="str">
+        <f t="shared" ref="F17:G17" si="14">E17</f>
+        <v>Strava</v>
+      </c>
+      <c r="G17" s="7" t="str">
+        <f t="shared" si="14"/>
+        <v>Strava</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8">
       <c r="A18" s="6">
         <v>46130</v>
       </c>
       <c r="B18" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C18" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D18" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F18" s="4" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6">
+        <v>36</v>
+      </c>
+      <c r="F18" s="7" t="str">
+        <f t="shared" ref="F18:G18" si="15">E18</f>
+        <v>Strava</v>
+      </c>
+      <c r="G18" s="7" t="str">
+        <f t="shared" si="15"/>
+        <v>Strava</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8">
       <c r="A19" s="6">
         <v>46137</v>
       </c>
       <c r="B19" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C19" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D19" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F19" s="4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6">
+        <v>36</v>
+      </c>
+      <c r="F19" s="7" t="str">
+        <f t="shared" ref="F19:G19" si="16">E19</f>
+        <v>Strava</v>
+      </c>
+      <c r="G19" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>Strava</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8">
       <c r="A20" s="6">
         <v>46143</v>
       </c>
       <c r="B20" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C20" t="s">
+        <v>313</v>
+      </c>
+      <c r="D20" t="s">
+        <v>27</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="F20" s="7" t="str">
+        <f t="shared" ref="F20:G20" si="17">E20</f>
+        <v>Strava</v>
+      </c>
+      <c r="G20" s="7" t="str">
+        <f t="shared" si="17"/>
+        <v>Strava</v>
+      </c>
+      <c r="H20" s="4" t="s">
         <v>314</v>
       </c>
-      <c r="D20" t="s">
-        <v>28</v>
-      </c>
-      <c r="E20" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F20" s="4" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6">
+    </row>
+    <row r="21" spans="1:8">
       <c r="A21" s="6">
         <v>46150</v>
       </c>
       <c r="B21" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C21" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D21" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E21" t="s">
-        <v>38</v>
-      </c>
-      <c r="F21" s="4" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6">
+        <v>37</v>
+      </c>
+      <c r="F21" s="7" t="str">
+        <f t="shared" ref="F21:G21" si="18">E21</f>
+        <v>Por definir</v>
+      </c>
+      <c r="G21" s="7" t="str">
+        <f t="shared" si="18"/>
+        <v>Por definir</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
       <c r="A22" s="6">
         <v>46151</v>
       </c>
       <c r="B22" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C22" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D22" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E22" t="s">
-        <v>38</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6">
+        <v>37</v>
+      </c>
+      <c r="F22" s="7" t="str">
+        <f t="shared" ref="F22:G22" si="19">E22</f>
+        <v>Por definir</v>
+      </c>
+      <c r="G22" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>Por definir</v>
+      </c>
+      <c r="H22" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
       <c r="A23" s="6">
         <v>46152</v>
       </c>
       <c r="B23" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C23" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D23" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E23" t="s">
-        <v>38</v>
-      </c>
-      <c r="F23" s="4" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6">
+        <v>37</v>
+      </c>
+      <c r="F23" s="7" t="str">
+        <f t="shared" ref="F23:G23" si="20">E23</f>
+        <v>Por definir</v>
+      </c>
+      <c r="G23" s="7" t="str">
+        <f t="shared" si="20"/>
+        <v>Por definir</v>
+      </c>
+      <c r="H23" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8">
       <c r="A24" s="6">
         <v>46151</v>
       </c>
       <c r="B24" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C24" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D24" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F24" s="4" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6">
+        <v>36</v>
+      </c>
+      <c r="F24" s="7" t="str">
+        <f t="shared" ref="F24:G24" si="21">E24</f>
+        <v>Strava</v>
+      </c>
+      <c r="G24" s="7" t="str">
+        <f t="shared" si="21"/>
+        <v>Strava</v>
+      </c>
+      <c r="H24" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8">
       <c r="A25" s="6">
         <v>46158</v>
       </c>
       <c r="B25" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C25" t="s">
+        <v>315</v>
+      </c>
+      <c r="D25" t="s">
+        <v>317</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="F25" s="7" t="str">
+        <f t="shared" ref="F25:G25" si="22">E25</f>
+        <v>Strava</v>
+      </c>
+      <c r="G25" s="7" t="str">
+        <f t="shared" si="22"/>
+        <v>Strava</v>
+      </c>
+      <c r="H25" s="4" t="s">
         <v>316</v>
       </c>
-      <c r="D25" t="s">
-        <v>318</v>
-      </c>
-      <c r="E25" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F25" s="4" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6">
+    </row>
+    <row r="26" spans="1:8">
       <c r="A26" s="6">
         <v>46165</v>
       </c>
       <c r="B26" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C26" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D26" t="s">
+        <v>35</v>
+      </c>
+      <c r="E26" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="E26" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F26" s="4" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6">
+      <c r="F26" s="7" t="str">
+        <f t="shared" ref="F26:G26" si="23">E26</f>
+        <v>Strava</v>
+      </c>
+      <c r="G26" s="7" t="str">
+        <f t="shared" si="23"/>
+        <v>Strava</v>
+      </c>
+      <c r="H26" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8">
       <c r="A27" s="6">
         <v>46172</v>
       </c>
       <c r="B27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C27" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D27" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F27" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6">
+        <v>36</v>
+      </c>
+      <c r="F27" s="7" t="str">
+        <f t="shared" ref="F27:G27" si="24">E27</f>
+        <v>Strava</v>
+      </c>
+      <c r="G27" s="7" t="str">
+        <f t="shared" si="24"/>
+        <v>Strava</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8">
       <c r="A28" s="6">
         <v>46179</v>
       </c>
       <c r="B28" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C28" t="s">
+        <v>355</v>
+      </c>
+      <c r="D28" t="s">
         <v>356</v>
       </c>
-      <c r="D28" t="s">
-        <v>357</v>
-      </c>
       <c r="E28" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F28" s="4" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6">
+        <v>36</v>
+      </c>
+      <c r="F28" s="7" t="str">
+        <f t="shared" ref="F28:G28" si="25">E28</f>
+        <v>Strava</v>
+      </c>
+      <c r="G28" s="7" t="str">
+        <f t="shared" si="25"/>
+        <v>Strava</v>
+      </c>
+      <c r="H28" s="4" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8">
       <c r="A29" s="6">
         <v>46186</v>
       </c>
       <c r="B29" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C29" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D29" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F29" s="4" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6">
+        <v>36</v>
+      </c>
+      <c r="F29" s="7" t="str">
+        <f t="shared" ref="F29:G29" si="26">E29</f>
+        <v>Strava</v>
+      </c>
+      <c r="G29" s="7" t="str">
+        <f t="shared" si="26"/>
+        <v>Strava</v>
+      </c>
+      <c r="H29" s="4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8">
       <c r="A30" s="6">
         <v>46193</v>
       </c>
       <c r="B30" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C30" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D30" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F30" s="4" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6">
+        <v>36</v>
+      </c>
+      <c r="F30" s="7" t="str">
+        <f t="shared" ref="F30:G30" si="27">E30</f>
+        <v>Strava</v>
+      </c>
+      <c r="G30" s="7" t="str">
+        <f t="shared" si="27"/>
+        <v>Strava</v>
+      </c>
+      <c r="H30" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8">
       <c r="A31" s="6">
         <v>46200</v>
       </c>
       <c r="B31" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C31" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D31" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E31" t="s">
-        <v>38</v>
-      </c>
-      <c r="F31" s="4" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6">
+        <v>37</v>
+      </c>
+      <c r="F31" s="7" t="str">
+        <f t="shared" ref="F31:G31" si="28">E31</f>
+        <v>Por definir</v>
+      </c>
+      <c r="G31" s="7" t="str">
+        <f t="shared" si="28"/>
+        <v>Por definir</v>
+      </c>
+      <c r="H31" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8">
       <c r="A32" s="6">
         <v>46201</v>
       </c>
       <c r="B32" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C32" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D32" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E32" t="s">
-        <v>38</v>
-      </c>
-      <c r="F32" s="4" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6">
+        <v>37</v>
+      </c>
+      <c r="F32" s="7" t="str">
+        <f t="shared" ref="F32:G32" si="29">E32</f>
+        <v>Por definir</v>
+      </c>
+      <c r="G32" s="7" t="str">
+        <f t="shared" si="29"/>
+        <v>Por definir</v>
+      </c>
+      <c r="H32" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8">
       <c r="A33" s="6">
         <v>46202</v>
       </c>
       <c r="B33" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C33" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D33" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E33" t="s">
-        <v>38</v>
-      </c>
-      <c r="F33" s="4" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6">
+        <v>37</v>
+      </c>
+      <c r="F33" s="7" t="str">
+        <f t="shared" ref="F33:G33" si="30">E33</f>
+        <v>Por definir</v>
+      </c>
+      <c r="G33" s="7" t="str">
+        <f t="shared" si="30"/>
+        <v>Por definir</v>
+      </c>
+      <c r="H33" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8">
       <c r="A34" s="6">
         <v>46207</v>
       </c>
       <c r="B34" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C34" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D34" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E34" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F34" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6">
+        <v>36</v>
+      </c>
+      <c r="F34" s="7" t="str">
+        <f t="shared" ref="F34:G34" si="31">E34</f>
+        <v>Strava</v>
+      </c>
+      <c r="G34" s="7" t="str">
+        <f t="shared" si="31"/>
+        <v>Strava</v>
+      </c>
+      <c r="H34" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8">
       <c r="A35" s="6">
         <v>46214</v>
       </c>
       <c r="B35" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C35" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D35" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E35" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F35" s="4" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6">
+        <v>36</v>
+      </c>
+      <c r="F35" s="7" t="str">
+        <f t="shared" ref="F35:G35" si="32">E35</f>
+        <v>Strava</v>
+      </c>
+      <c r="G35" s="7" t="str">
+        <f t="shared" si="32"/>
+        <v>Strava</v>
+      </c>
+      <c r="H35" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8">
       <c r="A36" s="6">
         <v>46207</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C36" s="3" t="s">
+        <v>357</v>
+      </c>
+      <c r="D36" s="3" t="s">
         <v>358</v>
       </c>
-      <c r="D36" s="3" t="s">
-        <v>359</v>
-      </c>
       <c r="E36" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F36" s="3" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6">
+        <v>36</v>
+      </c>
+      <c r="F36" s="7" t="str">
+        <f t="shared" ref="F36:G36" si="33">E36</f>
+        <v>Strava</v>
+      </c>
+      <c r="G36" s="7" t="str">
+        <f t="shared" si="33"/>
+        <v>Strava</v>
+      </c>
+      <c r="H36" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8">
       <c r="A37" s="6">
         <v>46214</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C37" s="29" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E37" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F37" s="29" t="s">
-        <v>363</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6">
+        <v>36</v>
+      </c>
+      <c r="F37" s="7" t="str">
+        <f t="shared" ref="F37:G37" si="34">E37</f>
+        <v>Strava</v>
+      </c>
+      <c r="G37" s="7" t="str">
+        <f t="shared" si="34"/>
+        <v>Strava</v>
+      </c>
+      <c r="H37" s="29" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8">
       <c r="A38" s="6">
         <v>46221</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D38" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E38" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F38" s="4" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6">
+        <v>36</v>
+      </c>
+      <c r="F38" s="7" t="str">
+        <f t="shared" ref="F38:G38" si="35">E38</f>
+        <v>Strava</v>
+      </c>
+      <c r="G38" s="7" t="str">
+        <f t="shared" si="35"/>
+        <v>Strava</v>
+      </c>
+      <c r="H38" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8">
       <c r="A39" s="6">
         <v>46228</v>
       </c>
       <c r="B39" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C39" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D39" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E39" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F39" s="4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6">
+        <v>36</v>
+      </c>
+      <c r="F39" s="7" t="str">
+        <f t="shared" ref="F39:G39" si="36">E39</f>
+        <v>Strava</v>
+      </c>
+      <c r="G39" s="7" t="str">
+        <f t="shared" si="36"/>
+        <v>Strava</v>
+      </c>
+      <c r="H39" s="4" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8">
       <c r="A40" s="6">
         <v>46235</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="E40" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F40" s="3" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6">
+        <v>36</v>
+      </c>
+      <c r="F40" s="7" t="str">
+        <f t="shared" ref="F40:G40" si="37">E40</f>
+        <v>Strava</v>
+      </c>
+      <c r="G40" s="7" t="str">
+        <f t="shared" si="37"/>
+        <v>Strava</v>
+      </c>
+      <c r="H40" s="3" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8">
       <c r="A41" s="6">
         <v>46242</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E41" t="s">
-        <v>38</v>
-      </c>
-      <c r="F41" s="4" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6">
+        <v>37</v>
+      </c>
+      <c r="F41" s="7" t="str">
+        <f t="shared" ref="F41:G41" si="38">E41</f>
+        <v>Por definir</v>
+      </c>
+      <c r="G41" s="7" t="str">
+        <f t="shared" si="38"/>
+        <v>Por definir</v>
+      </c>
+      <c r="H41" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8">
       <c r="A42" s="6">
         <v>46249</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D42" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E42" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F42" s="4" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6">
+        <v>36</v>
+      </c>
+      <c r="F42" s="7" t="str">
+        <f t="shared" ref="F42:G42" si="39">E42</f>
+        <v>Strava</v>
+      </c>
+      <c r="G42" s="7" t="str">
+        <f t="shared" si="39"/>
+        <v>Strava</v>
+      </c>
+      <c r="H42" s="4" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8">
       <c r="A43" s="6">
         <v>46256</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="E43" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F43" s="3" t="s">
-        <v>362</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6">
+        <v>36</v>
+      </c>
+      <c r="F43" s="7" t="str">
+        <f t="shared" ref="F43:G43" si="40">E43</f>
+        <v>Strava</v>
+      </c>
+      <c r="G43" s="7" t="str">
+        <f t="shared" si="40"/>
+        <v>Strava</v>
+      </c>
+      <c r="H43" s="3" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8">
       <c r="A44" s="6">
         <v>46263</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C44" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D44" t="s">
+        <v>35</v>
+      </c>
+      <c r="E44" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="E44" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F44" s="4" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6">
+      <c r="F44" s="7" t="str">
+        <f t="shared" ref="F44:G44" si="41">E44</f>
+        <v>Strava</v>
+      </c>
+      <c r="G44" s="7" t="str">
+        <f t="shared" si="41"/>
+        <v>Strava</v>
+      </c>
+      <c r="H44" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8">
       <c r="A45" s="6">
         <v>46270</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C45" s="29" t="s">
+        <v>372</v>
+      </c>
+      <c r="D45" s="3" t="s">
         <v>373</v>
       </c>
-      <c r="D45" s="3" t="s">
-        <v>374</v>
-      </c>
       <c r="E45" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F45" s="29" t="s">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6">
+        <v>36</v>
+      </c>
+      <c r="F45" s="7" t="str">
+        <f t="shared" ref="F45:G45" si="42">E45</f>
+        <v>Strava</v>
+      </c>
+      <c r="G45" s="7" t="str">
+        <f t="shared" si="42"/>
+        <v>Strava</v>
+      </c>
+      <c r="H45" s="29" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8">
       <c r="A46" s="6">
         <v>46277</v>
       </c>
       <c r="B46" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D46" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E46" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F46" s="4" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6">
+        <v>36</v>
+      </c>
+      <c r="F46" s="7" t="str">
+        <f t="shared" ref="F46:G46" si="43">E46</f>
+        <v>Strava</v>
+      </c>
+      <c r="G46" s="7" t="str">
+        <f t="shared" si="43"/>
+        <v>Strava</v>
+      </c>
+      <c r="H46" s="4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8">
       <c r="A47" s="6">
         <v>46284</v>
       </c>
       <c r="B47" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C47" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D47" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E47" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F47" s="4" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6">
+        <v>36</v>
+      </c>
+      <c r="F47" s="7" t="str">
+        <f t="shared" ref="F47:G47" si="44">E47</f>
+        <v>Strava</v>
+      </c>
+      <c r="G47" s="7" t="str">
+        <f t="shared" si="44"/>
+        <v>Strava</v>
+      </c>
+      <c r="H47" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8">
       <c r="A48" s="6">
         <v>46291</v>
       </c>
       <c r="B48" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C48" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D48" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E48" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F48" s="4" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6">
+        <v>36</v>
+      </c>
+      <c r="F48" s="7" t="str">
+        <f t="shared" ref="F48:G48" si="45">E48</f>
+        <v>Strava</v>
+      </c>
+      <c r="G48" s="7" t="str">
+        <f t="shared" si="45"/>
+        <v>Strava</v>
+      </c>
+      <c r="H48" s="4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8">
       <c r="A49" s="6">
         <v>46298</v>
       </c>
       <c r="B49" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C49" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="D49" s="28" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E49" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F49" t="s">
-        <v>372</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6">
+        <v>36</v>
+      </c>
+      <c r="F49" s="7" t="str">
+        <f t="shared" ref="F49:G49" si="46">E49</f>
+        <v>Strava</v>
+      </c>
+      <c r="G49" s="7" t="str">
+        <f t="shared" si="46"/>
+        <v>Strava</v>
+      </c>
+      <c r="H49" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8">
       <c r="A50" s="6">
         <v>46304</v>
       </c>
       <c r="B50" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C50" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="D50" s="28" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E50" t="s">
-        <v>38</v>
-      </c>
-      <c r="F50" s="4" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6">
+        <v>37</v>
+      </c>
+      <c r="F50" s="7" t="str">
+        <f t="shared" ref="F50:G50" si="47">E50</f>
+        <v>Por definir</v>
+      </c>
+      <c r="G50" s="7" t="str">
+        <f t="shared" si="47"/>
+        <v>Por definir</v>
+      </c>
+      <c r="H50" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8">
       <c r="A51" s="6">
         <v>46305</v>
       </c>
       <c r="B51" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C51" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="D51" s="28" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E51" t="s">
-        <v>38</v>
-      </c>
-      <c r="F51" s="4" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6">
+        <v>37</v>
+      </c>
+      <c r="F51" s="7" t="str">
+        <f t="shared" ref="F51:G51" si="48">E51</f>
+        <v>Por definir</v>
+      </c>
+      <c r="G51" s="7" t="str">
+        <f t="shared" si="48"/>
+        <v>Por definir</v>
+      </c>
+      <c r="H51" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8">
       <c r="A52" s="6">
         <v>46306</v>
       </c>
       <c r="B52" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C52" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="D52" s="28" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E52" t="s">
-        <v>38</v>
-      </c>
-      <c r="F52" s="4" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6">
+        <v>37</v>
+      </c>
+      <c r="F52" s="7" t="str">
+        <f t="shared" ref="F52:G52" si="49">E52</f>
+        <v>Por definir</v>
+      </c>
+      <c r="G52" s="7" t="str">
+        <f t="shared" si="49"/>
+        <v>Por definir</v>
+      </c>
+      <c r="H52" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8">
       <c r="A53" s="6">
         <v>46308</v>
       </c>
       <c r="B53" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C53" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="D53" s="28" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E53" t="s">
-        <v>38</v>
-      </c>
-      <c r="F53" s="4" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6">
+        <v>37</v>
+      </c>
+      <c r="F53" s="7" t="str">
+        <f t="shared" ref="F53:G53" si="50">E53</f>
+        <v>Por definir</v>
+      </c>
+      <c r="G53" s="7" t="str">
+        <f t="shared" si="50"/>
+        <v>Por definir</v>
+      </c>
+      <c r="H53" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8">
       <c r="A54" s="6">
         <v>46305</v>
       </c>
       <c r="B54" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C54" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D54" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E54" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F54" s="4" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6">
+        <v>36</v>
+      </c>
+      <c r="F54" s="7" t="str">
+        <f t="shared" ref="F54:G54" si="51">E54</f>
+        <v>Strava</v>
+      </c>
+      <c r="G54" s="7" t="str">
+        <f t="shared" si="51"/>
+        <v>Strava</v>
+      </c>
+      <c r="H54" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8">
       <c r="A55" s="6">
         <v>46312</v>
       </c>
       <c r="B55" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C55" t="s">
+        <v>315</v>
+      </c>
+      <c r="D55" t="s">
+        <v>317</v>
+      </c>
+      <c r="E55" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="F55" s="7" t="str">
+        <f t="shared" ref="F55:G55" si="52">E55</f>
+        <v>Strava</v>
+      </c>
+      <c r="G55" s="7" t="str">
+        <f t="shared" si="52"/>
+        <v>Strava</v>
+      </c>
+      <c r="H55" s="4" t="s">
         <v>316</v>
       </c>
-      <c r="D55" t="s">
-        <v>318</v>
-      </c>
-      <c r="E55" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F55" s="4" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6">
+    </row>
+    <row r="56" spans="1:8">
       <c r="A56" s="6">
         <v>46319</v>
       </c>
       <c r="B56" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C56" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D56" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E56" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F56" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6">
+        <v>36</v>
+      </c>
+      <c r="F56" s="7" t="str">
+        <f t="shared" ref="F56:G56" si="53">E56</f>
+        <v>Strava</v>
+      </c>
+      <c r="G56" s="7" t="str">
+        <f t="shared" si="53"/>
+        <v>Strava</v>
+      </c>
+      <c r="H56" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8">
       <c r="A57" s="6">
         <v>46326</v>
       </c>
       <c r="B57" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C57" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D57" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="E57" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F57" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6">
+        <v>36</v>
+      </c>
+      <c r="F57" s="7" t="str">
+        <f t="shared" ref="F57:G57" si="54">E57</f>
+        <v>Strava</v>
+      </c>
+      <c r="G57" s="7" t="str">
+        <f t="shared" si="54"/>
+        <v>Strava</v>
+      </c>
+      <c r="H57" s="4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8">
       <c r="A58" s="6">
         <v>46333</v>
       </c>
       <c r="B58" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C58" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D58" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E58" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F58" s="4" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6">
+        <v>36</v>
+      </c>
+      <c r="F58" s="7" t="str">
+        <f t="shared" ref="F58:G58" si="55">E58</f>
+        <v>Strava</v>
+      </c>
+      <c r="G58" s="7" t="str">
+        <f t="shared" si="55"/>
+        <v>Strava</v>
+      </c>
+      <c r="H58" s="4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8">
       <c r="A59" s="6">
         <v>46340</v>
       </c>
       <c r="B59" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C59" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D59" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E59" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F59" s="4" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6">
+        <v>36</v>
+      </c>
+      <c r="F59" s="7" t="str">
+        <f t="shared" ref="F59:G59" si="56">E59</f>
+        <v>Strava</v>
+      </c>
+      <c r="G59" s="7" t="str">
+        <f t="shared" si="56"/>
+        <v>Strava</v>
+      </c>
+      <c r="H59" s="4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8">
       <c r="A60" s="6">
         <v>46347</v>
       </c>
       <c r="B60" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C60" t="s">
+        <v>355</v>
+      </c>
+      <c r="D60" t="s">
         <v>356</v>
       </c>
-      <c r="D60" t="s">
-        <v>357</v>
-      </c>
       <c r="E60" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F60" s="4" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6">
+        <v>36</v>
+      </c>
+      <c r="F60" s="7" t="str">
+        <f t="shared" ref="F60:G60" si="57">E60</f>
+        <v>Strava</v>
+      </c>
+      <c r="G60" s="7" t="str">
+        <f t="shared" si="57"/>
+        <v>Strava</v>
+      </c>
+      <c r="H60" s="4" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8">
       <c r="A61" s="6">
         <v>46354</v>
       </c>
       <c r="B61" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C61" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="D61" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="E61" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F61" t="s">
-        <v>366</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6">
+        <v>36</v>
+      </c>
+      <c r="F61" s="7" t="str">
+        <f t="shared" ref="F61:G61" si="58">E61</f>
+        <v>Strava</v>
+      </c>
+      <c r="G61" s="7" t="str">
+        <f t="shared" si="58"/>
+        <v>Strava</v>
+      </c>
+      <c r="H61" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8">
       <c r="A62" s="6">
         <v>46361</v>
       </c>
       <c r="B62" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C62" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="D62" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E62" t="s">
-        <v>38</v>
-      </c>
-      <c r="F62" s="4" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6">
+        <v>37</v>
+      </c>
+      <c r="F62" s="7" t="str">
+        <f t="shared" ref="F62:G62" si="59">E62</f>
+        <v>Por definir</v>
+      </c>
+      <c r="G62" s="7" t="str">
+        <f t="shared" si="59"/>
+        <v>Por definir</v>
+      </c>
+      <c r="H62" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8">
       <c r="A63" s="6">
         <v>46362</v>
       </c>
       <c r="B63" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C63" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="D63" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E63" t="s">
-        <v>38</v>
-      </c>
-      <c r="F63" s="4" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6">
+        <v>37</v>
+      </c>
+      <c r="F63" s="7" t="str">
+        <f t="shared" ref="F63:G63" si="60">E63</f>
+        <v>Por definir</v>
+      </c>
+      <c r="G63" s="7" t="str">
+        <f t="shared" si="60"/>
+        <v>Por definir</v>
+      </c>
+      <c r="H63" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8">
       <c r="A64" s="6">
         <v>46363</v>
       </c>
       <c r="B64" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C64" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="D64" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E64" t="s">
-        <v>38</v>
-      </c>
-      <c r="F64" s="4" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6">
+        <v>37</v>
+      </c>
+      <c r="F64" s="7" t="str">
+        <f t="shared" ref="F64:G64" si="61">E64</f>
+        <v>Por definir</v>
+      </c>
+      <c r="G64" s="7" t="str">
+        <f t="shared" si="61"/>
+        <v>Por definir</v>
+      </c>
+      <c r="H64" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8">
       <c r="A65" s="6">
         <v>46361</v>
       </c>
       <c r="B65" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C65" s="29" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="D65" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E65" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F65" s="29" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6">
+        <v>36</v>
+      </c>
+      <c r="F65" s="7" t="str">
+        <f t="shared" ref="F65:G65" si="62">E65</f>
+        <v>Strava</v>
+      </c>
+      <c r="G65" s="7" t="str">
+        <f t="shared" si="62"/>
+        <v>Strava</v>
+      </c>
+      <c r="H65" s="29" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8">
       <c r="A66" s="6">
         <v>46368</v>
       </c>
       <c r="B66" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C66" s="29" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="D66" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E66" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F66" s="29" t="s">
-        <v>371</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6">
+        <v>36</v>
+      </c>
+      <c r="F66" s="7" t="str">
+        <f t="shared" ref="F66:G66" si="63">E66</f>
+        <v>Strava</v>
+      </c>
+      <c r="G66" s="7" t="str">
+        <f t="shared" si="63"/>
+        <v>Strava</v>
+      </c>
+      <c r="H66" s="29" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8">
       <c r="A67" s="6">
         <v>46375</v>
       </c>
       <c r="B67" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C67" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D67" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E67" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F67" s="4" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6">
+        <v>36</v>
+      </c>
+      <c r="F67" s="7" t="str">
+        <f t="shared" ref="F67:G67" si="64">E67</f>
+        <v>Strava</v>
+      </c>
+      <c r="G67" s="7" t="str">
+        <f t="shared" si="64"/>
+        <v>Strava</v>
+      </c>
+      <c r="H67" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8">
       <c r="A68" s="6">
         <v>46382</v>
       </c>
       <c r="B68" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C68" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D68" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E68" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F68" s="2" t="s">
-        <v>50</v>
+        <v>36</v>
+      </c>
+      <c r="F68" s="7" t="str">
+        <f t="shared" ref="F68:G68" si="65">E68</f>
+        <v>Strava</v>
+      </c>
+      <c r="G68" s="7" t="str">
+        <f t="shared" si="65"/>
+        <v>Strava</v>
+      </c>
+      <c r="H68" s="2" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -3121,19 +3669,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="B1" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="C1" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="D1" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="E1" s="13" t="s">
         <v>75</v>
-      </c>
-      <c r="E1" s="13" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -3141,16 +3689,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="C2" s="16" t="s">
         <v>77</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="D2" s="16" t="s">
         <v>78</v>
       </c>
-      <c r="D2" s="16" t="s">
+      <c r="E2" s="17" t="s">
         <v>79</v>
-      </c>
-      <c r="E2" s="17" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -3158,16 +3706,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C3" s="16" t="s">
+        <v>80</v>
+      </c>
+      <c r="D3" s="16" t="s">
         <v>81</v>
       </c>
-      <c r="D3" s="16" t="s">
+      <c r="E3" s="17" t="s">
         <v>82</v>
-      </c>
-      <c r="E3" s="17" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -3175,16 +3723,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C4" s="16" t="s">
+        <v>83</v>
+      </c>
+      <c r="D4" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="D4" s="18" t="s">
+      <c r="E4" s="18" t="s">
         <v>85</v>
-      </c>
-      <c r="E4" s="18" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -3192,16 +3740,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C5" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="D5" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="D5" s="18" t="s">
+      <c r="E5" s="18" t="s">
         <v>88</v>
-      </c>
-      <c r="E5" s="18" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -3209,16 +3757,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C6" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="D6" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="E6" s="18" t="s">
         <v>91</v>
-      </c>
-      <c r="E6" s="18" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -3226,16 +3774,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C7" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="D7" s="16" t="s">
         <v>93</v>
       </c>
-      <c r="D7" s="16" t="s">
+      <c r="E7" s="16" t="s">
         <v>94</v>
-      </c>
-      <c r="E7" s="16" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -3243,16 +3791,16 @@
         <v>7</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C8" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="D8" s="16" t="s">
         <v>96</v>
       </c>
-      <c r="D8" s="16" t="s">
+      <c r="E8" s="17" t="s">
         <v>97</v>
-      </c>
-      <c r="E8" s="17" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -3260,16 +3808,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C9" s="16" t="s">
+        <v>98</v>
+      </c>
+      <c r="D9" s="16" t="s">
         <v>99</v>
       </c>
-      <c r="D9" s="16" t="s">
+      <c r="E9" s="17" t="s">
         <v>100</v>
-      </c>
-      <c r="E9" s="17" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -3277,16 +3825,16 @@
         <v>9</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C10" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="D10" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="D10" s="18" t="s">
+      <c r="E10" s="18" t="s">
         <v>103</v>
-      </c>
-      <c r="E10" s="18" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -3294,16 +3842,16 @@
         <v>10</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C11" s="16" t="s">
+        <v>104</v>
+      </c>
+      <c r="D11" s="18" t="s">
         <v>105</v>
       </c>
-      <c r="D11" s="18" t="s">
+      <c r="E11" s="18" t="s">
         <v>106</v>
-      </c>
-      <c r="E11" s="18" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -3311,16 +3859,16 @@
         <v>11</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C12" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="D12" s="16" t="s">
         <v>108</v>
       </c>
-      <c r="D12" s="16" t="s">
+      <c r="E12" s="17" t="s">
         <v>109</v>
-      </c>
-      <c r="E12" s="17" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -3328,16 +3876,16 @@
         <v>12</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C13" s="16" t="s">
+        <v>110</v>
+      </c>
+      <c r="D13" s="16" t="s">
         <v>111</v>
       </c>
-      <c r="D13" s="16" t="s">
-        <v>112</v>
-      </c>
       <c r="E13" s="17" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -3345,16 +3893,16 @@
         <v>13</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C14" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="D14" s="16" t="s">
         <v>113</v>
       </c>
-      <c r="D14" s="16" t="s">
+      <c r="E14" s="17" t="s">
         <v>114</v>
-      </c>
-      <c r="E14" s="17" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -3362,16 +3910,16 @@
         <v>14</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C15" s="16" t="s">
+        <v>115</v>
+      </c>
+      <c r="D15" s="16" t="s">
         <v>116</v>
       </c>
-      <c r="D15" s="16" t="s">
+      <c r="E15" s="17" t="s">
         <v>117</v>
-      </c>
-      <c r="E15" s="17" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -3379,16 +3927,16 @@
         <v>15</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C16" s="16" t="s">
+        <v>118</v>
+      </c>
+      <c r="D16" s="16" t="s">
         <v>119</v>
       </c>
-      <c r="D16" s="16" t="s">
+      <c r="E16" s="17" t="s">
         <v>120</v>
-      </c>
-      <c r="E16" s="17" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -3396,16 +3944,16 @@
         <v>16</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C17" s="16" t="s">
+        <v>121</v>
+      </c>
+      <c r="D17" s="16" t="s">
         <v>122</v>
       </c>
-      <c r="D17" s="16" t="s">
+      <c r="E17" s="17" t="s">
         <v>123</v>
-      </c>
-      <c r="E17" s="17" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -3413,16 +3961,16 @@
         <v>17</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C18" s="16" t="s">
+        <v>124</v>
+      </c>
+      <c r="D18" s="16" t="s">
         <v>125</v>
       </c>
-      <c r="D18" s="16" t="s">
+      <c r="E18" s="17" t="s">
         <v>126</v>
-      </c>
-      <c r="E18" s="17" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -3430,16 +3978,16 @@
         <v>18</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C19" s="16" t="s">
+        <v>127</v>
+      </c>
+      <c r="D19" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="D19" s="16" t="s">
-        <v>129</v>
-      </c>
       <c r="E19" s="17" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -3447,16 +3995,16 @@
         <v>19</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C20" s="16" t="s">
+        <v>129</v>
+      </c>
+      <c r="D20" s="16" t="s">
         <v>130</v>
       </c>
-      <c r="D20" s="16" t="s">
+      <c r="E20" s="17" t="s">
         <v>131</v>
-      </c>
-      <c r="E20" s="17" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -3464,16 +4012,16 @@
         <v>20</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C21" s="16" t="s">
+        <v>132</v>
+      </c>
+      <c r="D21" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="D21" s="18" t="s">
+      <c r="E21" s="18" t="s">
         <v>134</v>
-      </c>
-      <c r="E21" s="18" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -3481,16 +4029,16 @@
         <v>21</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C22" s="16" t="s">
+        <v>135</v>
+      </c>
+      <c r="D22" s="18" t="s">
         <v>136</v>
       </c>
-      <c r="D22" s="18" t="s">
+      <c r="E22" s="18" t="s">
         <v>137</v>
-      </c>
-      <c r="E22" s="18" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -3498,16 +4046,16 @@
         <v>22</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C23" s="16" t="s">
+        <v>138</v>
+      </c>
+      <c r="D23" s="16" t="s">
         <v>139</v>
       </c>
-      <c r="D23" s="16" t="s">
+      <c r="E23" s="17" t="s">
         <v>140</v>
-      </c>
-      <c r="E23" s="17" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -3515,16 +4063,16 @@
         <v>23</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C24" s="16" t="s">
+        <v>141</v>
+      </c>
+      <c r="D24" s="16" t="s">
         <v>142</v>
       </c>
-      <c r="D24" s="16" t="s">
+      <c r="E24" s="17" t="s">
         <v>143</v>
-      </c>
-      <c r="E24" s="17" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -3532,16 +4080,16 @@
         <v>24</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C25" s="16" t="s">
+        <v>144</v>
+      </c>
+      <c r="D25" s="16" t="s">
         <v>145</v>
       </c>
-      <c r="D25" s="16" t="s">
+      <c r="E25" s="17" t="s">
         <v>146</v>
-      </c>
-      <c r="E25" s="17" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -3549,16 +4097,16 @@
         <v>25</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C26" s="16" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D26" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="E26" s="18" t="s">
         <v>148</v>
-      </c>
-      <c r="E26" s="18" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -3566,16 +4114,16 @@
         <v>26</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C27" s="16" t="s">
+        <v>149</v>
+      </c>
+      <c r="D27" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="D27" s="16" t="s">
+      <c r="E27" s="17" t="s">
         <v>151</v>
-      </c>
-      <c r="E27" s="17" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -3583,16 +4131,16 @@
         <v>27</v>
       </c>
       <c r="B28" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C28" s="16" t="s">
+        <v>152</v>
+      </c>
+      <c r="D28" s="16" t="s">
         <v>153</v>
       </c>
-      <c r="D28" s="16" t="s">
+      <c r="E28" s="17" t="s">
         <v>154</v>
-      </c>
-      <c r="E28" s="17" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -3600,16 +4148,16 @@
         <v>28</v>
       </c>
       <c r="B29" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C29" s="16" t="s">
+        <v>155</v>
+      </c>
+      <c r="D29" s="16" t="s">
         <v>156</v>
       </c>
-      <c r="D29" s="16" t="s">
+      <c r="E29" s="17" t="s">
         <v>157</v>
-      </c>
-      <c r="E29" s="17" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="30" spans="1:5">
@@ -3617,16 +4165,16 @@
         <v>29</v>
       </c>
       <c r="B30" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C30" s="16" t="s">
+        <v>158</v>
+      </c>
+      <c r="D30" s="18" t="s">
         <v>159</v>
       </c>
-      <c r="D30" s="18" t="s">
+      <c r="E30" s="18" t="s">
         <v>160</v>
-      </c>
-      <c r="E30" s="18" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="31" spans="1:5">
@@ -3634,16 +4182,16 @@
         <v>30</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C31" s="16" t="s">
+        <v>161</v>
+      </c>
+      <c r="D31" s="16" t="s">
         <v>162</v>
       </c>
-      <c r="D31" s="16" t="s">
+      <c r="E31" s="17" t="s">
         <v>163</v>
-      </c>
-      <c r="E31" s="17" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="32" spans="1:5">
@@ -3651,16 +4199,16 @@
         <v>31</v>
       </c>
       <c r="B32" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C32" s="16" t="s">
+        <v>164</v>
+      </c>
+      <c r="D32" s="16" t="s">
         <v>165</v>
       </c>
-      <c r="D32" s="16" t="s">
+      <c r="E32" s="17" t="s">
         <v>166</v>
-      </c>
-      <c r="E32" s="17" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="33" spans="1:5">
@@ -3668,16 +4216,16 @@
         <v>32</v>
       </c>
       <c r="B33" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C33" s="16" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D33" s="16" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E33" s="17" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="34" spans="1:5">
@@ -3685,16 +4233,16 @@
         <v>33</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="D34" s="16" t="s">
+        <v>168</v>
+      </c>
+      <c r="E34" s="17" t="s">
         <v>169</v>
-      </c>
-      <c r="E34" s="17" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="35" spans="1:5">
@@ -3702,16 +4250,16 @@
         <v>34</v>
       </c>
       <c r="B35" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C35" s="16" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="D35" s="16" t="s">
+        <v>170</v>
+      </c>
+      <c r="E35" s="17" t="s">
         <v>171</v>
-      </c>
-      <c r="E35" s="17" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="36" spans="1:5">
@@ -3719,16 +4267,16 @@
         <v>35</v>
       </c>
       <c r="B36" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C36" s="16" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D36" s="16" t="s">
+        <v>172</v>
+      </c>
+      <c r="E36" s="17" t="s">
         <v>173</v>
-      </c>
-      <c r="E36" s="17" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="37" spans="1:5">
@@ -3736,16 +4284,16 @@
         <v>36</v>
       </c>
       <c r="B37" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C37" s="16" t="s">
+        <v>174</v>
+      </c>
+      <c r="D37" s="16" t="s">
         <v>175</v>
       </c>
-      <c r="D37" s="16" t="s">
+      <c r="E37" s="17" t="s">
         <v>176</v>
-      </c>
-      <c r="E37" s="17" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="38" spans="1:5">
@@ -3753,16 +4301,16 @@
         <v>37</v>
       </c>
       <c r="B38" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C38" s="16" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="D38" s="16" t="s">
+        <v>177</v>
+      </c>
+      <c r="E38" s="17" t="s">
         <v>178</v>
-      </c>
-      <c r="E38" s="17" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="39" spans="1:5">
@@ -3770,16 +4318,16 @@
         <v>38</v>
       </c>
       <c r="B39" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C39" s="16" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="D39" s="16" t="s">
+        <v>179</v>
+      </c>
+      <c r="E39" s="17" t="s">
         <v>180</v>
-      </c>
-      <c r="E39" s="17" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="40" spans="1:5">
@@ -3787,16 +4335,16 @@
         <v>39</v>
       </c>
       <c r="B40" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C40" s="16" t="s">
+        <v>181</v>
+      </c>
+      <c r="D40" s="16" t="s">
         <v>182</v>
       </c>
-      <c r="D40" s="16" t="s">
+      <c r="E40" s="17" t="s">
         <v>183</v>
-      </c>
-      <c r="E40" s="17" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="41" spans="1:5">
@@ -3804,16 +4352,16 @@
         <v>40</v>
       </c>
       <c r="B41" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C41" s="20" t="s">
+        <v>184</v>
+      </c>
+      <c r="D41" s="16" t="s">
         <v>185</v>
       </c>
-      <c r="D41" s="16" t="s">
+      <c r="E41" s="17" t="s">
         <v>186</v>
-      </c>
-      <c r="E41" s="17" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="42" spans="1:5">
@@ -3821,16 +4369,16 @@
         <v>41</v>
       </c>
       <c r="B42" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C42" s="16" t="s">
+        <v>187</v>
+      </c>
+      <c r="D42" s="18" t="s">
+        <v>172</v>
+      </c>
+      <c r="E42" s="18" t="s">
         <v>188</v>
-      </c>
-      <c r="D42" s="18" t="s">
-        <v>173</v>
-      </c>
-      <c r="E42" s="18" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="43" spans="1:5">
@@ -3838,16 +4386,16 @@
         <v>42</v>
       </c>
       <c r="B43" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C43" s="16" t="s">
+        <v>189</v>
+      </c>
+      <c r="D43" s="18" t="s">
         <v>190</v>
       </c>
-      <c r="D43" s="18" t="s">
+      <c r="E43" s="18" t="s">
         <v>191</v>
-      </c>
-      <c r="E43" s="18" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="44" spans="1:5">
@@ -3855,16 +4403,16 @@
         <v>43</v>
       </c>
       <c r="B44" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="D44" s="16" t="s">
+        <v>192</v>
+      </c>
+      <c r="E44" s="17" t="s">
         <v>193</v>
-      </c>
-      <c r="E44" s="17" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="45" spans="1:5">
@@ -3872,16 +4420,16 @@
         <v>44</v>
       </c>
       <c r="B45" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C45" s="16" t="s">
+        <v>194</v>
+      </c>
+      <c r="D45" s="18" t="s">
         <v>195</v>
       </c>
-      <c r="D45" s="18" t="s">
+      <c r="E45" s="18" t="s">
         <v>196</v>
-      </c>
-      <c r="E45" s="18" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="46" spans="1:5">
@@ -3889,16 +4437,16 @@
         <v>45</v>
       </c>
       <c r="B46" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C46" s="19" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="D46" s="16" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E46" s="17" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="47" spans="1:5">
@@ -3906,16 +4454,16 @@
         <v>46</v>
       </c>
       <c r="B47" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C47" s="16" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D47" s="16" t="s">
+        <v>198</v>
+      </c>
+      <c r="E47" s="17" t="s">
         <v>199</v>
-      </c>
-      <c r="E47" s="17" t="s">
-        <v>200</v>
       </c>
     </row>
     <row r="48" spans="1:5">
@@ -3923,16 +4471,16 @@
         <v>47</v>
       </c>
       <c r="B48" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C48" s="16" t="s">
+        <v>200</v>
+      </c>
+      <c r="D48" s="16" t="s">
         <v>201</v>
       </c>
-      <c r="D48" s="16" t="s">
+      <c r="E48" s="17" t="s">
         <v>202</v>
-      </c>
-      <c r="E48" s="17" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="49" spans="1:5">
@@ -3940,16 +4488,16 @@
         <v>48</v>
       </c>
       <c r="B49" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C49" s="16" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D49" s="16" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E49" s="17" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="50" spans="1:5">
@@ -3957,16 +4505,16 @@
         <v>49</v>
       </c>
       <c r="B50" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C50" s="16" t="s">
+        <v>204</v>
+      </c>
+      <c r="D50" s="18" t="s">
+        <v>96</v>
+      </c>
+      <c r="E50" s="18" t="s">
         <v>205</v>
-      </c>
-      <c r="D50" s="18" t="s">
-        <v>97</v>
-      </c>
-      <c r="E50" s="18" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="51" spans="1:5">
@@ -3974,16 +4522,16 @@
         <v>50</v>
       </c>
       <c r="B51" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C51" s="16" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D51" s="16" t="s">
+        <v>206</v>
+      </c>
+      <c r="E51" s="17" t="s">
         <v>207</v>
-      </c>
-      <c r="E51" s="17" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="52" spans="1:5">
@@ -3991,16 +4539,16 @@
         <v>51</v>
       </c>
       <c r="B52" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C52" s="16" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D52" s="16" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E52" s="17" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="53" spans="1:5">
@@ -4008,16 +4556,16 @@
         <v>52</v>
       </c>
       <c r="B53" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C53" s="16" t="s">
+        <v>209</v>
+      </c>
+      <c r="D53" s="16" t="s">
         <v>210</v>
       </c>
-      <c r="D53" s="16" t="s">
+      <c r="E53" s="17" t="s">
         <v>211</v>
-      </c>
-      <c r="E53" s="17" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="54" spans="1:5">
@@ -4025,16 +4573,16 @@
         <v>53</v>
       </c>
       <c r="B54" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C54" s="16" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D54" s="16" t="s">
+        <v>212</v>
+      </c>
+      <c r="E54" s="17" t="s">
         <v>213</v>
-      </c>
-      <c r="E54" s="17" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="55" spans="1:5">
@@ -4042,16 +4590,16 @@
         <v>54</v>
       </c>
       <c r="B55" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C55" s="16" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="D55" s="16" t="s">
+        <v>214</v>
+      </c>
+      <c r="E55" s="17" t="s">
         <v>215</v>
-      </c>
-      <c r="E55" s="17" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="56" spans="1:5">
@@ -4059,16 +4607,16 @@
         <v>55</v>
       </c>
       <c r="B56" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C56" s="16" t="s">
+        <v>216</v>
+      </c>
+      <c r="D56" s="18" t="s">
         <v>217</v>
       </c>
-      <c r="D56" s="18" t="s">
+      <c r="E56" s="18" t="s">
         <v>218</v>
-      </c>
-      <c r="E56" s="18" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="57" spans="1:5">
@@ -4076,16 +4624,16 @@
         <v>56</v>
       </c>
       <c r="B57" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C57" s="16" t="s">
+        <v>219</v>
+      </c>
+      <c r="D57" s="18" t="s">
         <v>220</v>
       </c>
-      <c r="D57" s="18" t="s">
+      <c r="E57" s="18" t="s">
         <v>221</v>
-      </c>
-      <c r="E57" s="18" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="58" spans="1:5">
@@ -4093,16 +4641,16 @@
         <v>57</v>
       </c>
       <c r="B58" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C58" s="16" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D58" s="16" t="s">
+        <v>222</v>
+      </c>
+      <c r="E58" s="17" t="s">
         <v>223</v>
-      </c>
-      <c r="E58" s="17" t="s">
-        <v>224</v>
       </c>
     </row>
     <row r="59" spans="1:5">
@@ -4110,16 +4658,16 @@
         <v>58</v>
       </c>
       <c r="B59" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C59" s="16" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="D59" s="18" t="s">
+        <v>224</v>
+      </c>
+      <c r="E59" s="18" t="s">
         <v>225</v>
-      </c>
-      <c r="E59" s="18" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="60" spans="1:5">
@@ -4127,16 +4675,16 @@
         <v>59</v>
       </c>
       <c r="B60" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C60" s="16" t="s">
+        <v>226</v>
+      </c>
+      <c r="D60" s="16" t="s">
         <v>227</v>
       </c>
-      <c r="D60" s="16" t="s">
+      <c r="E60" s="17" t="s">
         <v>228</v>
-      </c>
-      <c r="E60" s="17" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="61" spans="1:5">
@@ -4144,16 +4692,16 @@
         <v>60</v>
       </c>
       <c r="B61" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C61" s="16" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="D61" s="16" t="s">
+        <v>229</v>
+      </c>
+      <c r="E61" s="17" t="s">
         <v>230</v>
-      </c>
-      <c r="E61" s="17" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="62" spans="1:5">
@@ -4161,16 +4709,16 @@
         <v>61</v>
       </c>
       <c r="B62" s="18" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C62" s="16" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="D62" s="16" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E62" s="17" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="63" spans="1:5">
@@ -4178,16 +4726,16 @@
         <v>62</v>
       </c>
       <c r="B63" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C63" s="16" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="D63" s="16" t="s">
+        <v>232</v>
+      </c>
+      <c r="E63" s="17" t="s">
         <v>233</v>
-      </c>
-      <c r="E63" s="17" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="64" spans="1:5">
@@ -4195,16 +4743,16 @@
         <v>63</v>
       </c>
       <c r="B64" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C64" s="16" t="s">
+        <v>234</v>
+      </c>
+      <c r="D64" s="16" t="s">
         <v>235</v>
       </c>
-      <c r="D64" s="16" t="s">
+      <c r="E64" s="17" t="s">
         <v>236</v>
-      </c>
-      <c r="E64" s="17" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="65" spans="1:5">
@@ -4212,16 +4760,16 @@
         <v>64</v>
       </c>
       <c r="B65" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C65" s="16" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="D65" s="16" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E65" s="17" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="66" spans="1:5">
@@ -4229,16 +4777,16 @@
         <v>65</v>
       </c>
       <c r="B66" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C66" s="16" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D66" s="16" t="s">
+        <v>238</v>
+      </c>
+      <c r="E66" s="17" t="s">
         <v>239</v>
-      </c>
-      <c r="E66" s="17" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="67" spans="1:5">
@@ -4246,16 +4794,16 @@
         <v>66</v>
       </c>
       <c r="B67" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C67" s="16" t="s">
+        <v>240</v>
+      </c>
+      <c r="D67" s="16" t="s">
         <v>241</v>
       </c>
-      <c r="D67" s="16" t="s">
+      <c r="E67" s="17" t="s">
         <v>242</v>
-      </c>
-      <c r="E67" s="17" t="s">
-        <v>243</v>
       </c>
     </row>
     <row r="68" spans="1:5">
@@ -4263,16 +4811,16 @@
         <v>67</v>
       </c>
       <c r="B68" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C68" s="16" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="D68" s="16" t="s">
+        <v>243</v>
+      </c>
+      <c r="E68" s="17" t="s">
         <v>244</v>
-      </c>
-      <c r="E68" s="17" t="s">
-        <v>245</v>
       </c>
     </row>
     <row r="69" spans="1:5">
@@ -4280,16 +4828,16 @@
         <v>68</v>
       </c>
       <c r="B69" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C69" s="16" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="D69" s="16" t="s">
+        <v>245</v>
+      </c>
+      <c r="E69" s="17" t="s">
         <v>246</v>
-      </c>
-      <c r="E69" s="17" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="70" spans="1:5">
@@ -4297,16 +4845,16 @@
         <v>69</v>
       </c>
       <c r="B70" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C70" s="16" t="s">
+        <v>247</v>
+      </c>
+      <c r="D70" s="18" t="s">
         <v>248</v>
       </c>
-      <c r="D70" s="18" t="s">
+      <c r="E70" s="18" t="s">
         <v>249</v>
-      </c>
-      <c r="E70" s="18" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="71" spans="1:5">
@@ -4314,16 +4862,16 @@
         <v>70</v>
       </c>
       <c r="B71" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C71" s="16" t="s">
+        <v>250</v>
+      </c>
+      <c r="D71" s="16" t="s">
         <v>251</v>
       </c>
-      <c r="D71" s="16" t="s">
+      <c r="E71" s="17" t="s">
         <v>252</v>
-      </c>
-      <c r="E71" s="17" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="72" spans="1:5">
@@ -4331,16 +4879,16 @@
         <v>71</v>
       </c>
       <c r="B72" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C72" s="16" t="s">
+        <v>253</v>
+      </c>
+      <c r="D72" s="18" t="s">
         <v>254</v>
       </c>
-      <c r="D72" s="18" t="s">
+      <c r="E72" s="18" t="s">
         <v>255</v>
-      </c>
-      <c r="E72" s="18" t="s">
-        <v>256</v>
       </c>
     </row>
     <row r="73" spans="1:5">
@@ -4348,16 +4896,16 @@
         <v>72</v>
       </c>
       <c r="B73" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C73" s="16" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="D73" s="16" t="s">
+        <v>256</v>
+      </c>
+      <c r="E73" s="17" t="s">
         <v>257</v>
-      </c>
-      <c r="E73" s="17" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="74" spans="1:5">
@@ -4365,16 +4913,16 @@
         <v>73</v>
       </c>
       <c r="B74" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C74" s="16" t="s">
+        <v>258</v>
+      </c>
+      <c r="D74" s="16" t="s">
         <v>259</v>
       </c>
-      <c r="D74" s="16" t="s">
+      <c r="E74" s="17" t="s">
         <v>260</v>
-      </c>
-      <c r="E74" s="17" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="75" spans="1:5">
@@ -4382,16 +4930,16 @@
         <v>74</v>
       </c>
       <c r="B75" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C75" s="16" t="s">
+        <v>261</v>
+      </c>
+      <c r="D75" s="18" t="s">
+        <v>111</v>
+      </c>
+      <c r="E75" s="18" t="s">
         <v>262</v>
-      </c>
-      <c r="D75" s="18" t="s">
-        <v>112</v>
-      </c>
-      <c r="E75" s="18" t="s">
-        <v>263</v>
       </c>
     </row>
     <row r="76" spans="1:5">
@@ -4399,16 +4947,16 @@
         <v>75</v>
       </c>
       <c r="B76" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C76" s="16" t="s">
+        <v>263</v>
+      </c>
+      <c r="D76" s="18" t="s">
         <v>264</v>
       </c>
-      <c r="D76" s="18" t="s">
+      <c r="E76" s="18" t="s">
         <v>265</v>
-      </c>
-      <c r="E76" s="18" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="77" spans="1:5">
@@ -4416,16 +4964,16 @@
         <v>76</v>
       </c>
       <c r="B77" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C77" s="16" t="s">
+        <v>266</v>
+      </c>
+      <c r="D77" s="18" t="s">
         <v>267</v>
       </c>
-      <c r="D77" s="18" t="s">
+      <c r="E77" s="18" t="s">
         <v>268</v>
-      </c>
-      <c r="E77" s="18" t="s">
-        <v>269</v>
       </c>
     </row>
     <row r="78" spans="1:5">
@@ -4433,16 +4981,16 @@
         <v>77</v>
       </c>
       <c r="B78" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C78" s="16" t="s">
+        <v>269</v>
+      </c>
+      <c r="D78" s="18" t="s">
         <v>270</v>
       </c>
-      <c r="D78" s="18" t="s">
+      <c r="E78" s="18" t="s">
         <v>271</v>
-      </c>
-      <c r="E78" s="18" t="s">
-        <v>272</v>
       </c>
     </row>
     <row r="79" spans="1:5">
@@ -4450,16 +4998,16 @@
         <v>78</v>
       </c>
       <c r="B79" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C79" s="16" t="s">
+        <v>272</v>
+      </c>
+      <c r="D79" s="16" t="s">
+        <v>251</v>
+      </c>
+      <c r="E79" s="17" t="s">
         <v>273</v>
-      </c>
-      <c r="D79" s="16" t="s">
-        <v>252</v>
-      </c>
-      <c r="E79" s="17" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="80" spans="1:5">
@@ -4467,16 +5015,16 @@
         <v>79</v>
       </c>
       <c r="B80" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C80" s="16" t="s">
+        <v>274</v>
+      </c>
+      <c r="D80" s="18" t="s">
         <v>275</v>
       </c>
-      <c r="D80" s="18" t="s">
+      <c r="E80" s="18" t="s">
         <v>276</v>
-      </c>
-      <c r="E80" s="18" t="s">
-        <v>277</v>
       </c>
     </row>
     <row r="81" spans="1:5">
@@ -4484,16 +5032,16 @@
         <v>80</v>
       </c>
       <c r="B81" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C81" s="16" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="D81" s="16" t="s">
+        <v>277</v>
+      </c>
+      <c r="E81" s="17" t="s">
         <v>278</v>
-      </c>
-      <c r="E81" s="17" t="s">
-        <v>279</v>
       </c>
     </row>
     <row r="82" spans="1:5">
@@ -4501,16 +5049,16 @@
         <v>81</v>
       </c>
       <c r="B82" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C82" s="16" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="D82" s="16" t="s">
+        <v>279</v>
+      </c>
+      <c r="E82" s="17" t="s">
         <v>280</v>
-      </c>
-      <c r="E82" s="17" t="s">
-        <v>281</v>
       </c>
     </row>
     <row r="83" spans="1:5">
@@ -4518,16 +5066,16 @@
         <v>82</v>
       </c>
       <c r="B83" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C83" s="16" t="s">
+        <v>281</v>
+      </c>
+      <c r="D83" s="16" t="s">
         <v>282</v>
       </c>
-      <c r="D83" s="16" t="s">
+      <c r="E83" s="17" t="s">
         <v>283</v>
-      </c>
-      <c r="E83" s="17" t="s">
-        <v>284</v>
       </c>
     </row>
     <row r="84" spans="1:5">
@@ -4535,16 +5083,16 @@
         <v>83</v>
       </c>
       <c r="B84" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C84" s="16" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="D84" s="16" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="E84" s="17" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="85" spans="1:5">
@@ -4552,16 +5100,16 @@
         <v>84</v>
       </c>
       <c r="B85" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C85" s="16" t="s">
+        <v>285</v>
+      </c>
+      <c r="D85" s="16" t="s">
         <v>286</v>
       </c>
-      <c r="D85" s="16" t="s">
+      <c r="E85" s="17" t="s">
         <v>287</v>
-      </c>
-      <c r="E85" s="17" t="s">
-        <v>288</v>
       </c>
     </row>
     <row r="86" spans="1:5">
@@ -4569,16 +5117,16 @@
         <v>85</v>
       </c>
       <c r="B86" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C86" s="16" t="s">
+        <v>288</v>
+      </c>
+      <c r="D86" s="16" t="s">
+        <v>277</v>
+      </c>
+      <c r="E86" s="17" t="s">
         <v>289</v>
-      </c>
-      <c r="D86" s="16" t="s">
-        <v>278</v>
-      </c>
-      <c r="E86" s="17" t="s">
-        <v>290</v>
       </c>
     </row>
     <row r="87" spans="1:5">
@@ -4586,16 +5134,16 @@
         <v>86</v>
       </c>
       <c r="B87" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C87" s="16" t="s">
+        <v>290</v>
+      </c>
+      <c r="D87" s="16" t="s">
         <v>291</v>
       </c>
-      <c r="D87" s="16" t="s">
+      <c r="E87" s="17" t="s">
         <v>292</v>
-      </c>
-      <c r="E87" s="17" t="s">
-        <v>293</v>
       </c>
     </row>
     <row r="88" spans="1:5">
@@ -4603,16 +5151,16 @@
         <v>87</v>
       </c>
       <c r="B88" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C88" s="16" t="s">
+        <v>293</v>
+      </c>
+      <c r="D88" s="16" t="s">
+        <v>279</v>
+      </c>
+      <c r="E88" s="17" t="s">
         <v>294</v>
-      </c>
-      <c r="D88" s="16" t="s">
-        <v>280</v>
-      </c>
-      <c r="E88" s="17" t="s">
-        <v>295</v>
       </c>
     </row>
     <row r="89" spans="1:5">
@@ -4620,16 +5168,16 @@
         <v>88</v>
       </c>
       <c r="B89" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C89" s="16" t="s">
+        <v>295</v>
+      </c>
+      <c r="D89" s="16" t="s">
+        <v>96</v>
+      </c>
+      <c r="E89" s="17" t="s">
         <v>296</v>
-      </c>
-      <c r="D89" s="16" t="s">
-        <v>97</v>
-      </c>
-      <c r="E89" s="17" t="s">
-        <v>297</v>
       </c>
     </row>
     <row r="90" spans="1:5">
@@ -4637,16 +5185,16 @@
         <v>89</v>
       </c>
       <c r="B90" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C90" s="16" t="s">
+        <v>297</v>
+      </c>
+      <c r="D90" s="16" t="s">
         <v>298</v>
       </c>
-      <c r="D90" s="16" t="s">
+      <c r="E90" s="17" t="s">
         <v>299</v>
-      </c>
-      <c r="E90" s="17" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="91" spans="1:5">
@@ -4654,16 +5202,16 @@
         <v>90</v>
       </c>
       <c r="B91" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C91" s="16" t="s">
+        <v>300</v>
+      </c>
+      <c r="D91" s="16" t="s">
         <v>301</v>
       </c>
-      <c r="D91" s="16" t="s">
+      <c r="E91" s="17" t="s">
         <v>302</v>
-      </c>
-      <c r="E91" s="17" t="s">
-        <v>303</v>
       </c>
     </row>
     <row r="92" spans="1:5">
@@ -4671,16 +5219,16 @@
         <v>91</v>
       </c>
       <c r="B92" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C92" s="16" t="s">
+        <v>303</v>
+      </c>
+      <c r="D92" s="16" t="s">
         <v>304</v>
       </c>
-      <c r="D92" s="16" t="s">
+      <c r="E92" s="17" t="s">
         <v>305</v>
-      </c>
-      <c r="E92" s="17" t="s">
-        <v>306</v>
       </c>
     </row>
     <row r="93" spans="1:5">
@@ -4688,16 +5236,16 @@
         <v>92</v>
       </c>
       <c r="B93" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C93" s="16" t="s">
+        <v>306</v>
+      </c>
+      <c r="D93" s="16" t="s">
+        <v>182</v>
+      </c>
+      <c r="E93" s="17" t="s">
         <v>307</v>
-      </c>
-      <c r="D93" s="16" t="s">
-        <v>183</v>
-      </c>
-      <c r="E93" s="17" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="94" spans="1:5">
@@ -4705,16 +5253,16 @@
         <v>93</v>
       </c>
       <c r="B94" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C94" s="16" t="s">
+        <v>308</v>
+      </c>
+      <c r="D94" s="18" t="s">
         <v>309</v>
       </c>
-      <c r="D94" s="18" t="s">
+      <c r="E94" s="18" t="s">
         <v>310</v>
-      </c>
-      <c r="E94" s="18" t="s">
-        <v>311</v>
       </c>
     </row>
     <row r="95" spans="1:5">
@@ -4722,16 +5270,16 @@
         <v>94</v>
       </c>
       <c r="B95" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C95" s="25" t="s">
+        <v>321</v>
+      </c>
+      <c r="D95" s="23" t="s">
         <v>322</v>
       </c>
-      <c r="D95" s="23" t="s">
+      <c r="E95" s="23" t="s">
         <v>323</v>
-      </c>
-      <c r="E95" s="23" t="s">
-        <v>324</v>
       </c>
     </row>
     <row r="96" spans="1:5">
@@ -4740,16 +5288,16 @@
         <v>95</v>
       </c>
       <c r="B96" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C96" s="26" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="D96" s="27" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E96" s="27" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="97" spans="1:5">
@@ -4758,16 +5306,16 @@
         <v>96</v>
       </c>
       <c r="B97" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C97" s="22" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="D97" s="23" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E97" s="23" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="98" spans="1:5">
@@ -4776,16 +5324,16 @@
         <v>97</v>
       </c>
       <c r="B98" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C98" s="22" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D98" s="23" t="s">
+        <v>318</v>
+      </c>
+      <c r="E98" s="23" t="s">
         <v>319</v>
-      </c>
-      <c r="E98" s="23" t="s">
-        <v>320</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
actualiza calendario desde Excel (67 -> 63 rutas)
- 2 nuevas (Lo Prado - Cuesta Ibacache Bis 05/09, Giro Zapallar 10/10)
- 6 quitadas (Enjoy Los Andes a Zapallar, bloque Criterium Ruta de las Estrellas,
  Mc Chamisero - Til Til - Cumbre La Dormida Bis)
- regenera datos y reporte (GPX no encontrados: 0, 97 usuarios)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Template_Calendario_CCS_GPX.xlsx
+++ b/Template_Calendario_CCS_GPX.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cesarmora/Library/Mobile Documents/com~apple~CloudDocs/Personal/Ciclismo/Calendario/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A23A874-A946-6244-AD08-7401901FEE09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFFBE002-7076-234F-866B-5CDE89A1DC5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="30240" windowHeight="17780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template_Calendario_CCS" sheetId="1" r:id="rId1"/>
     <sheet name="Usuarios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Template_Calendario_CCS!$A$1:$M$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Template_Calendario_CCS!$A$1:$M$64</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="741" uniqueCount="378">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="721" uniqueCount="376">
   <si>
     <t>Fecha</t>
   </si>
@@ -1128,9 +1128,6 @@
     <t>Aurora - Cuesta Barriga - Cuesta Mallarauco - Chorombo</t>
   </si>
   <si>
-    <t>Criterium Ruta de las Estrellas</t>
-  </si>
-  <si>
     <t>Kross - Pangue - Casa Blanca - Cuesta Zapata - Kross</t>
   </si>
   <si>
@@ -1155,12 +1152,6 @@
     <t>Vizcachas - Toyo - Lagunillas</t>
   </si>
   <si>
-    <t>Enjoy Los Andes a Zapallar</t>
-  </si>
-  <si>
-    <t>Enjoy</t>
-  </si>
-  <si>
     <t>Aurora - Chorombo Alto - Mallarauco - Barriga - Aurora</t>
   </si>
   <si>
@@ -1171,6 +1162,9 @@
   </si>
   <si>
     <t>C</t>
+  </si>
+  <si>
+    <t>Giro Zapallar</t>
   </si>
 </sst>
 </file>
@@ -1662,8 +1656,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M68"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <dimension ref="A1:M64"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="14" style="6" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -1692,13 +1686,13 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>4</v>
@@ -2430,7 +2424,7 @@
         <v>22</v>
       </c>
       <c r="D27" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="E27" s="7" t="s">
         <v>36</v>
@@ -2699,7 +2693,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="37" spans="1:8">
+    <row r="37" spans="1:8" ht="15">
       <c r="A37" s="6">
         <v>46214</v>
       </c>
@@ -2794,7 +2788,7 @@
         <v>359</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="E40" s="7" t="s">
         <v>36</v>
@@ -2878,7 +2872,7 @@
         <v>361</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="E43" s="7" t="s">
         <v>36</v>
@@ -2912,7 +2906,7 @@
         <v>36</v>
       </c>
       <c r="F44" s="7" t="str">
-        <f t="shared" ref="F44:G44" si="41">E44</f>
+        <f t="shared" ref="F44:G45" si="41">E44</f>
         <v>Strava</v>
       </c>
       <c r="G44" s="7" t="str">
@@ -2927,28 +2921,28 @@
       <c r="A45" s="6">
         <v>46270</v>
       </c>
-      <c r="B45" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C45" s="29" t="s">
-        <v>372</v>
-      </c>
-      <c r="D45" s="3" t="s">
-        <v>373</v>
+      <c r="B45" t="s">
+        <v>5</v>
+      </c>
+      <c r="C45" t="s">
+        <v>22</v>
+      </c>
+      <c r="D45" t="s">
+        <v>367</v>
       </c>
       <c r="E45" s="7" t="s">
         <v>36</v>
       </c>
       <c r="F45" s="7" t="str">
-        <f t="shared" ref="F45:G45" si="42">E45</f>
+        <f t="shared" si="41"/>
         <v>Strava</v>
       </c>
       <c r="G45" s="7" t="str">
-        <f t="shared" si="42"/>
-        <v>Strava</v>
-      </c>
-      <c r="H45" s="29" t="s">
-        <v>372</v>
+        <f t="shared" si="41"/>
+        <v>Strava</v>
+      </c>
+      <c r="H45" s="4" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="46" spans="1:8">
@@ -2968,11 +2962,11 @@
         <v>36</v>
       </c>
       <c r="F46" s="7" t="str">
-        <f t="shared" ref="F46:G46" si="43">E46</f>
+        <f t="shared" ref="F46:G46" si="42">E46</f>
         <v>Strava</v>
       </c>
       <c r="G46" s="7" t="str">
-        <f t="shared" si="43"/>
+        <f t="shared" si="42"/>
         <v>Strava</v>
       </c>
       <c r="H46" s="4" t="s">
@@ -2996,11 +2990,11 @@
         <v>36</v>
       </c>
       <c r="F47" s="7" t="str">
-        <f t="shared" ref="F47:G47" si="44">E47</f>
+        <f t="shared" ref="F47:G47" si="43">E47</f>
         <v>Strava</v>
       </c>
       <c r="G47" s="7" t="str">
-        <f t="shared" si="44"/>
+        <f t="shared" si="43"/>
         <v>Strava</v>
       </c>
       <c r="H47" s="4" t="s">
@@ -3024,11 +3018,11 @@
         <v>36</v>
       </c>
       <c r="F48" s="7" t="str">
-        <f t="shared" ref="F48:G48" si="45">E48</f>
+        <f t="shared" ref="F48:G48" si="44">E48</f>
         <v>Strava</v>
       </c>
       <c r="G48" s="7" t="str">
-        <f t="shared" si="45"/>
+        <f t="shared" si="44"/>
         <v>Strava</v>
       </c>
       <c r="H48" s="4" t="s">
@@ -3043,7 +3037,7 @@
         <v>5</v>
       </c>
       <c r="C49" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="D49" s="28" t="s">
         <v>29</v>
@@ -3052,39 +3046,39 @@
         <v>36</v>
       </c>
       <c r="F49" s="7" t="str">
-        <f t="shared" ref="F49:G49" si="46">E49</f>
+        <f t="shared" ref="F49:G50" si="45">E49</f>
         <v>Strava</v>
       </c>
       <c r="G49" s="7" t="str">
-        <f t="shared" si="46"/>
+        <f t="shared" si="45"/>
         <v>Strava</v>
       </c>
       <c r="H49" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="50" spans="1:8">
       <c r="A50" s="6">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B50" t="s">
         <v>6</v>
       </c>
       <c r="C50" t="s">
-        <v>363</v>
-      </c>
-      <c r="D50" s="28" t="s">
+        <v>375</v>
+      </c>
+      <c r="D50" t="s">
         <v>70</v>
       </c>
       <c r="E50" t="s">
         <v>37</v>
       </c>
       <c r="F50" s="7" t="str">
-        <f t="shared" ref="F50:G50" si="47">E50</f>
+        <f t="shared" si="45"/>
         <v>Por definir</v>
       </c>
       <c r="G50" s="7" t="str">
-        <f t="shared" si="47"/>
+        <f t="shared" si="45"/>
         <v>Por definir</v>
       </c>
       <c r="H50" s="4" t="s">
@@ -3093,505 +3087,393 @@
     </row>
     <row r="51" spans="1:8">
       <c r="A51" s="6">
-        <v>46305</v>
+        <v>46312</v>
       </c>
       <c r="B51" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C51" t="s">
-        <v>363</v>
-      </c>
-      <c r="D51" s="28" t="s">
-        <v>70</v>
-      </c>
-      <c r="E51" t="s">
-        <v>37</v>
+        <v>315</v>
+      </c>
+      <c r="D51" t="s">
+        <v>317</v>
+      </c>
+      <c r="E51" s="7" t="s">
+        <v>36</v>
       </c>
       <c r="F51" s="7" t="str">
-        <f t="shared" ref="F51:G51" si="48">E51</f>
-        <v>Por definir</v>
+        <f t="shared" ref="F51:G51" si="46">E51</f>
+        <v>Strava</v>
       </c>
       <c r="G51" s="7" t="str">
-        <f t="shared" si="48"/>
-        <v>Por definir</v>
+        <f t="shared" si="46"/>
+        <v>Strava</v>
       </c>
       <c r="H51" s="4" t="s">
-        <v>70</v>
+        <v>316</v>
       </c>
     </row>
     <row r="52" spans="1:8">
       <c r="A52" s="6">
-        <v>46306</v>
+        <v>46319</v>
       </c>
       <c r="B52" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C52" t="s">
         <v>363</v>
       </c>
-      <c r="D52" s="28" t="s">
-        <v>70</v>
-      </c>
-      <c r="E52" t="s">
-        <v>37</v>
+      <c r="D52" t="s">
+        <v>28</v>
+      </c>
+      <c r="E52" s="7" t="s">
+        <v>36</v>
       </c>
       <c r="F52" s="7" t="str">
-        <f t="shared" ref="F52:G52" si="49">E52</f>
-        <v>Por definir</v>
+        <f t="shared" ref="F52:G52" si="47">E52</f>
+        <v>Strava</v>
       </c>
       <c r="G52" s="7" t="str">
-        <f t="shared" si="49"/>
-        <v>Por definir</v>
-      </c>
-      <c r="H52" s="4" t="s">
-        <v>70</v>
+        <f t="shared" si="47"/>
+        <v>Strava</v>
+      </c>
+      <c r="H52" t="s">
+        <v>363</v>
       </c>
     </row>
     <row r="53" spans="1:8">
       <c r="A53" s="6">
-        <v>46308</v>
+        <v>46326</v>
       </c>
       <c r="B53" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C53" t="s">
-        <v>363</v>
-      </c>
-      <c r="D53" s="28" t="s">
-        <v>70</v>
-      </c>
-      <c r="E53" t="s">
-        <v>37</v>
+        <v>22</v>
+      </c>
+      <c r="D53" t="s">
+        <v>367</v>
+      </c>
+      <c r="E53" s="7" t="s">
+        <v>36</v>
       </c>
       <c r="F53" s="7" t="str">
-        <f t="shared" ref="F53:G53" si="50">E53</f>
-        <v>Por definir</v>
+        <f t="shared" ref="F53:G53" si="48">E53</f>
+        <v>Strava</v>
       </c>
       <c r="G53" s="7" t="str">
-        <f t="shared" si="50"/>
-        <v>Por definir</v>
+        <f t="shared" si="48"/>
+        <v>Strava</v>
       </c>
       <c r="H53" s="4" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
     </row>
     <row r="54" spans="1:8">
       <c r="A54" s="6">
-        <v>46305</v>
+        <v>46333</v>
       </c>
       <c r="B54" t="s">
-        <v>369</v>
+        <v>6</v>
       </c>
       <c r="C54" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D54" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E54" s="7" t="s">
         <v>36</v>
       </c>
       <c r="F54" s="7" t="str">
-        <f t="shared" ref="F54:G54" si="51">E54</f>
+        <f t="shared" ref="F54:G54" si="49">E54</f>
         <v>Strava</v>
       </c>
       <c r="G54" s="7" t="str">
-        <f t="shared" si="51"/>
+        <f t="shared" si="49"/>
         <v>Strava</v>
       </c>
       <c r="H54" s="4" t="s">
-        <v>43</v>
+        <v>62</v>
       </c>
     </row>
     <row r="55" spans="1:8">
       <c r="A55" s="6">
-        <v>46312</v>
+        <v>46340</v>
       </c>
       <c r="B55" t="s">
         <v>5</v>
       </c>
       <c r="C55" t="s">
-        <v>315</v>
+        <v>23</v>
       </c>
       <c r="D55" t="s">
-        <v>317</v>
+        <v>30</v>
       </c>
       <c r="E55" s="7" t="s">
         <v>36</v>
       </c>
       <c r="F55" s="7" t="str">
-        <f t="shared" ref="F55:G55" si="52">E55</f>
+        <f t="shared" ref="F55:G55" si="50">E55</f>
         <v>Strava</v>
       </c>
       <c r="G55" s="7" t="str">
-        <f t="shared" si="52"/>
+        <f t="shared" si="50"/>
         <v>Strava</v>
       </c>
       <c r="H55" s="4" t="s">
-        <v>316</v>
+        <v>67</v>
       </c>
     </row>
     <row r="56" spans="1:8">
       <c r="A56" s="6">
-        <v>46319</v>
+        <v>46347</v>
       </c>
       <c r="B56" t="s">
         <v>5</v>
       </c>
       <c r="C56" t="s">
-        <v>364</v>
+        <v>355</v>
       </c>
       <c r="D56" t="s">
-        <v>28</v>
+        <v>356</v>
       </c>
       <c r="E56" s="7" t="s">
         <v>36</v>
       </c>
       <c r="F56" s="7" t="str">
-        <f t="shared" ref="F56:G56" si="53">E56</f>
+        <f t="shared" ref="F56:G56" si="51">E56</f>
         <v>Strava</v>
       </c>
       <c r="G56" s="7" t="str">
-        <f t="shared" si="53"/>
-        <v>Strava</v>
-      </c>
-      <c r="H56" t="s">
-        <v>364</v>
+        <f t="shared" si="51"/>
+        <v>Strava</v>
+      </c>
+      <c r="H56" s="4" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="57" spans="1:8">
       <c r="A57" s="6">
-        <v>46326</v>
+        <v>46354</v>
       </c>
       <c r="B57" t="s">
         <v>5</v>
       </c>
       <c r="C57" t="s">
-        <v>22</v>
+        <v>364</v>
       </c>
       <c r="D57" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="E57" s="7" t="s">
         <v>36</v>
       </c>
       <c r="F57" s="7" t="str">
-        <f t="shared" ref="F57:G57" si="54">E57</f>
+        <f t="shared" ref="F57:G57" si="52">E57</f>
         <v>Strava</v>
       </c>
       <c r="G57" s="7" t="str">
-        <f t="shared" si="54"/>
-        <v>Strava</v>
-      </c>
-      <c r="H57" s="4" t="s">
-        <v>64</v>
+        <f t="shared" si="52"/>
+        <v>Strava</v>
+      </c>
+      <c r="H57" t="s">
+        <v>364</v>
       </c>
     </row>
     <row r="58" spans="1:8">
       <c r="A58" s="6">
-        <v>46333</v>
+        <v>46361</v>
       </c>
       <c r="B58" t="s">
         <v>6</v>
       </c>
       <c r="C58" t="s">
-        <v>18</v>
+        <v>365</v>
       </c>
       <c r="D58" t="s">
-        <v>33</v>
-      </c>
-      <c r="E58" s="7" t="s">
-        <v>36</v>
+        <v>70</v>
+      </c>
+      <c r="E58" t="s">
+        <v>37</v>
       </c>
       <c r="F58" s="7" t="str">
-        <f t="shared" ref="F58:G58" si="55">E58</f>
-        <v>Strava</v>
+        <f t="shared" ref="F58:G58" si="53">E58</f>
+        <v>Por definir</v>
       </c>
       <c r="G58" s="7" t="str">
-        <f t="shared" si="55"/>
-        <v>Strava</v>
+        <f t="shared" si="53"/>
+        <v>Por definir</v>
       </c>
       <c r="H58" s="4" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
     </row>
     <row r="59" spans="1:8">
       <c r="A59" s="6">
-        <v>46340</v>
+        <v>46362</v>
       </c>
       <c r="B59" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C59" t="s">
-        <v>23</v>
+        <v>365</v>
       </c>
       <c r="D59" t="s">
-        <v>30</v>
-      </c>
-      <c r="E59" s="7" t="s">
-        <v>36</v>
+        <v>70</v>
+      </c>
+      <c r="E59" t="s">
+        <v>37</v>
       </c>
       <c r="F59" s="7" t="str">
-        <f t="shared" ref="F59:G59" si="56">E59</f>
-        <v>Strava</v>
+        <f t="shared" ref="F59:G59" si="54">E59</f>
+        <v>Por definir</v>
       </c>
       <c r="G59" s="7" t="str">
-        <f t="shared" si="56"/>
-        <v>Strava</v>
+        <f t="shared" si="54"/>
+        <v>Por definir</v>
       </c>
       <c r="H59" s="4" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="60" spans="1:8">
       <c r="A60" s="6">
-        <v>46347</v>
+        <v>46363</v>
       </c>
       <c r="B60" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C60" t="s">
-        <v>355</v>
+        <v>365</v>
       </c>
       <c r="D60" t="s">
-        <v>356</v>
-      </c>
-      <c r="E60" s="7" t="s">
-        <v>36</v>
+        <v>70</v>
+      </c>
+      <c r="E60" t="s">
+        <v>37</v>
       </c>
       <c r="F60" s="7" t="str">
-        <f t="shared" ref="F60:G60" si="57">E60</f>
-        <v>Strava</v>
+        <f t="shared" ref="F60:G60" si="55">E60</f>
+        <v>Por definir</v>
       </c>
       <c r="G60" s="7" t="str">
-        <f t="shared" si="57"/>
-        <v>Strava</v>
+        <f t="shared" si="55"/>
+        <v>Por definir</v>
       </c>
       <c r="H60" s="4" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="61" spans="1:8">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" ht="15">
       <c r="A61" s="6">
-        <v>46354</v>
+        <v>46361</v>
       </c>
       <c r="B61" t="s">
-        <v>5</v>
-      </c>
-      <c r="C61" t="s">
-        <v>365</v>
+        <v>368</v>
+      </c>
+      <c r="C61" s="29" t="s">
+        <v>371</v>
       </c>
       <c r="D61" t="s">
-        <v>367</v>
+        <v>26</v>
       </c>
       <c r="E61" s="7" t="s">
         <v>36</v>
       </c>
       <c r="F61" s="7" t="str">
-        <f t="shared" ref="F61:G61" si="58">E61</f>
+        <f t="shared" ref="F61:G61" si="56">E61</f>
         <v>Strava</v>
       </c>
       <c r="G61" s="7" t="str">
-        <f t="shared" si="58"/>
-        <v>Strava</v>
-      </c>
-      <c r="H61" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="62" spans="1:8">
+        <f t="shared" si="56"/>
+        <v>Strava</v>
+      </c>
+      <c r="H61" s="29" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" ht="15">
       <c r="A62" s="6">
-        <v>46361</v>
+        <v>46368</v>
       </c>
       <c r="B62" t="s">
-        <v>6</v>
-      </c>
-      <c r="C62" t="s">
-        <v>366</v>
+        <v>5</v>
+      </c>
+      <c r="C62" s="29" t="s">
+        <v>369</v>
       </c>
       <c r="D62" t="s">
-        <v>70</v>
-      </c>
-      <c r="E62" t="s">
-        <v>37</v>
+        <v>29</v>
+      </c>
+      <c r="E62" s="7" t="s">
+        <v>36</v>
       </c>
       <c r="F62" s="7" t="str">
-        <f t="shared" ref="F62:G62" si="59">E62</f>
-        <v>Por definir</v>
+        <f t="shared" ref="F62:G62" si="57">E62</f>
+        <v>Strava</v>
       </c>
       <c r="G62" s="7" t="str">
-        <f t="shared" si="59"/>
-        <v>Por definir</v>
-      </c>
-      <c r="H62" s="4" t="s">
-        <v>70</v>
+        <f t="shared" si="57"/>
+        <v>Strava</v>
+      </c>
+      <c r="H62" s="29" t="s">
+        <v>369</v>
       </c>
     </row>
     <row r="63" spans="1:8">
       <c r="A63" s="6">
-        <v>46362</v>
+        <v>46375</v>
       </c>
       <c r="B63" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C63" t="s">
-        <v>366</v>
+        <v>13</v>
       </c>
       <c r="D63" t="s">
-        <v>70</v>
-      </c>
-      <c r="E63" t="s">
-        <v>37</v>
+        <v>27</v>
+      </c>
+      <c r="E63" s="7" t="s">
+        <v>36</v>
       </c>
       <c r="F63" s="7" t="str">
-        <f t="shared" ref="F63:G63" si="60">E63</f>
-        <v>Por definir</v>
+        <f t="shared" ref="F63:G63" si="58">E63</f>
+        <v>Strava</v>
       </c>
       <c r="G63" s="7" t="str">
-        <f t="shared" si="60"/>
-        <v>Por definir</v>
+        <f t="shared" si="58"/>
+        <v>Strava</v>
       </c>
       <c r="H63" s="4" t="s">
-        <v>70</v>
+        <v>55</v>
       </c>
     </row>
     <row r="64" spans="1:8">
       <c r="A64" s="6">
-        <v>46363</v>
+        <v>46382</v>
       </c>
       <c r="B64" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C64" t="s">
-        <v>366</v>
+        <v>7</v>
       </c>
       <c r="D64" t="s">
-        <v>70</v>
-      </c>
-      <c r="E64" t="s">
-        <v>37</v>
+        <v>26</v>
+      </c>
+      <c r="E64" s="7" t="s">
+        <v>36</v>
       </c>
       <c r="F64" s="7" t="str">
-        <f t="shared" ref="F64:G64" si="61">E64</f>
-        <v>Por definir</v>
+        <f t="shared" ref="F64:G64" si="59">E64</f>
+        <v>Strava</v>
       </c>
       <c r="G64" s="7" t="str">
-        <f t="shared" si="61"/>
-        <v>Por definir</v>
-      </c>
-      <c r="H64" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="65" spans="1:8">
-      <c r="A65" s="6">
-        <v>46361</v>
-      </c>
-      <c r="B65" t="s">
-        <v>369</v>
-      </c>
-      <c r="C65" s="29" t="s">
-        <v>374</v>
-      </c>
-      <c r="D65" t="s">
-        <v>26</v>
-      </c>
-      <c r="E65" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="F65" s="7" t="str">
-        <f t="shared" ref="F65:G65" si="62">E65</f>
-        <v>Strava</v>
-      </c>
-      <c r="G65" s="7" t="str">
-        <f t="shared" si="62"/>
-        <v>Strava</v>
-      </c>
-      <c r="H65" s="29" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="66" spans="1:8">
-      <c r="A66" s="6">
-        <v>46368</v>
-      </c>
-      <c r="B66" t="s">
-        <v>5</v>
-      </c>
-      <c r="C66" s="29" t="s">
-        <v>370</v>
-      </c>
-      <c r="D66" t="s">
-        <v>29</v>
-      </c>
-      <c r="E66" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="F66" s="7" t="str">
-        <f t="shared" ref="F66:G66" si="63">E66</f>
-        <v>Strava</v>
-      </c>
-      <c r="G66" s="7" t="str">
-        <f t="shared" si="63"/>
-        <v>Strava</v>
-      </c>
-      <c r="H66" s="29" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="67" spans="1:8">
-      <c r="A67" s="6">
-        <v>46375</v>
-      </c>
-      <c r="B67" t="s">
-        <v>5</v>
-      </c>
-      <c r="C67" t="s">
-        <v>13</v>
-      </c>
-      <c r="D67" t="s">
-        <v>27</v>
-      </c>
-      <c r="E67" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="F67" s="7" t="str">
-        <f t="shared" ref="F67:G67" si="64">E67</f>
-        <v>Strava</v>
-      </c>
-      <c r="G67" s="7" t="str">
-        <f t="shared" si="64"/>
-        <v>Strava</v>
-      </c>
-      <c r="H67" s="4" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="68" spans="1:8">
-      <c r="A68" s="6">
-        <v>46382</v>
-      </c>
-      <c r="B68" t="s">
-        <v>5</v>
-      </c>
-      <c r="C68" t="s">
-        <v>7</v>
-      </c>
-      <c r="D68" t="s">
-        <v>26</v>
-      </c>
-      <c r="E68" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="F68" s="7" t="str">
-        <f t="shared" ref="F68:G68" si="65">E68</f>
-        <v>Strava</v>
-      </c>
-      <c r="G68" s="7" t="str">
-        <f t="shared" si="65"/>
-        <v>Strava</v>
-      </c>
-      <c r="H68" s="2" t="s">
+        <f t="shared" si="59"/>
+        <v>Strava</v>
+      </c>
+      <c r="H64" s="2" t="s">
         <v>49</v>
       </c>
     </row>
@@ -3625,31 +3507,30 @@
     <hyperlink ref="E20" r:id="rId26" xr:uid="{8866888E-71DF-3944-9620-4E948829D43F}"/>
     <hyperlink ref="E25" r:id="rId27" xr:uid="{F67F5632-1B2B-C049-8C5C-D8F9CF9A87E3}"/>
     <hyperlink ref="E24" r:id="rId28" xr:uid="{F51A13EB-7897-0D42-A463-97945F82F47E}"/>
-    <hyperlink ref="E57" r:id="rId29" xr:uid="{8F50E81C-F18A-CE4F-A98D-3D4F1A293290}"/>
-    <hyperlink ref="E58" r:id="rId30" xr:uid="{B1BBA9B4-EBD6-9343-BDD3-B3D8AA59AD32}"/>
-    <hyperlink ref="E59" r:id="rId31" xr:uid="{BAEB0B98-6FB1-434C-B4D4-0C351FA1E8AA}"/>
-    <hyperlink ref="E60" r:id="rId32" xr:uid="{A1058D29-89CB-8B47-A38D-E24CFFAD7387}"/>
-    <hyperlink ref="E68" r:id="rId33" xr:uid="{0A9781F8-06DF-AD4B-8C0E-450CBD0E1ED5}"/>
+    <hyperlink ref="E53" r:id="rId29" xr:uid="{8F50E81C-F18A-CE4F-A98D-3D4F1A293290}"/>
+    <hyperlink ref="E54" r:id="rId30" xr:uid="{B1BBA9B4-EBD6-9343-BDD3-B3D8AA59AD32}"/>
+    <hyperlink ref="E55" r:id="rId31" xr:uid="{BAEB0B98-6FB1-434C-B4D4-0C351FA1E8AA}"/>
+    <hyperlink ref="E56" r:id="rId32" xr:uid="{A1058D29-89CB-8B47-A38D-E24CFFAD7387}"/>
+    <hyperlink ref="E64" r:id="rId33" xr:uid="{0A9781F8-06DF-AD4B-8C0E-450CBD0E1ED5}"/>
     <hyperlink ref="E39" r:id="rId34" xr:uid="{5D621643-1857-6949-A5EE-8D21ACA6D173}"/>
     <hyperlink ref="E48" r:id="rId35" xr:uid="{28C15F8B-DF41-8E47-BE95-3FF9ADA04A9D}"/>
     <hyperlink ref="E46" r:id="rId36" xr:uid="{050206DA-2A1C-9247-B538-A6C21B74792C}"/>
-    <hyperlink ref="E55" r:id="rId37" xr:uid="{DDF27CF3-067C-2C40-831B-B30E6A059FA4}"/>
+    <hyperlink ref="E51" r:id="rId37" xr:uid="{DDF27CF3-067C-2C40-831B-B30E6A059FA4}"/>
     <hyperlink ref="E42" r:id="rId38" xr:uid="{5FE6AEA5-9829-0A4C-901D-15C508BE82B4}"/>
-    <hyperlink ref="E54" r:id="rId39" xr:uid="{1A25A1F2-21AF-A04A-B17E-17C89C4EB59F}"/>
-    <hyperlink ref="E38" r:id="rId40" xr:uid="{7D056CB1-8218-B047-8B01-6450203D5916}"/>
-    <hyperlink ref="E47" r:id="rId41" xr:uid="{72C58610-12F4-3347-94C5-89094846F7BC}"/>
-    <hyperlink ref="E67" r:id="rId42" xr:uid="{3081F97D-82DE-804B-AF13-E78A89A26914}"/>
-    <hyperlink ref="E49" r:id="rId43" xr:uid="{9AEFB797-EACB-874E-98CC-22F5AB6C6FDF}"/>
-    <hyperlink ref="E44" r:id="rId44" xr:uid="{6DE013C7-DC12-5045-8866-5F063A0E4BBC}"/>
-    <hyperlink ref="E36" r:id="rId45" xr:uid="{8ABC89D8-C10E-0C45-833D-F730BBEC276D}"/>
-    <hyperlink ref="E37" r:id="rId46" xr:uid="{610CEF98-CEDF-3B46-95F5-F415021045BC}"/>
-    <hyperlink ref="E40" r:id="rId47" xr:uid="{2B098DA7-1C63-7346-BDC5-428B06DB46E4}"/>
-    <hyperlink ref="E43" r:id="rId48" xr:uid="{E7F94F05-CCA9-B043-B789-CE3339CC6812}"/>
-    <hyperlink ref="E45" r:id="rId49" xr:uid="{3491218D-359D-1443-8DBA-9498E5017523}"/>
-    <hyperlink ref="E56" r:id="rId50" xr:uid="{C00B5D1B-6D1B-5F46-9E19-728B32AD9191}"/>
-    <hyperlink ref="E61" r:id="rId51" xr:uid="{C923ADC7-05BB-7744-8BF3-B3DF402E49A0}"/>
-    <hyperlink ref="E65" r:id="rId52" xr:uid="{583CF50F-498E-0841-9BC9-5A9E3F837061}"/>
-    <hyperlink ref="E66" r:id="rId53" xr:uid="{030FBD56-AB0C-764C-BC0B-06F85764D9FD}"/>
+    <hyperlink ref="E38" r:id="rId39" xr:uid="{7D056CB1-8218-B047-8B01-6450203D5916}"/>
+    <hyperlink ref="E47" r:id="rId40" xr:uid="{72C58610-12F4-3347-94C5-89094846F7BC}"/>
+    <hyperlink ref="E63" r:id="rId41" xr:uid="{3081F97D-82DE-804B-AF13-E78A89A26914}"/>
+    <hyperlink ref="E49" r:id="rId42" xr:uid="{9AEFB797-EACB-874E-98CC-22F5AB6C6FDF}"/>
+    <hyperlink ref="E44" r:id="rId43" xr:uid="{6DE013C7-DC12-5045-8866-5F063A0E4BBC}"/>
+    <hyperlink ref="E36" r:id="rId44" xr:uid="{8ABC89D8-C10E-0C45-833D-F730BBEC276D}"/>
+    <hyperlink ref="E37" r:id="rId45" xr:uid="{610CEF98-CEDF-3B46-95F5-F415021045BC}"/>
+    <hyperlink ref="E40" r:id="rId46" xr:uid="{2B098DA7-1C63-7346-BDC5-428B06DB46E4}"/>
+    <hyperlink ref="E43" r:id="rId47" xr:uid="{E7F94F05-CCA9-B043-B789-CE3339CC6812}"/>
+    <hyperlink ref="E52" r:id="rId48" xr:uid="{C00B5D1B-6D1B-5F46-9E19-728B32AD9191}"/>
+    <hyperlink ref="E57" r:id="rId49" xr:uid="{C923ADC7-05BB-7744-8BF3-B3DF402E49A0}"/>
+    <hyperlink ref="E61" r:id="rId50" xr:uid="{583CF50F-498E-0841-9BC9-5A9E3F837061}"/>
+    <hyperlink ref="E62" r:id="rId51" xr:uid="{030FBD56-AB0C-764C-BC0B-06F85764D9FD}"/>
+    <hyperlink ref="E45" r:id="rId52" xr:uid="{5BD7D123-7286-5A47-A0D9-8170243675C4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3658,7 +3539,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B1CA8C7-05A5-DA44-B969-9E41B832BB96}">
   <dimension ref="A1:E98"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="7.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.6640625" bestFit="1" customWidth="1"/>

</xml_diff>

<commit_message>
actualiza calendario: links C (Capuccino) en 18 rutas y corrige RUT de socio
- se pegaron los links propios de Strava C en 18 rutas (antes caian a R); M sigue = R
- usuario Rodrigo Martinez: RUT 10.652.669.9 -> 10.652.669-9 (arregla su PIN/login)
- regenera datos y reporte (63 rutas, 97 usuarios, GPX no encontrados: 0)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Template_Calendario_CCS_GPX.xlsx
+++ b/Template_Calendario_CCS_GPX.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cesarmora/Library/Mobile Documents/com~apple~CloudDocs/Personal/Ciclismo/Calendario/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFFBE002-7076-234F-866B-5CDE89A1DC5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{013BB8FF-DD14-E145-98F9-8B8ABA873EEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="30240" windowHeight="17780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,6 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Template_Calendario_CCS!$A$1:$M$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Usuarios!$A$1:$E$98</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="721" uniqueCount="376">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="739" uniqueCount="377">
   <si>
     <t>Fecha</t>
   </si>
@@ -696,9 +697,6 @@
     <t xml:space="preserve">Martin </t>
   </si>
   <si>
-    <t>10.652.669.9</t>
-  </si>
-  <si>
     <t xml:space="preserve">Rodrigo </t>
   </si>
   <si>
@@ -1165,6 +1163,12 @@
   </si>
   <si>
     <t>Giro Zapallar</t>
+  </si>
+  <si>
+    <t>https://www.strava.com/routes/3283543710152062118</t>
+  </si>
+  <si>
+    <t>10.652.669-9</t>
   </si>
 </sst>
 </file>
@@ -1657,11 +1661,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M64"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14" style="6" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="66.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="53.1640625" customWidth="1"/>
     <col min="4" max="4" width="24" customWidth="1"/>
     <col min="5" max="7" width="9.33203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="49.5" bestFit="1" customWidth="1"/>
@@ -1686,13 +1690,13 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>372</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>373</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>374</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>4</v>
@@ -1945,10 +1949,10 @@
         <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="D10" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="E10" s="7" t="s">
         <v>36</v>
@@ -1973,10 +1977,10 @@
         <v>6</v>
       </c>
       <c r="C11" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="D11" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="E11" s="7" t="s">
         <v>36</v>
@@ -2057,7 +2061,7 @@
         <v>5</v>
       </c>
       <c r="C14" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D14" t="s">
         <v>32</v>
@@ -2225,7 +2229,7 @@
         <v>5</v>
       </c>
       <c r="C20" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D20" t="s">
         <v>27</v>
@@ -2242,7 +2246,7 @@
         <v>Strava</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -2365,10 +2369,10 @@
         <v>5</v>
       </c>
       <c r="C25" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="D25" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="E25" s="7" t="s">
         <v>36</v>
@@ -2382,7 +2386,7 @@
         <v>Strava</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -2424,7 +2428,7 @@
         <v>22</v>
       </c>
       <c r="D27" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="E27" s="7" t="s">
         <v>36</v>
@@ -2449,10 +2453,10 @@
         <v>5</v>
       </c>
       <c r="C28" t="s">
+        <v>354</v>
+      </c>
+      <c r="D28" t="s">
         <v>355</v>
-      </c>
-      <c r="D28" t="s">
-        <v>356</v>
       </c>
       <c r="E28" s="7" t="s">
         <v>36</v>
@@ -2673,10 +2677,10 @@
         <v>6</v>
       </c>
       <c r="C36" s="3" t="s">
+        <v>356</v>
+      </c>
+      <c r="D36" s="3" t="s">
         <v>357</v>
-      </c>
-      <c r="D36" s="3" t="s">
-        <v>358</v>
       </c>
       <c r="E36" s="7" t="s">
         <v>36</v>
@@ -2690,10 +2694,10 @@
         <v>Strava</v>
       </c>
       <c r="H36" s="3" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" ht="15">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8">
       <c r="A37" s="6">
         <v>46214</v>
       </c>
@@ -2701,7 +2705,7 @@
         <v>5</v>
       </c>
       <c r="C37" s="29" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="D37" s="3" t="s">
         <v>26</v>
@@ -2718,7 +2722,7 @@
         <v>Strava</v>
       </c>
       <c r="H37" s="29" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="38" spans="1:8">
@@ -2785,24 +2789,23 @@
         <v>5</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="E40" s="7" t="s">
         <v>36</v>
       </c>
       <c r="F40" s="7" t="str">
-        <f t="shared" ref="F40:G40" si="37">E40</f>
-        <v>Strava</v>
-      </c>
-      <c r="G40" s="7" t="str">
-        <f t="shared" si="37"/>
-        <v>Strava</v>
+        <f t="shared" ref="F40" si="37">E40</f>
+        <v>Strava</v>
+      </c>
+      <c r="G40" s="7" t="s">
+        <v>36</v>
       </c>
       <c r="H40" s="3" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
     <row r="41" spans="1:8">
@@ -2813,7 +2816,7 @@
         <v>6</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="D41" s="3" t="s">
         <v>70</v>
@@ -2850,12 +2853,11 @@
         <v>36</v>
       </c>
       <c r="F42" s="7" t="str">
-        <f t="shared" ref="F42:G42" si="39">E42</f>
-        <v>Strava</v>
-      </c>
-      <c r="G42" s="7" t="str">
-        <f t="shared" si="39"/>
-        <v>Strava</v>
+        <f t="shared" ref="F42" si="39">E42</f>
+        <v>Strava</v>
+      </c>
+      <c r="G42" s="7" t="s">
+        <v>36</v>
       </c>
       <c r="H42" s="4" t="s">
         <v>61</v>
@@ -2869,24 +2871,23 @@
         <v>5</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="E43" s="7" t="s">
         <v>36</v>
       </c>
       <c r="F43" s="7" t="str">
-        <f t="shared" ref="F43:G43" si="40">E43</f>
-        <v>Strava</v>
-      </c>
-      <c r="G43" s="7" t="str">
-        <f t="shared" si="40"/>
-        <v>Strava</v>
+        <f t="shared" ref="F43" si="40">E43</f>
+        <v>Strava</v>
+      </c>
+      <c r="G43" s="7" t="s">
+        <v>36</v>
       </c>
       <c r="H43" s="3" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="44" spans="1:8">
@@ -2909,9 +2910,8 @@
         <f t="shared" ref="F44:G45" si="41">E44</f>
         <v>Strava</v>
       </c>
-      <c r="G44" s="7" t="str">
-        <f t="shared" si="41"/>
-        <v>Strava</v>
+      <c r="G44" s="7" t="s">
+        <v>36</v>
       </c>
       <c r="H44" s="4" t="s">
         <v>65</v>
@@ -2928,7 +2928,7 @@
         <v>22</v>
       </c>
       <c r="D45" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="E45" s="7" t="s">
         <v>36</v>
@@ -2962,12 +2962,11 @@
         <v>36</v>
       </c>
       <c r="F46" s="7" t="str">
-        <f t="shared" ref="F46:G46" si="42">E46</f>
-        <v>Strava</v>
-      </c>
-      <c r="G46" s="7" t="str">
-        <f t="shared" si="42"/>
-        <v>Strava</v>
+        <f t="shared" ref="F46" si="42">E46</f>
+        <v>Strava</v>
+      </c>
+      <c r="G46" s="7" t="s">
+        <v>36</v>
       </c>
       <c r="H46" s="4" t="s">
         <v>56</v>
@@ -2990,12 +2989,11 @@
         <v>36</v>
       </c>
       <c r="F47" s="7" t="str">
-        <f t="shared" ref="F47:G47" si="43">E47</f>
-        <v>Strava</v>
-      </c>
-      <c r="G47" s="7" t="str">
-        <f t="shared" si="43"/>
-        <v>Strava</v>
+        <f t="shared" ref="F47" si="43">E47</f>
+        <v>Strava</v>
+      </c>
+      <c r="G47" s="7" t="s">
+        <v>36</v>
       </c>
       <c r="H47" s="4" t="s">
         <v>55</v>
@@ -3018,12 +3016,11 @@
         <v>36</v>
       </c>
       <c r="F48" s="7" t="str">
-        <f t="shared" ref="F48:G48" si="44">E48</f>
-        <v>Strava</v>
-      </c>
-      <c r="G48" s="7" t="str">
-        <f t="shared" si="44"/>
-        <v>Strava</v>
+        <f t="shared" ref="F48" si="44">E48</f>
+        <v>Strava</v>
+      </c>
+      <c r="G48" s="7" t="s">
+        <v>36</v>
       </c>
       <c r="H48" s="4" t="s">
         <v>63</v>
@@ -3037,7 +3034,7 @@
         <v>5</v>
       </c>
       <c r="C49" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="D49" s="28" t="s">
         <v>29</v>
@@ -3049,12 +3046,11 @@
         <f t="shared" ref="F49:G50" si="45">E49</f>
         <v>Strava</v>
       </c>
-      <c r="G49" s="7" t="str">
-        <f t="shared" si="45"/>
-        <v>Strava</v>
+      <c r="G49" s="7" t="s">
+        <v>375</v>
       </c>
       <c r="H49" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="50" spans="1:8">
@@ -3065,7 +3061,7 @@
         <v>6</v>
       </c>
       <c r="C50" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="D50" t="s">
         <v>70</v>
@@ -3093,24 +3089,23 @@
         <v>5</v>
       </c>
       <c r="C51" t="s">
+        <v>314</v>
+      </c>
+      <c r="D51" t="s">
+        <v>316</v>
+      </c>
+      <c r="E51" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="F51" s="7" t="str">
+        <f t="shared" ref="F51" si="46">E51</f>
+        <v>Strava</v>
+      </c>
+      <c r="G51" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="H51" s="4" t="s">
         <v>315</v>
-      </c>
-      <c r="D51" t="s">
-        <v>317</v>
-      </c>
-      <c r="E51" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="F51" s="7" t="str">
-        <f t="shared" ref="F51:G51" si="46">E51</f>
-        <v>Strava</v>
-      </c>
-      <c r="G51" s="7" t="str">
-        <f t="shared" si="46"/>
-        <v>Strava</v>
-      </c>
-      <c r="H51" s="4" t="s">
-        <v>316</v>
       </c>
     </row>
     <row r="52" spans="1:8">
@@ -3121,7 +3116,7 @@
         <v>5</v>
       </c>
       <c r="C52" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D52" t="s">
         <v>28</v>
@@ -3130,15 +3125,14 @@
         <v>36</v>
       </c>
       <c r="F52" s="7" t="str">
-        <f t="shared" ref="F52:G52" si="47">E52</f>
-        <v>Strava</v>
-      </c>
-      <c r="G52" s="7" t="str">
-        <f t="shared" si="47"/>
-        <v>Strava</v>
+        <f t="shared" ref="F52" si="47">E52</f>
+        <v>Strava</v>
+      </c>
+      <c r="G52" s="7" t="s">
+        <v>36</v>
       </c>
       <c r="H52" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="53" spans="1:8">
@@ -3152,18 +3146,17 @@
         <v>22</v>
       </c>
       <c r="D53" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="E53" s="7" t="s">
         <v>36</v>
       </c>
       <c r="F53" s="7" t="str">
-        <f t="shared" ref="F53:G53" si="48">E53</f>
-        <v>Strava</v>
-      </c>
-      <c r="G53" s="7" t="str">
-        <f t="shared" si="48"/>
-        <v>Strava</v>
+        <f t="shared" ref="F53" si="48">E53</f>
+        <v>Strava</v>
+      </c>
+      <c r="G53" s="7" t="s">
+        <v>36</v>
       </c>
       <c r="H53" s="4" t="s">
         <v>64</v>
@@ -3186,12 +3179,11 @@
         <v>36</v>
       </c>
       <c r="F54" s="7" t="str">
-        <f t="shared" ref="F54:G54" si="49">E54</f>
-        <v>Strava</v>
-      </c>
-      <c r="G54" s="7" t="str">
-        <f t="shared" si="49"/>
-        <v>Strava</v>
+        <f t="shared" ref="F54" si="49">E54</f>
+        <v>Strava</v>
+      </c>
+      <c r="G54" s="7" t="s">
+        <v>36</v>
       </c>
       <c r="H54" s="4" t="s">
         <v>62</v>
@@ -3233,21 +3225,20 @@
         <v>5</v>
       </c>
       <c r="C56" t="s">
+        <v>354</v>
+      </c>
+      <c r="D56" t="s">
         <v>355</v>
       </c>
-      <c r="D56" t="s">
-        <v>356</v>
-      </c>
       <c r="E56" s="7" t="s">
         <v>36</v>
       </c>
       <c r="F56" s="7" t="str">
-        <f t="shared" ref="F56:G56" si="51">E56</f>
-        <v>Strava</v>
-      </c>
-      <c r="G56" s="7" t="str">
-        <f t="shared" si="51"/>
-        <v>Strava</v>
+        <f t="shared" ref="F56" si="51">E56</f>
+        <v>Strava</v>
+      </c>
+      <c r="G56" s="7" t="s">
+        <v>36</v>
       </c>
       <c r="H56" s="4" t="s">
         <v>66</v>
@@ -3261,24 +3252,23 @@
         <v>5</v>
       </c>
       <c r="C57" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="D57" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="E57" s="7" t="s">
         <v>36</v>
       </c>
       <c r="F57" s="7" t="str">
-        <f t="shared" ref="F57:G57" si="52">E57</f>
-        <v>Strava</v>
-      </c>
-      <c r="G57" s="7" t="str">
-        <f t="shared" si="52"/>
-        <v>Strava</v>
+        <f t="shared" ref="F57" si="52">E57</f>
+        <v>Strava</v>
+      </c>
+      <c r="G57" s="7" t="s">
+        <v>36</v>
       </c>
       <c r="H57" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
     </row>
     <row r="58" spans="1:8">
@@ -3289,7 +3279,7 @@
         <v>6</v>
       </c>
       <c r="C58" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D58" t="s">
         <v>70</v>
@@ -3317,7 +3307,7 @@
         <v>6</v>
       </c>
       <c r="C59" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D59" t="s">
         <v>70</v>
@@ -3345,7 +3335,7 @@
         <v>6</v>
       </c>
       <c r="C60" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D60" t="s">
         <v>70</v>
@@ -3365,15 +3355,15 @@
         <v>70</v>
       </c>
     </row>
-    <row r="61" spans="1:8" ht="15">
+    <row r="61" spans="1:8">
       <c r="A61" s="6">
         <v>46361</v>
       </c>
       <c r="B61" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="C61" s="29" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="D61" t="s">
         <v>26</v>
@@ -3382,18 +3372,17 @@
         <v>36</v>
       </c>
       <c r="F61" s="7" t="str">
-        <f t="shared" ref="F61:G61" si="56">E61</f>
-        <v>Strava</v>
-      </c>
-      <c r="G61" s="7" t="str">
-        <f t="shared" si="56"/>
-        <v>Strava</v>
+        <f t="shared" ref="F61" si="56">E61</f>
+        <v>Strava</v>
+      </c>
+      <c r="G61" s="7" t="s">
+        <v>36</v>
       </c>
       <c r="H61" s="29" t="s">
-        <v>371</v>
-      </c>
-    </row>
-    <row r="62" spans="1:8" ht="15">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8">
       <c r="A62" s="6">
         <v>46368</v>
       </c>
@@ -3401,7 +3390,7 @@
         <v>5</v>
       </c>
       <c r="C62" s="29" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="D62" t="s">
         <v>29</v>
@@ -3410,15 +3399,14 @@
         <v>36</v>
       </c>
       <c r="F62" s="7" t="str">
-        <f t="shared" ref="F62:G62" si="57">E62</f>
-        <v>Strava</v>
-      </c>
-      <c r="G62" s="7" t="str">
-        <f t="shared" si="57"/>
-        <v>Strava</v>
+        <f t="shared" ref="F62" si="57">E62</f>
+        <v>Strava</v>
+      </c>
+      <c r="G62" s="7" t="s">
+        <v>36</v>
       </c>
       <c r="H62" s="29" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="63" spans="1:8">
@@ -3438,12 +3426,11 @@
         <v>36</v>
       </c>
       <c r="F63" s="7" t="str">
-        <f t="shared" ref="F63:G63" si="58">E63</f>
-        <v>Strava</v>
-      </c>
-      <c r="G63" s="7" t="str">
-        <f t="shared" si="58"/>
-        <v>Strava</v>
+        <f t="shared" ref="F63" si="58">E63</f>
+        <v>Strava</v>
+      </c>
+      <c r="G63" s="7" t="s">
+        <v>36</v>
       </c>
       <c r="H63" s="4" t="s">
         <v>55</v>
@@ -3466,12 +3453,11 @@
         <v>36</v>
       </c>
       <c r="F64" s="7" t="str">
-        <f t="shared" ref="F64:G64" si="59">E64</f>
-        <v>Strava</v>
-      </c>
-      <c r="G64" s="7" t="str">
-        <f t="shared" si="59"/>
-        <v>Strava</v>
+        <f t="shared" ref="F64" si="59">E64</f>
+        <v>Strava</v>
+      </c>
+      <c r="G64" s="7" t="s">
+        <v>36</v>
       </c>
       <c r="H64" s="2" t="s">
         <v>49</v>
@@ -3531,6 +3517,24 @@
     <hyperlink ref="E61" r:id="rId50" xr:uid="{583CF50F-498E-0841-9BC9-5A9E3F837061}"/>
     <hyperlink ref="E62" r:id="rId51" xr:uid="{030FBD56-AB0C-764C-BC0B-06F85764D9FD}"/>
     <hyperlink ref="E45" r:id="rId52" xr:uid="{5BD7D123-7286-5A47-A0D9-8170243675C4}"/>
+    <hyperlink ref="G40" r:id="rId53" xr:uid="{8B72540D-E184-594B-B7BB-931E8CE8066C}"/>
+    <hyperlink ref="G42" r:id="rId54" xr:uid="{FF907A16-C49B-6940-9A49-5174184D91E8}"/>
+    <hyperlink ref="G43" r:id="rId55" xr:uid="{80F54F31-0D14-BA40-9830-6A3A4B290D55}"/>
+    <hyperlink ref="G44" r:id="rId56" xr:uid="{8D267D2E-3A23-4B48-B88F-051285D7BA36}"/>
+    <hyperlink ref="G46" r:id="rId57" xr:uid="{361489AA-38BC-2442-A548-A3F7EDFC8002}"/>
+    <hyperlink ref="G47" r:id="rId58" xr:uid="{5F56807E-FBB9-7144-8BED-5D4FB192A8EE}"/>
+    <hyperlink ref="G48" r:id="rId59" xr:uid="{5363C3C8-9072-9A44-983D-1FD0E3428E68}"/>
+    <hyperlink ref="G49" r:id="rId60" xr:uid="{549A2681-C267-8E45-844F-EF310CCCFDB2}"/>
+    <hyperlink ref="G51" r:id="rId61" xr:uid="{63252D4C-E3AC-1148-8CA9-B56CCD344D36}"/>
+    <hyperlink ref="G52" r:id="rId62" xr:uid="{98440C2B-FB64-3B47-868F-4D555F1A88B1}"/>
+    <hyperlink ref="G53" r:id="rId63" xr:uid="{EBCB25C5-25F2-8847-BE10-5DC3A3FB264F}"/>
+    <hyperlink ref="G54" r:id="rId64" xr:uid="{9C5D2F10-3E58-BB41-B927-BFF3018F1450}"/>
+    <hyperlink ref="G56" r:id="rId65" xr:uid="{A7AA9CE7-D397-ED45-A134-D461653F928E}"/>
+    <hyperlink ref="G57" r:id="rId66" xr:uid="{54BD7C89-AE76-544E-ACFF-B6F9DDAB007A}"/>
+    <hyperlink ref="G61" r:id="rId67" xr:uid="{1A12B0E4-5936-BD49-B04D-141DE949D1CB}"/>
+    <hyperlink ref="G62" r:id="rId68" xr:uid="{676807D1-D959-964B-B19D-ABBB412ECB83}"/>
+    <hyperlink ref="G63" r:id="rId69" xr:uid="{55193CD3-AD02-9F4A-A96B-72D44533BB4F}"/>
+    <hyperlink ref="G64" r:id="rId70" xr:uid="{D1B99FE7-3D04-C048-9F49-E9DE3DCBD207}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3539,7 +3543,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B1CA8C7-05A5-DA44-B969-9E41B832BB96}">
   <dimension ref="A1:E98"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.6640625" bestFit="1" customWidth="1"/>
@@ -3981,7 +3985,7 @@
         <v>76</v>
       </c>
       <c r="C26" s="16" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="D26" s="18" t="s">
         <v>147</v>
@@ -4117,7 +4121,7 @@
         <v>76</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D34" s="16" t="s">
         <v>168</v>
@@ -4134,7 +4138,7 @@
         <v>76</v>
       </c>
       <c r="C35" s="16" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="D35" s="16" t="s">
         <v>170</v>
@@ -4151,7 +4155,7 @@
         <v>76</v>
       </c>
       <c r="C36" s="16" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="D36" s="16" t="s">
         <v>172</v>
@@ -4185,7 +4189,7 @@
         <v>76</v>
       </c>
       <c r="C38" s="16" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D38" s="16" t="s">
         <v>177</v>
@@ -4202,7 +4206,7 @@
         <v>76</v>
       </c>
       <c r="C39" s="16" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="D39" s="16" t="s">
         <v>179</v>
@@ -4287,7 +4291,7 @@
         <v>76</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D44" s="16" t="s">
         <v>192</v>
@@ -4321,7 +4325,7 @@
         <v>76</v>
       </c>
       <c r="C46" s="19" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="D46" s="16" t="s">
         <v>130</v>
@@ -4338,7 +4342,7 @@
         <v>76</v>
       </c>
       <c r="C47" s="16" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="D47" s="16" t="s">
         <v>198</v>
@@ -4372,7 +4376,7 @@
         <v>76</v>
       </c>
       <c r="C49" s="16" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D49" s="16" t="s">
         <v>156</v>
@@ -4406,7 +4410,7 @@
         <v>76</v>
       </c>
       <c r="C51" s="16" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D51" s="16" t="s">
         <v>206</v>
@@ -4423,7 +4427,7 @@
         <v>76</v>
       </c>
       <c r="C52" s="16" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D52" s="16" t="s">
         <v>208</v>
@@ -4457,7 +4461,7 @@
         <v>76</v>
       </c>
       <c r="C54" s="16" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D54" s="16" t="s">
         <v>212</v>
@@ -4474,7 +4478,7 @@
         <v>76</v>
       </c>
       <c r="C55" s="16" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D55" s="16" t="s">
         <v>214</v>
@@ -4508,13 +4512,13 @@
         <v>76</v>
       </c>
       <c r="C57" s="16" t="s">
+        <v>376</v>
+      </c>
+      <c r="D57" s="18" t="s">
         <v>219</v>
       </c>
-      <c r="D57" s="18" t="s">
+      <c r="E57" s="18" t="s">
         <v>220</v>
-      </c>
-      <c r="E57" s="18" t="s">
-        <v>221</v>
       </c>
     </row>
     <row r="58" spans="1:5">
@@ -4525,13 +4529,13 @@
         <v>76</v>
       </c>
       <c r="C58" s="16" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="D58" s="16" t="s">
+        <v>221</v>
+      </c>
+      <c r="E58" s="17" t="s">
         <v>222</v>
-      </c>
-      <c r="E58" s="17" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="59" spans="1:5">
@@ -4542,13 +4546,13 @@
         <v>76</v>
       </c>
       <c r="C59" s="16" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="D59" s="18" t="s">
+        <v>223</v>
+      </c>
+      <c r="E59" s="18" t="s">
         <v>224</v>
-      </c>
-      <c r="E59" s="18" t="s">
-        <v>225</v>
       </c>
     </row>
     <row r="60" spans="1:5">
@@ -4559,13 +4563,13 @@
         <v>76</v>
       </c>
       <c r="C60" s="16" t="s">
+        <v>225</v>
+      </c>
+      <c r="D60" s="16" t="s">
         <v>226</v>
       </c>
-      <c r="D60" s="16" t="s">
+      <c r="E60" s="17" t="s">
         <v>227</v>
-      </c>
-      <c r="E60" s="17" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="61" spans="1:5">
@@ -4576,13 +4580,13 @@
         <v>76</v>
       </c>
       <c r="C61" s="16" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D61" s="16" t="s">
+        <v>228</v>
+      </c>
+      <c r="E61" s="17" t="s">
         <v>229</v>
-      </c>
-      <c r="E61" s="17" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="62" spans="1:5">
@@ -4593,13 +4597,13 @@
         <v>76</v>
       </c>
       <c r="C62" s="16" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="D62" s="16" t="s">
         <v>172</v>
       </c>
       <c r="E62" s="17" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="63" spans="1:5">
@@ -4610,13 +4614,13 @@
         <v>76</v>
       </c>
       <c r="C63" s="16" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="D63" s="16" t="s">
+        <v>231</v>
+      </c>
+      <c r="E63" s="17" t="s">
         <v>232</v>
-      </c>
-      <c r="E63" s="17" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="64" spans="1:5">
@@ -4627,13 +4631,13 @@
         <v>76</v>
       </c>
       <c r="C64" s="16" t="s">
+        <v>233</v>
+      </c>
+      <c r="D64" s="16" t="s">
         <v>234</v>
       </c>
-      <c r="D64" s="16" t="s">
+      <c r="E64" s="17" t="s">
         <v>235</v>
-      </c>
-      <c r="E64" s="17" t="s">
-        <v>236</v>
       </c>
     </row>
     <row r="65" spans="1:5">
@@ -4644,13 +4648,13 @@
         <v>76</v>
       </c>
       <c r="C65" s="16" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="D65" s="16" t="s">
         <v>81</v>
       </c>
       <c r="E65" s="17" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="66" spans="1:5">
@@ -4661,13 +4665,13 @@
         <v>76</v>
       </c>
       <c r="C66" s="16" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="D66" s="16" t="s">
+        <v>237</v>
+      </c>
+      <c r="E66" s="17" t="s">
         <v>238</v>
-      </c>
-      <c r="E66" s="17" t="s">
-        <v>239</v>
       </c>
     </row>
     <row r="67" spans="1:5">
@@ -4678,13 +4682,13 @@
         <v>76</v>
       </c>
       <c r="C67" s="16" t="s">
+        <v>239</v>
+      </c>
+      <c r="D67" s="16" t="s">
         <v>240</v>
       </c>
-      <c r="D67" s="16" t="s">
+      <c r="E67" s="17" t="s">
         <v>241</v>
-      </c>
-      <c r="E67" s="17" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="68" spans="1:5">
@@ -4695,13 +4699,13 @@
         <v>76</v>
       </c>
       <c r="C68" s="16" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="D68" s="16" t="s">
+        <v>242</v>
+      </c>
+      <c r="E68" s="17" t="s">
         <v>243</v>
-      </c>
-      <c r="E68" s="17" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="69" spans="1:5">
@@ -4712,13 +4716,13 @@
         <v>76</v>
       </c>
       <c r="C69" s="16" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="D69" s="16" t="s">
+        <v>244</v>
+      </c>
+      <c r="E69" s="17" t="s">
         <v>245</v>
-      </c>
-      <c r="E69" s="17" t="s">
-        <v>246</v>
       </c>
     </row>
     <row r="70" spans="1:5">
@@ -4729,13 +4733,13 @@
         <v>76</v>
       </c>
       <c r="C70" s="16" t="s">
+        <v>246</v>
+      </c>
+      <c r="D70" s="18" t="s">
         <v>247</v>
       </c>
-      <c r="D70" s="18" t="s">
+      <c r="E70" s="18" t="s">
         <v>248</v>
-      </c>
-      <c r="E70" s="18" t="s">
-        <v>249</v>
       </c>
     </row>
     <row r="71" spans="1:5">
@@ -4746,13 +4750,13 @@
         <v>76</v>
       </c>
       <c r="C71" s="16" t="s">
+        <v>249</v>
+      </c>
+      <c r="D71" s="16" t="s">
         <v>250</v>
       </c>
-      <c r="D71" s="16" t="s">
+      <c r="E71" s="17" t="s">
         <v>251</v>
-      </c>
-      <c r="E71" s="17" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="72" spans="1:5">
@@ -4763,13 +4767,13 @@
         <v>76</v>
       </c>
       <c r="C72" s="16" t="s">
+        <v>252</v>
+      </c>
+      <c r="D72" s="18" t="s">
         <v>253</v>
       </c>
-      <c r="D72" s="18" t="s">
+      <c r="E72" s="18" t="s">
         <v>254</v>
-      </c>
-      <c r="E72" s="18" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="73" spans="1:5">
@@ -4780,13 +4784,13 @@
         <v>76</v>
       </c>
       <c r="C73" s="16" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="D73" s="16" t="s">
+        <v>255</v>
+      </c>
+      <c r="E73" s="17" t="s">
         <v>256</v>
-      </c>
-      <c r="E73" s="17" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="74" spans="1:5">
@@ -4797,13 +4801,13 @@
         <v>76</v>
       </c>
       <c r="C74" s="16" t="s">
+        <v>257</v>
+      </c>
+      <c r="D74" s="16" t="s">
         <v>258</v>
       </c>
-      <c r="D74" s="16" t="s">
+      <c r="E74" s="17" t="s">
         <v>259</v>
-      </c>
-      <c r="E74" s="17" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="75" spans="1:5">
@@ -4814,13 +4818,13 @@
         <v>76</v>
       </c>
       <c r="C75" s="16" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D75" s="18" t="s">
         <v>111</v>
       </c>
       <c r="E75" s="18" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="76" spans="1:5">
@@ -4831,13 +4835,13 @@
         <v>76</v>
       </c>
       <c r="C76" s="16" t="s">
+        <v>262</v>
+      </c>
+      <c r="D76" s="18" t="s">
         <v>263</v>
       </c>
-      <c r="D76" s="18" t="s">
+      <c r="E76" s="18" t="s">
         <v>264</v>
-      </c>
-      <c r="E76" s="18" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="77" spans="1:5">
@@ -4848,13 +4852,13 @@
         <v>76</v>
       </c>
       <c r="C77" s="16" t="s">
+        <v>265</v>
+      </c>
+      <c r="D77" s="18" t="s">
         <v>266</v>
       </c>
-      <c r="D77" s="18" t="s">
+      <c r="E77" s="18" t="s">
         <v>267</v>
-      </c>
-      <c r="E77" s="18" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="78" spans="1:5">
@@ -4865,13 +4869,13 @@
         <v>76</v>
       </c>
       <c r="C78" s="16" t="s">
+        <v>268</v>
+      </c>
+      <c r="D78" s="18" t="s">
         <v>269</v>
       </c>
-      <c r="D78" s="18" t="s">
+      <c r="E78" s="18" t="s">
         <v>270</v>
-      </c>
-      <c r="E78" s="18" t="s">
-        <v>271</v>
       </c>
     </row>
     <row r="79" spans="1:5">
@@ -4882,13 +4886,13 @@
         <v>76</v>
       </c>
       <c r="C79" s="16" t="s">
+        <v>271</v>
+      </c>
+      <c r="D79" s="16" t="s">
+        <v>250</v>
+      </c>
+      <c r="E79" s="17" t="s">
         <v>272</v>
-      </c>
-      <c r="D79" s="16" t="s">
-        <v>251</v>
-      </c>
-      <c r="E79" s="17" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="80" spans="1:5">
@@ -4899,13 +4903,13 @@
         <v>76</v>
       </c>
       <c r="C80" s="16" t="s">
+        <v>273</v>
+      </c>
+      <c r="D80" s="18" t="s">
         <v>274</v>
       </c>
-      <c r="D80" s="18" t="s">
+      <c r="E80" s="18" t="s">
         <v>275</v>
-      </c>
-      <c r="E80" s="18" t="s">
-        <v>276</v>
       </c>
     </row>
     <row r="81" spans="1:5">
@@ -4916,13 +4920,13 @@
         <v>76</v>
       </c>
       <c r="C81" s="16" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="D81" s="16" t="s">
+        <v>276</v>
+      </c>
+      <c r="E81" s="17" t="s">
         <v>277</v>
-      </c>
-      <c r="E81" s="17" t="s">
-        <v>278</v>
       </c>
     </row>
     <row r="82" spans="1:5">
@@ -4933,13 +4937,13 @@
         <v>76</v>
       </c>
       <c r="C82" s="16" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="D82" s="16" t="s">
+        <v>278</v>
+      </c>
+      <c r="E82" s="17" t="s">
         <v>279</v>
-      </c>
-      <c r="E82" s="17" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="83" spans="1:5">
@@ -4950,13 +4954,13 @@
         <v>76</v>
       </c>
       <c r="C83" s="16" t="s">
+        <v>280</v>
+      </c>
+      <c r="D83" s="16" t="s">
         <v>281</v>
       </c>
-      <c r="D83" s="16" t="s">
+      <c r="E83" s="17" t="s">
         <v>282</v>
-      </c>
-      <c r="E83" s="17" t="s">
-        <v>283</v>
       </c>
     </row>
     <row r="84" spans="1:5">
@@ -4967,13 +4971,13 @@
         <v>76</v>
       </c>
       <c r="C84" s="16" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="D84" s="16" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="E84" s="17" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="85" spans="1:5">
@@ -4984,13 +4988,13 @@
         <v>76</v>
       </c>
       <c r="C85" s="16" t="s">
+        <v>284</v>
+      </c>
+      <c r="D85" s="16" t="s">
         <v>285</v>
       </c>
-      <c r="D85" s="16" t="s">
+      <c r="E85" s="17" t="s">
         <v>286</v>
-      </c>
-      <c r="E85" s="17" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="86" spans="1:5">
@@ -5001,13 +5005,13 @@
         <v>76</v>
       </c>
       <c r="C86" s="16" t="s">
+        <v>287</v>
+      </c>
+      <c r="D86" s="16" t="s">
+        <v>276</v>
+      </c>
+      <c r="E86" s="17" t="s">
         <v>288</v>
-      </c>
-      <c r="D86" s="16" t="s">
-        <v>277</v>
-      </c>
-      <c r="E86" s="17" t="s">
-        <v>289</v>
       </c>
     </row>
     <row r="87" spans="1:5">
@@ -5018,13 +5022,13 @@
         <v>76</v>
       </c>
       <c r="C87" s="16" t="s">
+        <v>289</v>
+      </c>
+      <c r="D87" s="16" t="s">
         <v>290</v>
       </c>
-      <c r="D87" s="16" t="s">
+      <c r="E87" s="17" t="s">
         <v>291</v>
-      </c>
-      <c r="E87" s="17" t="s">
-        <v>292</v>
       </c>
     </row>
     <row r="88" spans="1:5">
@@ -5035,13 +5039,13 @@
         <v>76</v>
       </c>
       <c r="C88" s="16" t="s">
+        <v>292</v>
+      </c>
+      <c r="D88" s="16" t="s">
+        <v>278</v>
+      </c>
+      <c r="E88" s="17" t="s">
         <v>293</v>
-      </c>
-      <c r="D88" s="16" t="s">
-        <v>279</v>
-      </c>
-      <c r="E88" s="17" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="89" spans="1:5">
@@ -5052,13 +5056,13 @@
         <v>76</v>
       </c>
       <c r="C89" s="16" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D89" s="16" t="s">
         <v>96</v>
       </c>
       <c r="E89" s="17" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="90" spans="1:5">
@@ -5069,13 +5073,13 @@
         <v>76</v>
       </c>
       <c r="C90" s="16" t="s">
+        <v>296</v>
+      </c>
+      <c r="D90" s="16" t="s">
         <v>297</v>
       </c>
-      <c r="D90" s="16" t="s">
+      <c r="E90" s="17" t="s">
         <v>298</v>
-      </c>
-      <c r="E90" s="17" t="s">
-        <v>299</v>
       </c>
     </row>
     <row r="91" spans="1:5">
@@ -5086,13 +5090,13 @@
         <v>76</v>
       </c>
       <c r="C91" s="16" t="s">
+        <v>299</v>
+      </c>
+      <c r="D91" s="16" t="s">
         <v>300</v>
       </c>
-      <c r="D91" s="16" t="s">
+      <c r="E91" s="17" t="s">
         <v>301</v>
-      </c>
-      <c r="E91" s="17" t="s">
-        <v>302</v>
       </c>
     </row>
     <row r="92" spans="1:5">
@@ -5103,13 +5107,13 @@
         <v>76</v>
       </c>
       <c r="C92" s="16" t="s">
+        <v>302</v>
+      </c>
+      <c r="D92" s="16" t="s">
         <v>303</v>
       </c>
-      <c r="D92" s="16" t="s">
+      <c r="E92" s="17" t="s">
         <v>304</v>
-      </c>
-      <c r="E92" s="17" t="s">
-        <v>305</v>
       </c>
     </row>
     <row r="93" spans="1:5">
@@ -5120,13 +5124,13 @@
         <v>76</v>
       </c>
       <c r="C93" s="16" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="D93" s="16" t="s">
         <v>182</v>
       </c>
       <c r="E93" s="17" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="94" spans="1:5">
@@ -5137,13 +5141,13 @@
         <v>76</v>
       </c>
       <c r="C94" s="16" t="s">
+        <v>307</v>
+      </c>
+      <c r="D94" s="18" t="s">
         <v>308</v>
       </c>
-      <c r="D94" s="18" t="s">
+      <c r="E94" s="18" t="s">
         <v>309</v>
-      </c>
-      <c r="E94" s="18" t="s">
-        <v>310</v>
       </c>
     </row>
     <row r="95" spans="1:5">
@@ -5154,13 +5158,13 @@
         <v>76</v>
       </c>
       <c r="C95" s="25" t="s">
+        <v>320</v>
+      </c>
+      <c r="D95" s="23" t="s">
         <v>321</v>
       </c>
-      <c r="D95" s="23" t="s">
+      <c r="E95" s="23" t="s">
         <v>322</v>
-      </c>
-      <c r="E95" s="23" t="s">
-        <v>323</v>
       </c>
     </row>
     <row r="96" spans="1:5">
@@ -5172,13 +5176,13 @@
         <v>76</v>
       </c>
       <c r="C96" s="26" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="D96" s="27" t="s">
         <v>96</v>
       </c>
       <c r="E96" s="27" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="97" spans="1:5">
@@ -5190,13 +5194,13 @@
         <v>76</v>
       </c>
       <c r="C97" s="22" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="D97" s="23" t="s">
         <v>182</v>
       </c>
       <c r="E97" s="23" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="98" spans="1:5">
@@ -5208,16 +5212,17 @@
         <v>76</v>
       </c>
       <c r="C98" s="22" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="D98" s="23" t="s">
+        <v>317</v>
+      </c>
+      <c r="E98" s="23" t="s">
         <v>318</v>
       </c>
-      <c r="E98" s="23" t="s">
-        <v>319</v>
-      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:E98" xr:uid="{2B1CA8C7-05A5-DA44-B969-9E41B832BB96}"/>
   <hyperlinks>
     <hyperlink ref="C41" r:id="rId1" location="!" tooltip="Copiar RUT" display="https://app.clay.cl/moves/all/clp/67be238f0a446ac455f9fb131740514191735426 - !" xr:uid="{6663B4B4-EFE3-1D40-87F3-EEFD457C6AFA}"/>
   </hyperlinks>

</xml_diff>